<commit_message>
Calibration: Add geneticist age stages. Note: 1/4 to 3/4 represents full expression of the trait.
</commit_message>
<xml_diff>
--- a/ExcelInputs/Structural.xlsx
+++ b/ExcelInputs/Structural.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Models\AFO\ExcelInputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127C0B2D-B85A-4E4F-98F9-BA86FE1B5B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AA76A62-DC41-4944-96A6-32EDCF7AC316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="240" windowWidth="25950" windowHeight="15555" tabRatio="678" activeTab="1" xr2:uid="{0842FB8C-088A-42F9-B075-24D0619777A0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="678" activeTab="2" xr2:uid="{0842FB8C-088A-42F9-B075-24D0619777A0}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="24" r:id="rId1"/>
@@ -92,7 +92,7 @@
     <definedName name="i_lag_organs">Stock!$I$70</definedName>
     <definedName name="i_lag_wool">Stock!$I$69</definedName>
     <definedName name="i_landuse_is_dual" localSheetId="0">General!$Q$79:$Q$110</definedName>
-    <definedName name="i_len_f">StructuralSA!$I$200</definedName>
+    <definedName name="i_len_f">StructuralSA!$I$202</definedName>
     <definedName name="i_len_l">Stock!$M$159</definedName>
     <definedName name="i_len_m">Stock!$L$159</definedName>
     <definedName name="i_len_planning_horizon" localSheetId="2">StructuralSA!$M$46</definedName>
@@ -129,10 +129,11 @@
     <definedName name="i_prejoin_offset">Stock!$I$66</definedName>
     <definedName name="i_progeny_w2_len">StructuralSA!$Q$107</definedName>
     <definedName name="i_r2adjust_inc">StructuralSA!$U$148</definedName>
-    <definedName name="i_rev_age_stage" localSheetId="2">StructuralSA!$N$159:$Z$160</definedName>
+    <definedName name="i_rev_age_stage_afo" localSheetId="2">StructuralSA!$N$161:$Z$162</definedName>
+    <definedName name="i_rev_age_stage_asbv">StructuralSA!$N$160:$Z$160</definedName>
     <definedName name="i_rev_number" localSheetId="2">StructuralSA!$I$150</definedName>
-    <definedName name="i_rev_trait_name" localSheetId="2">StructuralSA!$H$162:$H$181</definedName>
-    <definedName name="i_rev_trait_scenario" localSheetId="2">StructuralSA!$I$162:$I$181</definedName>
+    <definedName name="i_rev_trait_name" localSheetId="2">StructuralSA!$H$164:$H$183</definedName>
+    <definedName name="i_rev_trait_scenario" localSheetId="2">StructuralSA!$I$164:$I$183</definedName>
     <definedName name="i_rev_update" localSheetId="2">StructuralSA!$I$148</definedName>
     <definedName name="i_sim_periods_year">Stock!$I$62</definedName>
     <definedName name="i_store_cs_rep" localSheetId="3">'Report Settings'!$K$18</definedName>
@@ -181,7 +182,7 @@
     <definedName name="ZA.WidthCol" localSheetId="4">Admin!$L$26</definedName>
     <definedName name="ZA.ZoomSheet" localSheetId="4">Admin!$O$26</definedName>
   </definedNames>
-  <calcPr calcId="191029" refMode="R1C1" iterate="1"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2213,7 +2214,79 @@
         </r>
       </text>
     </comment>
-    <comment ref="H161" authorId="1" shapeId="0" xr:uid="{FD0151C6-9F6F-4723-995E-804A9122F39A}">
+    <comment ref="N159" authorId="2" shapeId="0" xr:uid="{D52B6350-79DA-43ED-9DD3-35AB8C8E2C20}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>John:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+When using geneticist age stages adult and whole of life are allocated to the individual age stages. So age is not used.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y159" authorId="2" shapeId="0" xr:uid="{006B6E62-3675-41C9-9A10-C71798B4F55A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>John:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+When using geneticist age stages adult and whole of life are allocated to the individual age stages. So age is not used.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N160" authorId="2" shapeId="0" xr:uid="{E3693196-A31F-4656-BCF8-B8AE6FB68901}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>John:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Although not used this value needs to be 0 so that the np.roll works correctly</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H163" authorId="1" shapeId="0" xr:uid="{FD0151C6-9F6F-4723-995E-804A9122F39A}">
       <text>
         <r>
           <rPr>
@@ -2239,7 +2312,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I161" authorId="2" shapeId="0" xr:uid="{533029ED-41A1-487B-BDF7-AC2146E10D21}">
+    <comment ref="I163" authorId="2" shapeId="0" xr:uid="{533029ED-41A1-487B-BDF7-AC2146E10D21}">
       <text>
         <r>
           <rPr>
@@ -2264,7 +2337,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H165" authorId="2" shapeId="0" xr:uid="{A12E8373-CBF7-4301-8BBE-54FB2CD3F999}">
+    <comment ref="H167" authorId="2" shapeId="0" xr:uid="{A12E8373-CBF7-4301-8BBE-54FB2CD3F999}">
       <text>
         <r>
           <rPr>
@@ -2288,7 +2361,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H166" authorId="2" shapeId="0" xr:uid="{ADD99B78-258B-4112-BEFE-ACD7C132C257}">
+    <comment ref="H168" authorId="2" shapeId="0" xr:uid="{ADD99B78-258B-4112-BEFE-ACD7C132C257}">
       <text>
         <r>
           <rPr>
@@ -2312,7 +2385,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H167" authorId="2" shapeId="0" xr:uid="{F4A4ECC6-7846-4162-9607-F6E572F33EDF}">
+    <comment ref="H169" authorId="2" shapeId="0" xr:uid="{F4A4ECC6-7846-4162-9607-F6E572F33EDF}">
       <text>
         <r>
           <rPr>
@@ -2336,7 +2409,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H168" authorId="2" shapeId="0" xr:uid="{4C2B1933-42FC-4263-B576-C6A05675CBF9}">
+    <comment ref="H170" authorId="2" shapeId="0" xr:uid="{4C2B1933-42FC-4263-B576-C6A05675CBF9}">
       <text>
         <r>
           <rPr>
@@ -2360,7 +2433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H174" authorId="1" shapeId="0" xr:uid="{658A1575-7B6D-49A0-9205-9DD14E053E41}">
+    <comment ref="H176" authorId="1" shapeId="0" xr:uid="{658A1575-7B6D-49A0-9205-9DD14E053E41}">
       <text>
         <r>
           <rPr>
@@ -2384,7 +2457,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H179" authorId="2" shapeId="0" xr:uid="{7D72CFA0-EF47-40D9-9D6F-9FDC3F1C19F9}">
+    <comment ref="H181" authorId="2" shapeId="0" xr:uid="{7D72CFA0-EF47-40D9-9D6F-9FDC3F1C19F9}">
       <text>
         <r>
           <rPr>
@@ -2408,7 +2481,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H200" authorId="2" shapeId="0" xr:uid="{B39EFDC6-7ABB-4808-93B1-2819F2755236}">
+    <comment ref="H202" authorId="2" shapeId="0" xr:uid="{B39EFDC6-7ABB-4808-93B1-2819F2755236}">
       <text>
         <r>
           <rPr>
@@ -2471,7 +2544,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="450">
   <si>
     <t>Controls for this worksheet</t>
   </si>
@@ -3813,9 +3886,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Available trait timing (for information only)</t>
-  </si>
-  <si>
     <t>Geneticist definition (age)</t>
   </si>
   <si>
@@ -3887,7 +3957,52 @@
     <t>rr</t>
   </si>
   <si>
-    <t>31Jan26: Removed the Cutoff levels for the NV pools that have been moved to Property.xlsx
+    <t>Some arrays used for reporting are very big so the default is not to store them. This is the default settings which can be overwritten using sensitivity values</t>
+  </si>
+  <si>
+    <t>22Feb26: Change the value of Prejoining intial repro proportion to 100% in the 11 slice (was 100% in NM)
+20Jul22: Change i_chill_adj_b1 so that chill of the singles is increased (had been no change)
+19Jan22: Fix error in i_mask_g1g3 that included True for [BMT,BM]
+2Dec21 remove min numbers b1. it wasnt doing anything in the code.
+8Jun21: Change definition of the 'k2 input cluster' to include NM so these animals can be differentially fed.
+                 Add comments about difference between 'k2 input cluster' and 'k2 post processing cluster'
+                 Added comment about including the axis length inputs in the first table
+16May21: Remove heading user defined date
+14Apr21: MRY changes for EV pools and confinement (removed about confinement patterns being included)
+12Apr21: Change back to 3N for analysis
+                  1N for LW profile comparisons
+10Apr21: Altered k2 cluster for scan 0 to allocate all ewes to the 11 slice
+                   Changed inputs for GBAL because it can't be represented in the matrix
+4Apr21: Change to 3FVP with 3N
+2Apr21: Change to 3N for dams &amp; 5FVP
+31Mar21: Change the index for the k2 cluster (for the seasonality model)
+29Mar21: Changed to FVP3, 1N for dams, 3N for Offs
+22Mar21: Alter the initial weight &amp; wool spread for the weaners
+1: 1Apr19-Blank worksheet</t>
+  </si>
+  <si>
+    <t>22Feb26: Delete 'Prejoining initial repro propn' from Associatons table
+                   Change the order of the axes postion inputs so that they are in axis order rather than alphabetical order
+3May23: Convert chill adjustment scalars for GBAL slices to a formula (still needs work on the 11, 22 &amp; 33 slices)
+17Jun22: Add a chill adjustment scalar with a b1 axis (to scale Property.xlsx!i_chill_adj)
+11Jul21: dvp/fvp updates 
+27Apr21: Split fvp inputs
+25Apr21: Deleted range names i_w1_len &amp; w3
+9Apr21: Fix formatting (box) around k2 cluster definition.
+30Mar21: Added inputs for % dry and number dams mated
+2: 17Jul20-Added structural inputs table
+1: 1Apr19-Created the version control table</t>
+  </si>
+  <si>
+    <t>Available trait timing (REV trait / Model inversion) - for information only</t>
+  </si>
+  <si>
+    <t>Still to connect the FYI on model inversion traits</t>
+  </si>
+  <si>
+    <t>3May26: Change geneticist age stage named range to only include end and renamed to i_rev_age_stage_asbv
+17Apr29: Added details for geneticist age stage to calculate the midpoint. Converted adults to a 364 day year step
+31Jan26: Removed the Cutoff levels for the NV pools that have been moved to Property.xlsx
 9Dec25: Added sl &amp; rr as REV traits. Expanded era and rr to be available at all individual adult age stages not just overall.
 26Sep24: Add cfat (carcase fat depth) trait
 6Sep24: Alter order of age stages so that whole of life is [0] - which is the default in the code.
@@ -3919,43 +4034,6 @@
                    Moved FVP &amp; N inputs from Stock
 1: 1Apr19-Created the version control table</t>
   </si>
-  <si>
-    <t>Some arrays used for reporting are very big so the default is not to store them. This is the default settings which can be overwritten using sensitivity values</t>
-  </si>
-  <si>
-    <t>22Feb26: Change the value of Prejoining intial repro proportion to 100% in the 11 slice (was 100% in NM)
-20Jul22: Change i_chill_adj_b1 so that chill of the singles is increased (had been no change)
-19Jan22: Fix error in i_mask_g1g3 that included True for [BMT,BM]
-2Dec21 remove min numbers b1. it wasnt doing anything in the code.
-8Jun21: Change definition of the 'k2 input cluster' to include NM so these animals can be differentially fed.
-                 Add comments about difference between 'k2 input cluster' and 'k2 post processing cluster'
-                 Added comment about including the axis length inputs in the first table
-16May21: Remove heading user defined date
-14Apr21: MRY changes for EV pools and confinement (removed about confinement patterns being included)
-12Apr21: Change back to 3N for analysis
-                  1N for LW profile comparisons
-10Apr21: Altered k2 cluster for scan 0 to allocate all ewes to the 11 slice
-                   Changed inputs for GBAL because it can't be represented in the matrix
-4Apr21: Change to 3FVP with 3N
-2Apr21: Change to 3N for dams &amp; 5FVP
-31Mar21: Change the index for the k2 cluster (for the seasonality model)
-29Mar21: Changed to FVP3, 1N for dams, 3N for Offs
-22Mar21: Alter the initial weight &amp; wool spread for the weaners
-1: 1Apr19-Blank worksheet</t>
-  </si>
-  <si>
-    <t>22Feb26: Delete 'Prejoining initial repro propn' from Associatons table
-                   Change the order of the axes postion inputs so that they are in axis order rather than alphabetical order
-3May23: Convert chill adjustment scalars for GBAL slices to a formula (still needs work on the 11, 22 &amp; 33 slices)
-17Jun22: Add a chill adjustment scalar with a b1 axis (to scale Property.xlsx!i_chill_adj)
-11Jul21: dvp/fvp updates 
-27Apr21: Split fvp inputs
-25Apr21: Deleted range names i_w1_len &amp; w3
-9Apr21: Fix formatting (box) around k2 cluster definition.
-30Mar21: Added inputs for % dry and number dams mated
-2: 17Jul20-Added structural inputs table
-1: 1Apr19-Created the version control table</t>
-  </si>
 </sst>
 </file>
 
@@ -3967,7 +4045,7 @@
     <numFmt numFmtId="166" formatCode="0.00_)"/>
     <numFmt numFmtId="167" formatCode="[$-C09]dd\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4186,6 +4264,25 @@
       <color rgb="FF0000CC"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="40">
@@ -5370,7 +5467,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="228">
+  <cellXfs count="231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="25" xfId="3">
@@ -5959,6 +6056,15 @@
     <xf numFmtId="1" fontId="32" fillId="39" borderId="22" xfId="44" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="50" xfId="13" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="24" xfId="16" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="38" xfId="12" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -7125,19 +7231,19 @@
       <c r="I13" s="126">
         <v>44371.659649305599</v>
       </c>
-      <c r="J13" s="221" t="s">
+      <c r="J13" s="224" t="s">
         <v>293</v>
       </c>
-      <c r="K13" s="222"/>
-      <c r="L13" s="222"/>
-      <c r="M13" s="222"/>
-      <c r="N13" s="222"/>
-      <c r="O13" s="222"/>
-      <c r="P13" s="222"/>
-      <c r="Q13" s="222"/>
-      <c r="R13" s="222"/>
-      <c r="S13" s="222"/>
-      <c r="T13" s="223"/>
+      <c r="K13" s="225"/>
+      <c r="L13" s="225"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="225"/>
+      <c r="O13" s="225"/>
+      <c r="P13" s="225"/>
+      <c r="Q13" s="225"/>
+      <c r="R13" s="225"/>
+      <c r="S13" s="225"/>
+      <c r="T13" s="226"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
@@ -7164,19 +7270,19 @@
       <c r="I14" s="125">
         <v>44719.411846643503</v>
       </c>
-      <c r="J14" s="224" t="s">
+      <c r="J14" s="227" t="s">
         <v>352</v>
       </c>
-      <c r="K14" s="225"/>
-      <c r="L14" s="225"/>
-      <c r="M14" s="225"/>
-      <c r="N14" s="225"/>
-      <c r="O14" s="225"/>
-      <c r="P14" s="225"/>
-      <c r="Q14" s="225"/>
-      <c r="R14" s="225"/>
-      <c r="S14" s="225"/>
-      <c r="T14" s="225"/>
+      <c r="K14" s="228"/>
+      <c r="L14" s="228"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="228"/>
+      <c r="O14" s="228"/>
+      <c r="P14" s="228"/>
+      <c r="Q14" s="228"/>
+      <c r="R14" s="228"/>
+      <c r="S14" s="228"/>
+      <c r="T14" s="228"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -9793,7 +9899,7 @@
       <c r="G86" s="4"/>
       <c r="H86" s="148"/>
       <c r="I86" s="162" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="J86" s="162" t="b">
         <v>0</v>
@@ -9978,13 +10084,13 @@
       <c r="N90" s="164"/>
       <c r="O90" s="164"/>
       <c r="P90" s="162" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q90" s="162" t="b">
         <v>0</v>
       </c>
       <c r="R90" s="206" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
@@ -11813,19 +11919,19 @@
       <c r="I13" s="126">
         <v>46075.691937152798</v>
       </c>
-      <c r="J13" s="221" t="s">
-        <v>448</v>
-      </c>
-      <c r="K13" s="222"/>
-      <c r="L13" s="222"/>
-      <c r="M13" s="222"/>
-      <c r="N13" s="222"/>
-      <c r="O13" s="222"/>
-      <c r="P13" s="222"/>
-      <c r="Q13" s="222"/>
-      <c r="R13" s="222"/>
-      <c r="S13" s="222"/>
-      <c r="T13" s="223"/>
+      <c r="J13" s="224" t="s">
+        <v>446</v>
+      </c>
+      <c r="K13" s="225"/>
+      <c r="L13" s="225"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="225"/>
+      <c r="O13" s="225"/>
+      <c r="P13" s="225"/>
+      <c r="Q13" s="225"/>
+      <c r="R13" s="225"/>
+      <c r="S13" s="225"/>
+      <c r="T13" s="226"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
@@ -11852,19 +11958,19 @@
       <c r="I14" s="125">
         <v>46075.710698379597</v>
       </c>
-      <c r="J14" s="224" t="s">
-        <v>447</v>
-      </c>
-      <c r="K14" s="225"/>
-      <c r="L14" s="225"/>
-      <c r="M14" s="225"/>
-      <c r="N14" s="225"/>
-      <c r="O14" s="225"/>
-      <c r="P14" s="225"/>
-      <c r="Q14" s="225"/>
-      <c r="R14" s="225"/>
-      <c r="S14" s="225"/>
-      <c r="T14" s="225"/>
+      <c r="J14" s="227" t="s">
+        <v>445</v>
+      </c>
+      <c r="K14" s="228"/>
+      <c r="L14" s="228"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="228"/>
+      <c r="O14" s="228"/>
+      <c r="P14" s="228"/>
+      <c r="Q14" s="228"/>
+      <c r="R14" s="228"/>
+      <c r="S14" s="228"/>
+      <c r="T14" s="228"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -27026,7 +27132,7 @@
   <sheetPr codeName="Sheet3">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AE214"/>
+  <dimension ref="A1:AE216"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -27555,21 +27661,21 @@
         <v>16</v>
       </c>
       <c r="I13" s="126">
-        <v>46053.6384755787</v>
-      </c>
-      <c r="J13" s="221" t="s">
-        <v>445</v>
-      </c>
-      <c r="K13" s="222"/>
-      <c r="L13" s="222"/>
-      <c r="M13" s="222"/>
-      <c r="N13" s="222"/>
-      <c r="O13" s="222"/>
-      <c r="P13" s="222"/>
-      <c r="Q13" s="222"/>
-      <c r="R13" s="222"/>
-      <c r="S13" s="222"/>
-      <c r="T13" s="223"/>
+        <v>46145.506140277801</v>
+      </c>
+      <c r="J13" s="224" t="s">
+        <v>449</v>
+      </c>
+      <c r="K13" s="225"/>
+      <c r="L13" s="225"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="225"/>
+      <c r="O13" s="225"/>
+      <c r="P13" s="225"/>
+      <c r="Q13" s="225"/>
+      <c r="R13" s="225"/>
+      <c r="S13" s="225"/>
+      <c r="T13" s="226"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
@@ -27599,19 +27705,19 @@
       <c r="I14" s="125">
         <v>45593.407781134301</v>
       </c>
-      <c r="J14" s="224" t="s">
-        <v>441</v>
-      </c>
-      <c r="K14" s="225"/>
-      <c r="L14" s="225"/>
-      <c r="M14" s="225"/>
-      <c r="N14" s="225"/>
-      <c r="O14" s="225"/>
-      <c r="P14" s="225"/>
-      <c r="Q14" s="225"/>
-      <c r="R14" s="225"/>
-      <c r="S14" s="225"/>
-      <c r="T14" s="225"/>
+      <c r="J14" s="227" t="s">
+        <v>440</v>
+      </c>
+      <c r="K14" s="228"/>
+      <c r="L14" s="228"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="228"/>
+      <c r="O14" s="228"/>
+      <c r="P14" s="228"/>
+      <c r="Q14" s="228"/>
+      <c r="R14" s="228"/>
+      <c r="S14" s="228"/>
+      <c r="T14" s="228"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -28846,7 +28952,7 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="26" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="M46" s="220">
         <v>100</v>
@@ -28888,7 +28994,7 @@
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
       <c r="L47" s="26" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="M47" s="212" t="b">
         <v>0</v>
@@ -32852,7 +32958,7 @@
       <c r="A139" s="1"/>
       <c r="B139" s="33"/>
       <c r="C139" s="73">
-        <f>INT(MAX($C$147:$C$182))+1</f>
+        <f>INT(MAX($C$147:$C$184))+1</f>
         <v>5</v>
       </c>
       <c r="D139" s="3"/>
@@ -33536,7 +33642,7 @@
         <v>398</v>
       </c>
       <c r="N156" s="36" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O156" s="56" t="s">
         <v>401</v>
@@ -33599,37 +33705,37 @@
         <v>0</v>
       </c>
       <c r="O157" s="56" t="s">
+        <v>426</v>
+      </c>
+      <c r="P157" s="56" t="s">
         <v>427</v>
       </c>
-      <c r="P157" s="56" t="s">
+      <c r="Q157" s="56" t="s">
         <v>428</v>
       </c>
-      <c r="Q157" s="56" t="s">
+      <c r="R157" s="56" t="s">
         <v>429</v>
       </c>
-      <c r="R157" s="56" t="s">
+      <c r="S157" s="56" t="s">
         <v>430</v>
       </c>
-      <c r="S157" s="56" t="s">
+      <c r="T157" s="36" t="s">
         <v>431</v>
       </c>
-      <c r="T157" s="36" t="s">
+      <c r="U157" s="36" t="s">
         <v>432</v>
       </c>
-      <c r="U157" s="36" t="s">
+      <c r="V157" s="36" t="s">
         <v>433</v>
       </c>
-      <c r="V157" s="36" t="s">
+      <c r="W157" s="36" t="s">
         <v>434</v>
       </c>
-      <c r="W157" s="36" t="s">
+      <c r="X157" s="36" t="s">
         <v>435</v>
       </c>
-      <c r="X157" s="36" t="s">
+      <c r="Y157" s="36" t="s">
         <v>436</v>
-      </c>
-      <c r="Y157" s="36" t="s">
-        <v>437</v>
       </c>
       <c r="Z157" s="36">
         <v>12</v>
@@ -33644,7 +33750,7 @@
       <c r="A158" s="1"/>
       <c r="B158" s="33"/>
       <c r="C158" s="73">
-        <f t="shared" ref="C158:C160" si="11">INT(C$140+3)</f>
+        <f t="shared" ref="C158:C162" si="11">INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D158" s="4"/>
@@ -33656,7 +33762,7 @@
       <c r="J158" s="148"/>
       <c r="K158" s="148"/>
       <c r="L158" s="26" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="M158" s="52"/>
       <c r="N158" s="36"/>
@@ -33715,59 +33821,47 @@
       <c r="I159" s="148"/>
       <c r="J159" s="148"/>
       <c r="K159" s="148"/>
-      <c r="L159" s="151" t="s">
-        <v>425</v>
-      </c>
-      <c r="M159" s="151" t="s">
+      <c r="L159" s="148"/>
+      <c r="M159" s="52" t="s">
         <v>399</v>
       </c>
-      <c r="N159" s="31">
-        <v>0</v>
-      </c>
+      <c r="N159" s="36"/>
       <c r="O159" s="31">
         <v>0</v>
       </c>
       <c r="P159" s="31">
-        <f>O160+1</f>
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="Q159" s="31">
-        <f t="shared" ref="Q159" si="12">P160+1</f>
-        <v>101</v>
+        <v>150</v>
       </c>
       <c r="R159" s="31">
-        <f>P160+1</f>
-        <v>101</v>
+        <v>300</v>
       </c>
       <c r="S159" s="31">
-        <f>Q160+1</f>
-        <v>184</v>
+        <v>450</v>
       </c>
       <c r="T159" s="31">
-        <f>Y159</f>
-        <v>549</v>
-      </c>
-      <c r="U159" s="31">
-        <f t="shared" ref="U159" si="13">T160+1</f>
-        <v>914</v>
-      </c>
-      <c r="V159" s="31">
-        <f t="shared" ref="V159" si="14">U160+1</f>
-        <v>1279</v>
-      </c>
-      <c r="W159" s="31">
-        <f t="shared" ref="W159" si="15">V160+1</f>
-        <v>1644</v>
-      </c>
-      <c r="X159" s="31">
-        <f t="shared" ref="X159" si="16">W160+1</f>
-        <v>2009</v>
-      </c>
-      <c r="Y159" s="31">
-        <f>S160+1</f>
-        <v>549</v>
-      </c>
-      <c r="Z159" s="31"/>
+        <v>660</v>
+      </c>
+      <c r="U159" s="221">
+        <f>T159+364</f>
+        <v>1024</v>
+      </c>
+      <c r="V159" s="221">
+        <f t="shared" ref="V159:X159" si="12">U159+364</f>
+        <v>1388</v>
+      </c>
+      <c r="W159" s="221">
+        <f t="shared" si="12"/>
+        <v>1752</v>
+      </c>
+      <c r="X159" s="221">
+        <f t="shared" si="12"/>
+        <v>2116</v>
+      </c>
+      <c r="Y159" s="36"/>
+      <c r="Z159" s="36"/>
       <c r="AA159" s="4"/>
       <c r="AB159" s="16"/>
       <c r="AC159" s="1"/>
@@ -33790,210 +33884,246 @@
       <c r="J160" s="148"/>
       <c r="K160" s="148"/>
       <c r="L160" s="148"/>
-      <c r="M160" s="151" t="s">
+      <c r="M160" s="52" t="s">
         <v>400</v>
       </c>
-      <c r="N160" s="31">
-        <v>99999</v>
+      <c r="N160" s="36">
+        <v>0</v>
       </c>
       <c r="O160" s="31">
         <v>1</v>
       </c>
       <c r="P160" s="31">
-        <v>100</v>
+        <v>149</v>
       </c>
       <c r="Q160" s="31">
-        <v>183</v>
+        <v>299</v>
       </c>
       <c r="R160" s="31">
-        <v>425</v>
+        <v>449</v>
       </c>
       <c r="S160" s="31">
-        <f>S159+364</f>
-        <v>548</v>
+        <v>659</v>
       </c>
       <c r="T160" s="31">
-        <f>T159+364</f>
-        <v>913</v>
-      </c>
-      <c r="U160" s="31">
-        <f t="shared" ref="U160:X160" si="17">U159+364</f>
-        <v>1278</v>
-      </c>
-      <c r="V160" s="31">
-        <f t="shared" si="17"/>
-        <v>1643</v>
-      </c>
-      <c r="W160" s="31">
-        <f t="shared" si="17"/>
-        <v>2008</v>
-      </c>
-      <c r="X160" s="31">
-        <f t="shared" si="17"/>
-        <v>2373</v>
-      </c>
-      <c r="Y160" s="31">
-        <f>X160</f>
-        <v>2373</v>
-      </c>
-      <c r="Z160" s="31"/>
+        <v>1024</v>
+      </c>
+      <c r="U160" s="221">
+        <f t="shared" ref="U160:X160" si="13">T160+364</f>
+        <v>1388</v>
+      </c>
+      <c r="V160" s="221">
+        <f t="shared" si="13"/>
+        <v>1752</v>
+      </c>
+      <c r="W160" s="221">
+        <f t="shared" si="13"/>
+        <v>2116</v>
+      </c>
+      <c r="X160" s="221">
+        <f t="shared" si="13"/>
+        <v>2480</v>
+      </c>
+      <c r="Y160" s="36">
+        <v>0</v>
+      </c>
+      <c r="Z160" s="36">
+        <v>0</v>
+      </c>
       <c r="AA160" s="4"/>
       <c r="AB160" s="16"/>
       <c r="AC160" s="1"/>
       <c r="AD160" s="1"/>
       <c r="AE160" s="1"/>
     </row>
-    <row r="161" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
       <c r="B161" s="33"/>
       <c r="C161" s="73">
-        <f>INT($C$140)+2</f>
-        <v>3</v>
+        <f t="shared" si="11"/>
+        <v>4</v>
       </c>
       <c r="D161" s="4"/>
       <c r="E161" s="5"/>
       <c r="F161" s="5"/>
       <c r="G161" s="4"/>
-      <c r="H161" s="64" t="s">
-        <v>257</v>
-      </c>
-      <c r="I161" s="64" t="s">
-        <v>370</v>
-      </c>
-      <c r="J161" s="2"/>
-      <c r="K161" s="2"/>
-      <c r="L161" s="148"/>
-      <c r="M161" s="148"/>
-      <c r="N161" s="214"/>
-      <c r="O161" s="214"/>
-      <c r="P161" s="214"/>
-      <c r="Q161" s="160"/>
-      <c r="R161" s="160"/>
-      <c r="S161" s="160"/>
-      <c r="T161" s="160"/>
-      <c r="U161" s="160"/>
-      <c r="V161" s="160"/>
-      <c r="W161" s="160"/>
-      <c r="X161" s="160"/>
-      <c r="Y161" s="160"/>
-      <c r="Z161" s="160"/>
+      <c r="H161" s="148"/>
+      <c r="I161" s="148"/>
+      <c r="J161" s="148"/>
+      <c r="K161" s="148"/>
+      <c r="L161" s="151" t="s">
+        <v>424</v>
+      </c>
+      <c r="M161" s="151" t="s">
+        <v>399</v>
+      </c>
+      <c r="N161" s="31">
+        <v>0</v>
+      </c>
+      <c r="O161" s="31">
+        <v>0</v>
+      </c>
+      <c r="P161" s="31">
+        <f>O162+1</f>
+        <v>2</v>
+      </c>
+      <c r="Q161" s="31">
+        <f t="shared" ref="Q161" si="14">P162+1</f>
+        <v>101</v>
+      </c>
+      <c r="R161" s="31">
+        <f>P162+1</f>
+        <v>101</v>
+      </c>
+      <c r="S161" s="31">
+        <f>Q162+1</f>
+        <v>184</v>
+      </c>
+      <c r="T161" s="31">
+        <f t="shared" ref="T161" si="15">S162+1</f>
+        <v>549</v>
+      </c>
+      <c r="U161" s="221">
+        <f>T161+364</f>
+        <v>913</v>
+      </c>
+      <c r="V161" s="221">
+        <f t="shared" ref="V161:X161" si="16">U161+364</f>
+        <v>1277</v>
+      </c>
+      <c r="W161" s="221">
+        <f t="shared" si="16"/>
+        <v>1641</v>
+      </c>
+      <c r="X161" s="221">
+        <f t="shared" si="16"/>
+        <v>2005</v>
+      </c>
+      <c r="Y161" s="222">
+        <f>T161</f>
+        <v>549</v>
+      </c>
+      <c r="Z161" s="31">
+        <v>0</v>
+      </c>
       <c r="AA161" s="4"/>
       <c r="AB161" s="16"/>
       <c r="AC161" s="1"/>
       <c r="AD161" s="1"/>
       <c r="AE161" s="1"/>
     </row>
-    <row r="162" spans="1:31" outlineLevel="3" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
       <c r="B162" s="33"/>
       <c r="C162" s="73">
-        <f>INT($C$140)+3</f>
+        <f t="shared" si="11"/>
         <v>4</v>
       </c>
       <c r="D162" s="4"/>
-      <c r="E162" s="5">
-        <v>0</v>
-      </c>
+      <c r="E162" s="5"/>
       <c r="F162" s="5"/>
       <c r="G162" s="4"/>
-      <c r="H162" s="31" t="s">
-        <v>266</v>
-      </c>
-      <c r="I162" s="31">
-        <v>0</v>
-      </c>
+      <c r="H162" s="148"/>
+      <c r="I162" s="148"/>
       <c r="J162" s="148"/>
       <c r="K162" s="148"/>
       <c r="L162" s="148"/>
-      <c r="M162" s="148"/>
-      <c r="N162" s="218" t="s">
-        <v>423</v>
-      </c>
-      <c r="O162" s="218"/>
-      <c r="P162" s="218"/>
-      <c r="Q162" s="218"/>
-      <c r="R162" s="218"/>
-      <c r="S162" s="219"/>
-      <c r="T162" s="219"/>
-      <c r="U162" s="219"/>
-      <c r="V162" s="219"/>
-      <c r="W162" s="219"/>
-      <c r="X162" s="219"/>
-      <c r="Y162" s="219"/>
-      <c r="Z162" s="219"/>
+      <c r="M162" s="151" t="s">
+        <v>400</v>
+      </c>
+      <c r="N162" s="31">
+        <v>99999</v>
+      </c>
+      <c r="O162" s="31">
+        <v>1</v>
+      </c>
+      <c r="P162" s="31">
+        <v>100</v>
+      </c>
+      <c r="Q162" s="31">
+        <v>183</v>
+      </c>
+      <c r="R162" s="31">
+        <v>425</v>
+      </c>
+      <c r="S162" s="31">
+        <f>S161+364</f>
+        <v>548</v>
+      </c>
+      <c r="T162" s="31">
+        <f>T161+364</f>
+        <v>913</v>
+      </c>
+      <c r="U162" s="221">
+        <f t="shared" ref="U162:X162" si="17">T162+364</f>
+        <v>1277</v>
+      </c>
+      <c r="V162" s="221">
+        <f t="shared" si="17"/>
+        <v>1641</v>
+      </c>
+      <c r="W162" s="221">
+        <f t="shared" si="17"/>
+        <v>2005</v>
+      </c>
+      <c r="X162" s="221">
+        <f t="shared" si="17"/>
+        <v>2369</v>
+      </c>
+      <c r="Y162" s="222">
+        <f>X162</f>
+        <v>2369</v>
+      </c>
+      <c r="Z162" s="31">
+        <v>0</v>
+      </c>
       <c r="AA162" s="4"/>
       <c r="AB162" s="16"/>
       <c r="AC162" s="1"/>
       <c r="AD162" s="1"/>
       <c r="AE162" s="1"/>
     </row>
-    <row r="163" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="33"/>
       <c r="C163" s="73">
-        <f t="shared" ref="C163:C179" si="18">INT(C$140+3)</f>
-        <v>4</v>
+        <f>INT($C$140)+2</f>
+        <v>3</v>
       </c>
       <c r="D163" s="4"/>
-      <c r="E163" s="5">
-        <v>1</v>
-      </c>
+      <c r="E163" s="5"/>
       <c r="F163" s="5"/>
       <c r="G163" s="4"/>
-      <c r="H163" s="31" t="s">
-        <v>265</v>
-      </c>
-      <c r="I163" s="31">
-        <v>0</v>
-      </c>
-      <c r="J163" s="148"/>
-      <c r="K163" s="148"/>
+      <c r="H163" s="64" t="s">
+        <v>257</v>
+      </c>
+      <c r="I163" s="64" t="s">
+        <v>370</v>
+      </c>
+      <c r="J163" s="2"/>
+      <c r="K163" s="2"/>
       <c r="L163" s="148"/>
       <c r="M163" s="148"/>
-      <c r="N163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="O163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="P163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="Q163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="R163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="S163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="T163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="U163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="V163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="W163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="X163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="Y163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="Z163" s="217"/>
+      <c r="N163" s="214"/>
+      <c r="O163" s="214"/>
+      <c r="P163" s="214"/>
+      <c r="Q163" s="160"/>
+      <c r="R163" s="160"/>
+      <c r="S163" s="160"/>
+      <c r="T163" s="160"/>
+      <c r="U163" s="160"/>
+      <c r="V163" s="160"/>
+      <c r="W163" s="160"/>
+      <c r="X163" s="160"/>
+      <c r="Y163" s="160"/>
+      <c r="Z163" s="160"/>
       <c r="AA163" s="4"/>
       <c r="AB163" s="16"/>
       <c r="AC163" s="1"/>
       <c r="AD163" s="1"/>
       <c r="AE163" s="1"/>
     </row>
-    <row r="164" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:31" outlineLevel="3" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="33"/>
       <c r="C164" s="73">
@@ -34002,12 +34132,12 @@
       </c>
       <c r="D164" s="4"/>
       <c r="E164" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F164" s="5"/>
       <c r="G164" s="4"/>
       <c r="H164" s="31" t="s">
-        <v>372</v>
+        <v>266</v>
       </c>
       <c r="I164" s="31">
         <v>0</v>
@@ -34015,20 +34145,24 @@
       <c r="J164" s="148"/>
       <c r="K164" s="148"/>
       <c r="L164" s="148"/>
-      <c r="M164" s="148"/>
-      <c r="N164" s="148"/>
-      <c r="O164" s="148"/>
-      <c r="P164" s="148"/>
-      <c r="Q164" s="148"/>
-      <c r="R164" s="148"/>
-      <c r="S164" s="148"/>
-      <c r="T164" s="2"/>
-      <c r="U164" s="2"/>
-      <c r="V164" s="2"/>
-      <c r="W164" s="2"/>
-      <c r="X164" s="2"/>
-      <c r="Y164" s="2"/>
-      <c r="Z164" s="2"/>
+      <c r="M164" s="223" t="s">
+        <v>448</v>
+      </c>
+      <c r="N164" s="218" t="s">
+        <v>447</v>
+      </c>
+      <c r="O164" s="218"/>
+      <c r="P164" s="218"/>
+      <c r="Q164" s="218"/>
+      <c r="R164" s="218"/>
+      <c r="S164" s="219"/>
+      <c r="T164" s="219"/>
+      <c r="U164" s="219"/>
+      <c r="V164" s="219"/>
+      <c r="W164" s="219"/>
+      <c r="X164" s="219"/>
+      <c r="Y164" s="219"/>
+      <c r="Z164" s="219"/>
       <c r="AA164" s="4"/>
       <c r="AB164" s="16"/>
       <c r="AC164" s="1"/>
@@ -34039,17 +34173,17 @@
       <c r="A165" s="1"/>
       <c r="B165" s="33"/>
       <c r="C165" s="73">
-        <f>INT($C$140)+3</f>
+        <f t="shared" ref="C165:C181" si="18">INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D165" s="4"/>
       <c r="E165" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F165" s="5"/>
       <c r="G165" s="4"/>
       <c r="H165" s="31" t="s">
-        <v>373</v>
+        <v>265</v>
       </c>
       <c r="I165" s="31">
         <v>0</v>
@@ -34058,21 +34192,43 @@
       <c r="K165" s="148"/>
       <c r="L165" s="148"/>
       <c r="M165" s="148"/>
-      <c r="N165" s="56" t="s">
+      <c r="N165" s="217" t="s">
         <v>422</v>
       </c>
-      <c r="O165" s="148"/>
-      <c r="P165" s="148"/>
-      <c r="Q165" s="148"/>
-      <c r="R165" s="148"/>
-      <c r="S165" s="148"/>
-      <c r="T165" s="2"/>
-      <c r="U165" s="2"/>
-      <c r="V165" s="2"/>
-      <c r="W165" s="2"/>
-      <c r="X165" s="2"/>
-      <c r="Y165" s="2"/>
-      <c r="Z165" s="2"/>
+      <c r="O165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="P165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="Q165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="R165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="S165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="T165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="U165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="V165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="W165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="X165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z165" s="217"/>
       <c r="AA165" s="4"/>
       <c r="AB165" s="16"/>
       <c r="AC165" s="1"/>
@@ -34083,17 +34239,17 @@
       <c r="A166" s="1"/>
       <c r="B166" s="33"/>
       <c r="C166" s="73">
-        <f>INT(C$140+3)</f>
+        <f>INT($C$140)+3</f>
         <v>4</v>
       </c>
       <c r="D166" s="4"/>
       <c r="E166" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F166" s="5"/>
       <c r="G166" s="4"/>
       <c r="H166" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="I166" s="31">
         <v>0</v>
@@ -34102,9 +34258,7 @@
       <c r="K166" s="148"/>
       <c r="L166" s="148"/>
       <c r="M166" s="148"/>
-      <c r="N166" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N166" s="148"/>
       <c r="O166" s="148"/>
       <c r="P166" s="148"/>
       <c r="Q166" s="148"/>
@@ -34127,17 +34281,17 @@
       <c r="A167" s="1"/>
       <c r="B167" s="33"/>
       <c r="C167" s="73">
-        <f>INT(C$140+3)</f>
+        <f>INT($C$140)+3</f>
         <v>4</v>
       </c>
       <c r="D167" s="4"/>
       <c r="E167" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F167" s="5"/>
       <c r="G167" s="4"/>
       <c r="H167" s="31" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="I167" s="31">
         <v>0</v>
@@ -34171,17 +34325,17 @@
       <c r="A168" s="1"/>
       <c r="B168" s="33"/>
       <c r="C168" s="73">
-        <f t="shared" si="18"/>
+        <f>INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D168" s="4"/>
       <c r="E168" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F168" s="5"/>
       <c r="G168" s="4"/>
       <c r="H168" s="31" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="I168" s="31">
         <v>0</v>
@@ -34215,17 +34369,17 @@
       <c r="A169" s="1"/>
       <c r="B169" s="33"/>
       <c r="C169" s="73">
-        <f t="shared" si="18"/>
+        <f>INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D169" s="4"/>
       <c r="E169" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F169" s="5"/>
       <c r="G169" s="4"/>
       <c r="H169" s="31" t="s">
-        <v>397</v>
+        <v>375</v>
       </c>
       <c r="I169" s="31">
         <v>0</v>
@@ -34264,12 +34418,12 @@
       </c>
       <c r="D170" s="4"/>
       <c r="E170" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F170" s="5"/>
       <c r="G170" s="4"/>
       <c r="H170" s="31" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="I170" s="31">
         <v>0</v>
@@ -34278,7 +34432,9 @@
       <c r="K170" s="148"/>
       <c r="L170" s="148"/>
       <c r="M170" s="148"/>
-      <c r="N170" s="148"/>
+      <c r="N170" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="O170" s="148"/>
       <c r="P170" s="148"/>
       <c r="Q170" s="148"/>
@@ -34306,12 +34462,12 @@
       </c>
       <c r="D171" s="4"/>
       <c r="E171" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F171" s="5"/>
       <c r="G171" s="4"/>
       <c r="H171" s="31" t="s">
-        <v>377</v>
+        <v>397</v>
       </c>
       <c r="I171" s="31">
         <v>0</v>
@@ -34320,7 +34476,9 @@
       <c r="K171" s="148"/>
       <c r="L171" s="148"/>
       <c r="M171" s="148"/>
-      <c r="N171" s="148"/>
+      <c r="N171" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="O171" s="148"/>
       <c r="P171" s="148"/>
       <c r="Q171" s="148"/>
@@ -34348,12 +34506,12 @@
       </c>
       <c r="D172" s="4"/>
       <c r="E172" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F172" s="5"/>
       <c r="G172" s="4"/>
       <c r="H172" s="31" t="s">
-        <v>260</v>
+        <v>376</v>
       </c>
       <c r="I172" s="31">
         <v>0</v>
@@ -34362,24 +34520,18 @@
       <c r="K172" s="148"/>
       <c r="L172" s="148"/>
       <c r="M172" s="148"/>
-      <c r="N172" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N172" s="148"/>
       <c r="O172" s="148"/>
       <c r="P172" s="148"/>
       <c r="Q172" s="148"/>
-      <c r="R172" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="R172" s="148"/>
       <c r="S172" s="148"/>
       <c r="T172" s="2"/>
       <c r="U172" s="2"/>
       <c r="V172" s="2"/>
       <c r="W172" s="2"/>
       <c r="X172" s="2"/>
-      <c r="Y172" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="Y172" s="2"/>
       <c r="Z172" s="2"/>
       <c r="AA172" s="4"/>
       <c r="AB172" s="16"/>
@@ -34396,12 +34548,12 @@
       </c>
       <c r="D173" s="4"/>
       <c r="E173" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F173" s="5"/>
       <c r="G173" s="4"/>
       <c r="H173" s="31" t="s">
-        <v>261</v>
+        <v>377</v>
       </c>
       <c r="I173" s="31">
         <v>0</v>
@@ -34410,24 +34562,18 @@
       <c r="K173" s="148"/>
       <c r="L173" s="148"/>
       <c r="M173" s="148"/>
-      <c r="N173" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N173" s="148"/>
       <c r="O173" s="148"/>
       <c r="P173" s="148"/>
       <c r="Q173" s="148"/>
-      <c r="R173" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="R173" s="148"/>
       <c r="S173" s="148"/>
       <c r="T173" s="2"/>
       <c r="U173" s="2"/>
       <c r="V173" s="2"/>
       <c r="W173" s="2"/>
       <c r="X173" s="2"/>
-      <c r="Y173" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="Y173" s="2"/>
       <c r="Z173" s="2"/>
       <c r="AA173" s="4"/>
       <c r="AB173" s="16"/>
@@ -34444,12 +34590,12 @@
       </c>
       <c r="D174" s="4"/>
       <c r="E174" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F174" s="5"/>
       <c r="G174" s="4"/>
       <c r="H174" s="31" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I174" s="31">
         <v>0</v>
@@ -34468,21 +34614,11 @@
         <v>422</v>
       </c>
       <c r="S174" s="148"/>
-      <c r="T174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="U174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="V174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="W174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="X174" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="T174" s="2"/>
+      <c r="U174" s="2"/>
+      <c r="V174" s="2"/>
+      <c r="W174" s="2"/>
+      <c r="X174" s="2"/>
       <c r="Y174" s="56" t="s">
         <v>422</v>
       </c>
@@ -34502,12 +34638,12 @@
       </c>
       <c r="D175" s="4"/>
       <c r="E175" s="5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F175" s="5"/>
       <c r="G175" s="4"/>
       <c r="H175" s="31" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="I175" s="31">
         <v>0</v>
@@ -34516,18 +34652,24 @@
       <c r="K175" s="148"/>
       <c r="L175" s="148"/>
       <c r="M175" s="148"/>
-      <c r="N175" s="148"/>
+      <c r="N175" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="O175" s="148"/>
       <c r="P175" s="148"/>
       <c r="Q175" s="148"/>
-      <c r="R175" s="148"/>
+      <c r="R175" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="S175" s="148"/>
       <c r="T175" s="2"/>
       <c r="U175" s="2"/>
       <c r="V175" s="2"/>
       <c r="W175" s="2"/>
       <c r="X175" s="2"/>
-      <c r="Y175" s="2"/>
+      <c r="Y175" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="Z175" s="2"/>
       <c r="AA175" s="4"/>
       <c r="AB175" s="16"/>
@@ -34544,12 +34686,12 @@
       </c>
       <c r="D176" s="4"/>
       <c r="E176" s="5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F176" s="5"/>
       <c r="G176" s="4"/>
       <c r="H176" s="31" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="I176" s="31">
         <v>0</v>
@@ -34563,15 +34705,11 @@
       </c>
       <c r="O176" s="148"/>
       <c r="P176" s="148"/>
-      <c r="Q176" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="Q176" s="148"/>
       <c r="R176" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="S176" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="S176" s="148"/>
       <c r="T176" s="56" t="s">
         <v>422</v>
       </c>
@@ -34590,7 +34728,7 @@
       <c r="Y176" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Z176" s="56"/>
+      <c r="Z176" s="2"/>
       <c r="AA176" s="4"/>
       <c r="AB176" s="16"/>
       <c r="AC176" s="1"/>
@@ -34606,12 +34744,12 @@
       </c>
       <c r="D177" s="4"/>
       <c r="E177" s="5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F177" s="5"/>
       <c r="G177" s="4"/>
       <c r="H177" s="31" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="I177" s="31">
         <v>0</v>
@@ -34620,39 +34758,19 @@
       <c r="K177" s="148"/>
       <c r="L177" s="148"/>
       <c r="M177" s="148"/>
-      <c r="N177" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N177" s="148"/>
       <c r="O177" s="148"/>
       <c r="P177" s="148"/>
-      <c r="Q177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="R177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="S177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="T177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="U177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="V177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="W177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="X177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="Y177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="Z177" s="56"/>
+      <c r="Q177" s="148"/>
+      <c r="R177" s="148"/>
+      <c r="S177" s="148"/>
+      <c r="T177" s="2"/>
+      <c r="U177" s="2"/>
+      <c r="V177" s="2"/>
+      <c r="W177" s="2"/>
+      <c r="X177" s="2"/>
+      <c r="Y177" s="2"/>
+      <c r="Z177" s="2"/>
       <c r="AA177" s="4"/>
       <c r="AB177" s="16"/>
       <c r="AC177" s="1"/>
@@ -34668,12 +34786,12 @@
       </c>
       <c r="D178" s="4"/>
       <c r="E178" s="5">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F178" s="5"/>
       <c r="G178" s="4"/>
       <c r="H178" s="31" t="s">
-        <v>371</v>
+        <v>258</v>
       </c>
       <c r="I178" s="31">
         <v>0</v>
@@ -34730,12 +34848,12 @@
       </c>
       <c r="D179" s="4"/>
       <c r="E179" s="5">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F179" s="5"/>
       <c r="G179" s="4"/>
       <c r="H179" s="31" t="s">
-        <v>438</v>
+        <v>259</v>
       </c>
       <c r="I179" s="31">
         <v>0</v>
@@ -34787,17 +34905,17 @@
       <c r="A180" s="1"/>
       <c r="B180" s="33"/>
       <c r="C180" s="73">
-        <f>INT(C$140+3)</f>
+        <f t="shared" si="18"/>
         <v>4</v>
       </c>
       <c r="D180" s="4"/>
       <c r="E180" s="5">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F180" s="5"/>
       <c r="G180" s="4"/>
       <c r="H180" s="31" t="s">
-        <v>443</v>
+        <v>371</v>
       </c>
       <c r="I180" s="31">
         <v>0</v>
@@ -34849,17 +34967,17 @@
       <c r="A181" s="1"/>
       <c r="B181" s="33"/>
       <c r="C181" s="73">
-        <f>INT(C$140+3)</f>
+        <f t="shared" si="18"/>
         <v>4</v>
       </c>
       <c r="D181" s="4"/>
       <c r="E181" s="5">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F181" s="5"/>
       <c r="G181" s="4"/>
       <c r="H181" s="31" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="I181" s="31">
         <v>0</v>
@@ -34868,573 +34986,623 @@
       <c r="K181" s="148"/>
       <c r="L181" s="148"/>
       <c r="M181" s="148"/>
-      <c r="N181" s="216" t="s">
+      <c r="N181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="O181" s="215"/>
-      <c r="P181" s="215"/>
-      <c r="Q181" s="215"/>
-      <c r="R181" s="216" t="s">
+      <c r="O181" s="148"/>
+      <c r="P181" s="148"/>
+      <c r="Q181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="S181" s="215"/>
-      <c r="T181" s="216" t="s">
+      <c r="R181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="U181" s="216" t="s">
+      <c r="S181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="V181" s="216" t="s">
+      <c r="T181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="W181" s="216" t="s">
+      <c r="U181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="X181" s="216" t="s">
+      <c r="V181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Y181" s="216" t="s">
+      <c r="W181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Z181" s="216"/>
+      <c r="X181" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y181" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z181" s="56"/>
       <c r="AA181" s="4"/>
       <c r="AB181" s="16"/>
       <c r="AC181" s="1"/>
       <c r="AD181" s="1"/>
       <c r="AE181" s="1"/>
     </row>
-    <row r="182" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A182" s="1"/>
       <c r="B182" s="33"/>
       <c r="C182" s="73">
-        <f>INT($C$140)+3.005</f>
-        <v>4.0049999999999999</v>
+        <f>INT(C$140+3)</f>
+        <v>4</v>
       </c>
       <c r="D182" s="4"/>
-      <c r="E182" s="4"/>
-      <c r="F182" s="4"/>
+      <c r="E182" s="5">
+        <v>18</v>
+      </c>
+      <c r="F182" s="5"/>
       <c r="G182" s="4"/>
-      <c r="H182" s="4"/>
-      <c r="I182" s="4"/>
-      <c r="J182" s="4"/>
-      <c r="K182" s="4"/>
-      <c r="L182" s="4"/>
-      <c r="M182" s="4"/>
-      <c r="N182" s="4"/>
-      <c r="O182" s="4"/>
-      <c r="P182" s="4"/>
-      <c r="Q182" s="4"/>
-      <c r="R182" s="4"/>
-      <c r="S182" s="4"/>
-      <c r="T182" s="4"/>
-      <c r="U182" s="4"/>
-      <c r="V182" s="4"/>
-      <c r="W182" s="4"/>
-      <c r="X182" s="4"/>
-      <c r="Y182" s="4"/>
-      <c r="Z182" s="4"/>
-      <c r="AA182" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="H182" s="31" t="s">
+        <v>442</v>
+      </c>
+      <c r="I182" s="31">
+        <v>0</v>
+      </c>
+      <c r="J182" s="148"/>
+      <c r="K182" s="148"/>
+      <c r="L182" s="148"/>
+      <c r="M182" s="148"/>
+      <c r="N182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="O182" s="148"/>
+      <c r="P182" s="148"/>
+      <c r="Q182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="R182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="S182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="T182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="U182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="V182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="W182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="X182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z182" s="56"/>
+      <c r="AA182" s="4"/>
       <c r="AB182" s="16"/>
       <c r="AC182" s="1"/>
       <c r="AD182" s="1"/>
       <c r="AE182" s="1"/>
     </row>
-    <row r="183" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A183" s="1"/>
       <c r="B183" s="33"/>
       <c r="C183" s="73">
-        <f>INT($C$140)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>INT(C$140+3)</f>
+        <v>4</v>
       </c>
       <c r="D183" s="4"/>
-      <c r="E183" s="4"/>
-      <c r="F183" s="4"/>
+      <c r="E183" s="5">
+        <v>19</v>
+      </c>
+      <c r="F183" s="5"/>
       <c r="G183" s="4"/>
-      <c r="H183" s="4"/>
-      <c r="I183" s="4"/>
-      <c r="J183" s="4"/>
-      <c r="K183" s="4"/>
-      <c r="L183" s="4"/>
-      <c r="M183" s="4"/>
-      <c r="N183" s="4"/>
-      <c r="O183" s="4"/>
-      <c r="P183" s="4"/>
-      <c r="Q183" s="4"/>
-      <c r="R183" s="4"/>
-      <c r="S183" s="4"/>
-      <c r="T183" s="4"/>
-      <c r="U183" s="4"/>
-      <c r="V183" s="4"/>
-      <c r="W183" s="4"/>
-      <c r="X183" s="4"/>
-      <c r="Y183" s="4"/>
-      <c r="Z183" s="4"/>
+      <c r="H183" s="31" t="s">
+        <v>443</v>
+      </c>
+      <c r="I183" s="31">
+        <v>0</v>
+      </c>
+      <c r="J183" s="148"/>
+      <c r="K183" s="148"/>
+      <c r="L183" s="148"/>
+      <c r="M183" s="148"/>
+      <c r="N183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="O183" s="215"/>
+      <c r="P183" s="215"/>
+      <c r="Q183" s="215"/>
+      <c r="R183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="S183" s="215"/>
+      <c r="T183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="U183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="V183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="W183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="X183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z183" s="216"/>
       <c r="AA183" s="4"/>
       <c r="AB183" s="16"/>
       <c r="AC183" s="1"/>
       <c r="AD183" s="1"/>
       <c r="AE183" s="1"/>
     </row>
-    <row r="184" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
-      <c r="B184" s="35"/>
-      <c r="C184" s="76">
-        <f>INT($C$140)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D184" s="17"/>
-      <c r="E184" s="17"/>
-      <c r="F184" s="17"/>
-      <c r="G184" s="17"/>
-      <c r="H184" s="17"/>
-      <c r="I184" s="17"/>
-      <c r="J184" s="17"/>
-      <c r="K184" s="17"/>
-      <c r="L184" s="17"/>
-      <c r="M184" s="17"/>
-      <c r="N184" s="17"/>
-      <c r="O184" s="17"/>
-      <c r="P184" s="17"/>
-      <c r="Q184" s="17"/>
-      <c r="R184" s="17"/>
-      <c r="S184" s="17"/>
-      <c r="T184" s="17"/>
-      <c r="U184" s="17"/>
-      <c r="V184" s="17"/>
-      <c r="W184" s="17"/>
-      <c r="X184" s="17"/>
-      <c r="Y184" s="17"/>
-      <c r="Z184" s="17"/>
-      <c r="AA184" s="17"/>
-      <c r="AB184" s="18" t="s">
-        <v>1</v>
-      </c>
+      <c r="B184" s="33"/>
+      <c r="C184" s="73">
+        <f>INT($C$140)+3.005</f>
+        <v>4.0049999999999999</v>
+      </c>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+      <c r="H184" s="4"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="4"/>
+      <c r="K184" s="4"/>
+      <c r="L184" s="4"/>
+      <c r="M184" s="4"/>
+      <c r="N184" s="4"/>
+      <c r="O184" s="4"/>
+      <c r="P184" s="4"/>
+      <c r="Q184" s="4"/>
+      <c r="R184" s="4"/>
+      <c r="S184" s="4"/>
+      <c r="T184" s="4"/>
+      <c r="U184" s="4"/>
+      <c r="V184" s="4"/>
+      <c r="W184" s="4"/>
+      <c r="X184" s="4"/>
+      <c r="Y184" s="4"/>
+      <c r="Z184" s="4"/>
+      <c r="AA184" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB184" s="16"/>
       <c r="AC184" s="1"/>
       <c r="AD184" s="1"/>
       <c r="AE184" s="1"/>
     </row>
-    <row r="185" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
-      <c r="B185" s="19"/>
-      <c r="C185" s="77">
-        <f>INT($C$140)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D185" s="19"/>
-      <c r="E185" s="19"/>
-      <c r="F185" s="19"/>
-      <c r="G185" s="19"/>
-      <c r="H185" s="19"/>
-      <c r="I185" s="19"/>
-      <c r="J185" s="19"/>
-      <c r="K185" s="19"/>
-      <c r="L185" s="19"/>
-      <c r="M185" s="19"/>
-      <c r="N185" s="19"/>
-      <c r="O185" s="19"/>
-      <c r="P185" s="19"/>
-      <c r="Q185" s="19"/>
-      <c r="R185" s="19"/>
-      <c r="S185" s="19"/>
-      <c r="T185" s="19"/>
-      <c r="U185" s="19"/>
-      <c r="V185" s="19"/>
-      <c r="W185" s="19"/>
-      <c r="X185" s="19"/>
-      <c r="Y185" s="19"/>
-      <c r="Z185" s="19"/>
-      <c r="AA185" s="19"/>
-      <c r="AB185" s="19"/>
+      <c r="B185" s="33"/>
+      <c r="C185" s="73">
+        <f>INT($C$140)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D185" s="4"/>
+      <c r="E185" s="4"/>
+      <c r="F185" s="4"/>
+      <c r="G185" s="4"/>
+      <c r="H185" s="4"/>
+      <c r="I185" s="4"/>
+      <c r="J185" s="4"/>
+      <c r="K185" s="4"/>
+      <c r="L185" s="4"/>
+      <c r="M185" s="4"/>
+      <c r="N185" s="4"/>
+      <c r="O185" s="4"/>
+      <c r="P185" s="4"/>
+      <c r="Q185" s="4"/>
+      <c r="R185" s="4"/>
+      <c r="S185" s="4"/>
+      <c r="T185" s="4"/>
+      <c r="U185" s="4"/>
+      <c r="V185" s="4"/>
+      <c r="W185" s="4"/>
+      <c r="X185" s="4"/>
+      <c r="Y185" s="4"/>
+      <c r="Z185" s="4"/>
+      <c r="AA185" s="4"/>
+      <c r="AB185" s="16"/>
       <c r="AC185" s="1"/>
       <c r="AD185" s="1"/>
       <c r="AE185" s="1"/>
     </row>
-    <row r="186" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
-      <c r="B186" s="1"/>
-      <c r="C186" s="73">
-        <f>INT($C$140)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D186" s="1"/>
-      <c r="E186" s="1"/>
-      <c r="F186" s="1"/>
-      <c r="G186" s="1"/>
-      <c r="H186" s="1"/>
-      <c r="I186" s="1"/>
-      <c r="J186" s="1"/>
-      <c r="K186" s="1"/>
-      <c r="L186" s="1"/>
-      <c r="M186" s="1"/>
-      <c r="N186" s="1"/>
-      <c r="O186" s="1"/>
-      <c r="P186" s="1"/>
-      <c r="Q186" s="1"/>
-      <c r="R186" s="1"/>
-      <c r="S186" s="1"/>
-      <c r="T186" s="1"/>
-      <c r="U186" s="1"/>
-      <c r="V186" s="1"/>
-      <c r="W186" s="1"/>
-      <c r="X186" s="1"/>
-      <c r="Y186" s="1"/>
-      <c r="Z186" s="1"/>
-      <c r="AA186" s="1"/>
-      <c r="AB186" s="1"/>
+      <c r="B186" s="35"/>
+      <c r="C186" s="76">
+        <f>INT($C$140)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D186" s="17"/>
+      <c r="E186" s="17"/>
+      <c r="F186" s="17"/>
+      <c r="G186" s="17"/>
+      <c r="H186" s="17"/>
+      <c r="I186" s="17"/>
+      <c r="J186" s="17"/>
+      <c r="K186" s="17"/>
+      <c r="L186" s="17"/>
+      <c r="M186" s="17"/>
+      <c r="N186" s="17"/>
+      <c r="O186" s="17"/>
+      <c r="P186" s="17"/>
+      <c r="Q186" s="17"/>
+      <c r="R186" s="17"/>
+      <c r="S186" s="17"/>
+      <c r="T186" s="17"/>
+      <c r="U186" s="17"/>
+      <c r="V186" s="17"/>
+      <c r="W186" s="17"/>
+      <c r="X186" s="17"/>
+      <c r="Y186" s="17"/>
+      <c r="Z186" s="17"/>
+      <c r="AA186" s="17"/>
+      <c r="AB186" s="18" t="s">
+        <v>1</v>
+      </c>
       <c r="AC186" s="1"/>
       <c r="AD186" s="1"/>
       <c r="AE186" s="1"/>
     </row>
-    <row r="187" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
-      <c r="B187" s="1"/>
-      <c r="C187" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D187" s="1"/>
-      <c r="E187" s="1"/>
-      <c r="F187" s="1"/>
-      <c r="G187" s="1"/>
-      <c r="H187" s="1"/>
-      <c r="I187" s="1"/>
-      <c r="J187" s="1"/>
-      <c r="K187" s="1"/>
-      <c r="L187" s="1"/>
-      <c r="M187" s="1"/>
-      <c r="N187" s="1"/>
-      <c r="O187" s="1"/>
-      <c r="P187" s="1"/>
-      <c r="Q187" s="1"/>
-      <c r="R187" s="1"/>
-      <c r="S187" s="1"/>
-      <c r="T187" s="1"/>
-      <c r="U187" s="1"/>
-      <c r="V187" s="1"/>
-      <c r="W187" s="1"/>
-      <c r="X187" s="1"/>
-      <c r="Y187" s="1"/>
-      <c r="Z187" s="1"/>
-      <c r="AA187" s="1"/>
-      <c r="AB187" s="1"/>
+      <c r="B187" s="19"/>
+      <c r="C187" s="77">
+        <f>INT($C$140)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D187" s="19"/>
+      <c r="E187" s="19"/>
+      <c r="F187" s="19"/>
+      <c r="G187" s="19"/>
+      <c r="H187" s="19"/>
+      <c r="I187" s="19"/>
+      <c r="J187" s="19"/>
+      <c r="K187" s="19"/>
+      <c r="L187" s="19"/>
+      <c r="M187" s="19"/>
+      <c r="N187" s="19"/>
+      <c r="O187" s="19"/>
+      <c r="P187" s="19"/>
+      <c r="Q187" s="19"/>
+      <c r="R187" s="19"/>
+      <c r="S187" s="19"/>
+      <c r="T187" s="19"/>
+      <c r="U187" s="19"/>
+      <c r="V187" s="19"/>
+      <c r="W187" s="19"/>
+      <c r="X187" s="19"/>
+      <c r="Y187" s="19"/>
+      <c r="Z187" s="19"/>
+      <c r="AA187" s="19"/>
+      <c r="AB187" s="19"/>
       <c r="AC187" s="1"/>
       <c r="AD187" s="1"/>
       <c r="AE187" s="1"/>
     </row>
-    <row r="188" spans="1:31" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
-      <c r="B188" s="20"/>
-      <c r="C188" s="74">
-        <f>INT($C$191)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D188" s="20"/>
-      <c r="E188" s="20"/>
-      <c r="F188" s="20"/>
-      <c r="G188" s="20"/>
-      <c r="H188" s="20"/>
-      <c r="I188" s="20"/>
-      <c r="J188" s="20"/>
-      <c r="K188" s="20"/>
-      <c r="L188" s="20"/>
-      <c r="M188" s="20"/>
-      <c r="N188" s="20"/>
-      <c r="O188" s="20"/>
-      <c r="P188" s="20"/>
-      <c r="Q188" s="20"/>
-      <c r="R188" s="20"/>
-      <c r="S188" s="20"/>
-      <c r="T188" s="20"/>
-      <c r="U188" s="20"/>
-      <c r="V188" s="20"/>
-      <c r="W188" s="20"/>
-      <c r="X188" s="20"/>
-      <c r="Y188" s="20"/>
-      <c r="Z188" s="20"/>
-      <c r="AA188" s="20"/>
-      <c r="AB188" s="20"/>
+      <c r="B188" s="1"/>
+      <c r="C188" s="73">
+        <f>INT($C$140)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D188" s="1"/>
+      <c r="E188" s="1"/>
+      <c r="F188" s="1"/>
+      <c r="G188" s="1"/>
+      <c r="H188" s="1"/>
+      <c r="I188" s="1"/>
+      <c r="J188" s="1"/>
+      <c r="K188" s="1"/>
+      <c r="L188" s="1"/>
+      <c r="M188" s="1"/>
+      <c r="N188" s="1"/>
+      <c r="O188" s="1"/>
+      <c r="P188" s="1"/>
+      <c r="Q188" s="1"/>
+      <c r="R188" s="1"/>
+      <c r="S188" s="1"/>
+      <c r="T188" s="1"/>
+      <c r="U188" s="1"/>
+      <c r="V188" s="1"/>
+      <c r="W188" s="1"/>
+      <c r="X188" s="1"/>
+      <c r="Y188" s="1"/>
+      <c r="Z188" s="1"/>
+      <c r="AA188" s="1"/>
+      <c r="AB188" s="1"/>
       <c r="AC188" s="1"/>
       <c r="AD188" s="1"/>
       <c r="AE188" s="1"/>
     </row>
-    <row r="189" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
-      <c r="B189" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="C189" s="75">
-        <f>INT($C$191)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D189" s="14"/>
-      <c r="E189" s="14"/>
-      <c r="F189" s="14"/>
-      <c r="G189" s="14"/>
-      <c r="H189" s="14"/>
-      <c r="I189" s="14"/>
-      <c r="J189" s="14"/>
-      <c r="K189" s="14"/>
-      <c r="L189" s="14"/>
-      <c r="M189" s="14"/>
-      <c r="N189" s="14"/>
-      <c r="O189" s="14"/>
-      <c r="P189" s="14"/>
-      <c r="Q189" s="14"/>
-      <c r="R189" s="14"/>
-      <c r="S189" s="14"/>
-      <c r="T189" s="14"/>
-      <c r="U189" s="14"/>
-      <c r="V189" s="14"/>
-      <c r="W189" s="14"/>
-      <c r="X189" s="14"/>
-      <c r="Y189" s="14"/>
-      <c r="Z189" s="14"/>
-      <c r="AA189" s="14"/>
-      <c r="AB189" s="15"/>
+      <c r="B189" s="1"/>
+      <c r="C189" s="73">
+        <f>INT($C$193)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D189" s="1"/>
+      <c r="E189" s="1"/>
+      <c r="F189" s="1"/>
+      <c r="G189" s="1"/>
+      <c r="H189" s="1"/>
+      <c r="I189" s="1"/>
+      <c r="J189" s="1"/>
+      <c r="K189" s="1"/>
+      <c r="L189" s="1"/>
+      <c r="M189" s="1"/>
+      <c r="N189" s="1"/>
+      <c r="O189" s="1"/>
+      <c r="P189" s="1"/>
+      <c r="Q189" s="1"/>
+      <c r="R189" s="1"/>
+      <c r="S189" s="1"/>
+      <c r="T189" s="1"/>
+      <c r="U189" s="1"/>
+      <c r="V189" s="1"/>
+      <c r="W189" s="1"/>
+      <c r="X189" s="1"/>
+      <c r="Y189" s="1"/>
+      <c r="Z189" s="1"/>
+      <c r="AA189" s="1"/>
+      <c r="AB189" s="1"/>
       <c r="AC189" s="1"/>
       <c r="AD189" s="1"/>
       <c r="AE189" s="1"/>
     </row>
-    <row r="190" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:31" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A190" s="1"/>
-      <c r="B190" s="33"/>
-      <c r="C190" s="73">
-        <f>INT(MAX($C$199:$C$203))+1</f>
-        <v>5</v>
-      </c>
-      <c r="D190" s="3"/>
-      <c r="E190" s="3"/>
-      <c r="F190" s="3"/>
-      <c r="G190" s="3"/>
-      <c r="H190" s="27"/>
-      <c r="I190" s="27"/>
-      <c r="J190" s="27"/>
-      <c r="K190" s="27"/>
-      <c r="L190" s="27"/>
-      <c r="M190" s="27"/>
-      <c r="N190" s="27"/>
-      <c r="O190" s="27"/>
-      <c r="P190" s="27"/>
-      <c r="Q190" s="27"/>
-      <c r="R190" s="27"/>
-      <c r="S190" s="27"/>
-      <c r="T190" s="27"/>
-      <c r="U190" s="27"/>
-      <c r="V190" s="27"/>
-      <c r="W190" s="27"/>
-      <c r="X190" s="27"/>
-      <c r="Y190" s="27"/>
-      <c r="Z190" s="27"/>
-      <c r="AA190" s="3"/>
-      <c r="AB190" s="16"/>
+      <c r="B190" s="20"/>
+      <c r="C190" s="74">
+        <f>INT($C$193)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D190" s="20"/>
+      <c r="E190" s="20"/>
+      <c r="F190" s="20"/>
+      <c r="G190" s="20"/>
+      <c r="H190" s="20"/>
+      <c r="I190" s="20"/>
+      <c r="J190" s="20"/>
+      <c r="K190" s="20"/>
+      <c r="L190" s="20"/>
+      <c r="M190" s="20"/>
+      <c r="N190" s="20"/>
+      <c r="O190" s="20"/>
+      <c r="P190" s="20"/>
+      <c r="Q190" s="20"/>
+      <c r="R190" s="20"/>
+      <c r="S190" s="20"/>
+      <c r="T190" s="20"/>
+      <c r="U190" s="20"/>
+      <c r="V190" s="20"/>
+      <c r="W190" s="20"/>
+      <c r="X190" s="20"/>
+      <c r="Y190" s="20"/>
+      <c r="Z190" s="20"/>
+      <c r="AA190" s="20"/>
+      <c r="AB190" s="20"/>
       <c r="AC190" s="1"/>
       <c r="AD190" s="1"/>
       <c r="AE190" s="1"/>
     </row>
-    <row r="191" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
-      <c r="B191" s="33"/>
-      <c r="C191" s="73">
-        <v>1.02</v>
-      </c>
-      <c r="D191" s="21"/>
-      <c r="E191" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="F191" s="25"/>
-      <c r="G191" s="12"/>
-      <c r="H191" s="147" t="str">
-        <f>COUNTIFS($B$1:$B191, "«")&amp;" Feed Pool definitions"</f>
-        <v>6 Feed Pool definitions</v>
-      </c>
-      <c r="I191" s="6"/>
-      <c r="J191" s="6"/>
-      <c r="K191" s="6"/>
-      <c r="L191" s="6"/>
-      <c r="M191" s="6"/>
-      <c r="N191" s="6"/>
-      <c r="O191" s="6"/>
-      <c r="P191" s="6"/>
-      <c r="Q191" s="6"/>
-      <c r="R191" s="6"/>
-      <c r="S191" s="6"/>
-      <c r="T191" s="6"/>
-      <c r="U191" s="6"/>
-      <c r="V191" s="6"/>
-      <c r="W191" s="6"/>
-      <c r="X191" s="6"/>
-      <c r="Y191" s="6"/>
-      <c r="Z191" s="6"/>
-      <c r="AA191" s="10"/>
-      <c r="AB191" s="16"/>
+      <c r="B191" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C191" s="75">
+        <f>INT($C$193)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D191" s="14"/>
+      <c r="E191" s="14"/>
+      <c r="F191" s="14"/>
+      <c r="G191" s="14"/>
+      <c r="H191" s="14"/>
+      <c r="I191" s="14"/>
+      <c r="J191" s="14"/>
+      <c r="K191" s="14"/>
+      <c r="L191" s="14"/>
+      <c r="M191" s="14"/>
+      <c r="N191" s="14"/>
+      <c r="O191" s="14"/>
+      <c r="P191" s="14"/>
+      <c r="Q191" s="14"/>
+      <c r="R191" s="14"/>
+      <c r="S191" s="14"/>
+      <c r="T191" s="14"/>
+      <c r="U191" s="14"/>
+      <c r="V191" s="14"/>
+      <c r="W191" s="14"/>
+      <c r="X191" s="14"/>
+      <c r="Y191" s="14"/>
+      <c r="Z191" s="14"/>
+      <c r="AA191" s="14"/>
+      <c r="AB191" s="15"/>
       <c r="AC191" s="1"/>
       <c r="AD191" s="1"/>
       <c r="AE191" s="1"/>
     </row>
-    <row r="192" spans="1:31" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
       <c r="B192" s="33"/>
       <c r="C192" s="73">
-        <f>INT($C$191)+1.02</f>
-        <v>2.02</v>
-      </c>
-      <c r="D192" s="21"/>
-      <c r="E192" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="F192" s="28">
-        <v>1</v>
-      </c>
-      <c r="G192" s="13"/>
-      <c r="H192" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="I192" s="7"/>
-      <c r="J192" s="7"/>
-      <c r="K192" s="7"/>
-      <c r="L192" s="7"/>
-      <c r="M192" s="7"/>
-      <c r="N192" s="7"/>
-      <c r="O192" s="7"/>
-      <c r="P192" s="7"/>
-      <c r="Q192" s="7"/>
-      <c r="R192" s="7"/>
-      <c r="S192" s="7"/>
-      <c r="T192" s="7"/>
-      <c r="U192" s="7"/>
-      <c r="V192" s="7"/>
-      <c r="W192" s="7"/>
-      <c r="X192" s="7"/>
-      <c r="Y192" s="7"/>
-      <c r="Z192" s="7"/>
-      <c r="AA192" s="11"/>
+        <f>INT(MAX($C$201:$C$205))+1</f>
+        <v>5</v>
+      </c>
+      <c r="D192" s="3"/>
+      <c r="E192" s="3"/>
+      <c r="F192" s="3"/>
+      <c r="G192" s="3"/>
+      <c r="H192" s="27"/>
+      <c r="I192" s="27"/>
+      <c r="J192" s="27"/>
+      <c r="K192" s="27"/>
+      <c r="L192" s="27"/>
+      <c r="M192" s="27"/>
+      <c r="N192" s="27"/>
+      <c r="O192" s="27"/>
+      <c r="P192" s="27"/>
+      <c r="Q192" s="27"/>
+      <c r="R192" s="27"/>
+      <c r="S192" s="27"/>
+      <c r="T192" s="27"/>
+      <c r="U192" s="27"/>
+      <c r="V192" s="27"/>
+      <c r="W192" s="27"/>
+      <c r="X192" s="27"/>
+      <c r="Y192" s="27"/>
+      <c r="Z192" s="27"/>
+      <c r="AA192" s="3"/>
       <c r="AB192" s="16"/>
       <c r="AC192" s="1"/>
       <c r="AD192" s="1"/>
       <c r="AE192" s="1"/>
     </row>
-    <row r="193" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
       <c r="B193" s="33"/>
       <c r="C193" s="73">
-        <f>INT($C$191)+2.005</f>
-        <v>3.0049999999999999</v>
-      </c>
-      <c r="D193" s="3"/>
-      <c r="E193" s="3"/>
-      <c r="F193" s="3"/>
-      <c r="G193" s="3"/>
-      <c r="H193" s="3"/>
-      <c r="I193" s="3"/>
-      <c r="J193" s="3"/>
-      <c r="K193" s="3"/>
-      <c r="L193" s="3"/>
-      <c r="M193" s="3"/>
-      <c r="N193" s="3"/>
-      <c r="O193" s="3"/>
-      <c r="P193" s="3"/>
-      <c r="Q193" s="3"/>
-      <c r="R193" s="3"/>
-      <c r="S193" s="3"/>
-      <c r="T193" s="3"/>
-      <c r="U193" s="3"/>
-      <c r="V193" s="3"/>
-      <c r="W193" s="3"/>
-      <c r="X193" s="3"/>
-      <c r="Y193" s="3"/>
-      <c r="Z193" s="3"/>
-      <c r="AA193" s="3"/>
+        <v>1.02</v>
+      </c>
+      <c r="D193" s="21"/>
+      <c r="E193" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="F193" s="25"/>
+      <c r="G193" s="12"/>
+      <c r="H193" s="147" t="str">
+        <f>COUNTIFS($B$1:$B193, "«")&amp;" Feed Pool definitions"</f>
+        <v>6 Feed Pool definitions</v>
+      </c>
+      <c r="I193" s="6"/>
+      <c r="J193" s="6"/>
+      <c r="K193" s="6"/>
+      <c r="L193" s="6"/>
+      <c r="M193" s="6"/>
+      <c r="N193" s="6"/>
+      <c r="O193" s="6"/>
+      <c r="P193" s="6"/>
+      <c r="Q193" s="6"/>
+      <c r="R193" s="6"/>
+      <c r="S193" s="6"/>
+      <c r="T193" s="6"/>
+      <c r="U193" s="6"/>
+      <c r="V193" s="6"/>
+      <c r="W193" s="6"/>
+      <c r="X193" s="6"/>
+      <c r="Y193" s="6"/>
+      <c r="Z193" s="6"/>
+      <c r="AA193" s="10"/>
       <c r="AB193" s="16"/>
       <c r="AC193" s="1"/>
       <c r="AD193" s="1"/>
       <c r="AE193" s="1"/>
     </row>
-    <row r="194" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:31" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
       <c r="B194" s="33"/>
       <c r="C194" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D194" s="3"/>
-      <c r="E194" s="5"/>
-      <c r="F194" s="5"/>
-      <c r="G194" s="3"/>
-      <c r="H194" s="29"/>
-      <c r="I194" s="29"/>
-      <c r="J194" s="29"/>
-      <c r="K194" s="29"/>
-      <c r="L194" s="29"/>
-      <c r="M194" s="29"/>
-      <c r="N194" s="29"/>
-      <c r="O194" s="29"/>
-      <c r="P194" s="29"/>
-      <c r="Q194" s="29"/>
-      <c r="R194" s="29"/>
-      <c r="S194" s="29"/>
-      <c r="T194" s="29"/>
-      <c r="U194" s="29"/>
-      <c r="V194" s="29"/>
-      <c r="W194" s="29"/>
-      <c r="X194" s="29"/>
-      <c r="Y194" s="29"/>
-      <c r="Z194" s="29"/>
-      <c r="AA194" s="3"/>
+        <f>INT($C$193)+1.02</f>
+        <v>2.02</v>
+      </c>
+      <c r="D194" s="21"/>
+      <c r="E194" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F194" s="28">
+        <v>1</v>
+      </c>
+      <c r="G194" s="13"/>
+      <c r="H194" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="I194" s="7"/>
+      <c r="J194" s="7"/>
+      <c r="K194" s="7"/>
+      <c r="L194" s="7"/>
+      <c r="M194" s="7"/>
+      <c r="N194" s="7"/>
+      <c r="O194" s="7"/>
+      <c r="P194" s="7"/>
+      <c r="Q194" s="7"/>
+      <c r="R194" s="7"/>
+      <c r="S194" s="7"/>
+      <c r="T194" s="7"/>
+      <c r="U194" s="7"/>
+      <c r="V194" s="7"/>
+      <c r="W194" s="7"/>
+      <c r="X194" s="7"/>
+      <c r="Y194" s="7"/>
+      <c r="Z194" s="7"/>
+      <c r="AA194" s="11"/>
       <c r="AB194" s="16"/>
       <c r="AC194" s="1"/>
       <c r="AD194" s="1"/>
       <c r="AE194" s="1"/>
     </row>
-    <row r="195" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
       <c r="B195" s="33"/>
       <c r="C195" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
+        <f>INT($C$193)+2.005</f>
+        <v>3.0049999999999999</v>
       </c>
       <c r="D195" s="3"/>
-      <c r="E195" s="5"/>
-      <c r="F195" s="5"/>
+      <c r="E195" s="3"/>
+      <c r="F195" s="3"/>
       <c r="G195" s="3"/>
-      <c r="H195" s="29"/>
-      <c r="I195" s="29"/>
-      <c r="J195" s="29"/>
-      <c r="K195" s="29"/>
-      <c r="L195" s="29"/>
-      <c r="M195" s="29"/>
-      <c r="N195" s="29"/>
-      <c r="O195" s="29"/>
-      <c r="P195" s="29"/>
-      <c r="Q195" s="29"/>
-      <c r="R195" s="29"/>
-      <c r="S195" s="29"/>
-      <c r="T195" s="29"/>
-      <c r="U195" s="29"/>
-      <c r="V195" s="29"/>
-      <c r="W195" s="29"/>
-      <c r="X195" s="29"/>
-      <c r="Y195" s="29"/>
-      <c r="Z195" s="29"/>
+      <c r="H195" s="3"/>
+      <c r="I195" s="3"/>
+      <c r="J195" s="3"/>
+      <c r="K195" s="3"/>
+      <c r="L195" s="3"/>
+      <c r="M195" s="3"/>
+      <c r="N195" s="3"/>
+      <c r="O195" s="3"/>
+      <c r="P195" s="3"/>
+      <c r="Q195" s="3"/>
+      <c r="R195" s="3"/>
+      <c r="S195" s="3"/>
+      <c r="T195" s="3"/>
+      <c r="U195" s="3"/>
+      <c r="V195" s="3"/>
+      <c r="W195" s="3"/>
+      <c r="X195" s="3"/>
+      <c r="Y195" s="3"/>
+      <c r="Z195" s="3"/>
       <c r="AA195" s="3"/>
       <c r="AB195" s="16"/>
       <c r="AC195" s="1"/>
       <c r="AD195" s="1"/>
       <c r="AE195" s="1"/>
     </row>
-    <row r="196" spans="1:31" ht="9.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A196" s="1"/>
-      <c r="B196" s="33" t="s">
-        <v>20</v>
-      </c>
+      <c r="B196" s="33"/>
       <c r="C196" s="73">
-        <f>INT($C$191)+2.01</f>
-        <v>3.01</v>
+        <f>INT($C$193)+2</f>
+        <v>3</v>
       </c>
       <c r="D196" s="3"/>
-      <c r="E196" s="3"/>
-      <c r="F196" s="3"/>
+      <c r="E196" s="5"/>
+      <c r="F196" s="5"/>
       <c r="G196" s="3"/>
       <c r="H196" s="29"/>
       <c r="I196" s="29"/>
@@ -35461,220 +35629,222 @@
       <c r="AD196" s="1"/>
       <c r="AE196" s="1"/>
     </row>
-    <row r="197" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A197" s="1"/>
       <c r="B197" s="33"/>
       <c r="C197" s="73">
-        <f>C$190</f>
-        <v>5</v>
-      </c>
-      <c r="D197" s="4"/>
+        <f>INT($C$193)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D197" s="3"/>
       <c r="E197" s="5"/>
       <c r="F197" s="5"/>
-      <c r="G197" s="4"/>
-      <c r="H197" s="5"/>
-      <c r="I197" s="5"/>
-      <c r="J197" s="5"/>
-      <c r="K197" s="5"/>
-      <c r="L197" s="5"/>
-      <c r="M197" s="5"/>
-      <c r="N197" s="5"/>
-      <c r="O197" s="5"/>
-      <c r="P197" s="5"/>
-      <c r="Q197" s="5"/>
-      <c r="R197" s="5"/>
-      <c r="S197" s="5"/>
-      <c r="T197" s="5"/>
-      <c r="U197" s="5"/>
-      <c r="V197" s="5"/>
-      <c r="W197" s="5"/>
-      <c r="X197" s="5"/>
-      <c r="Y197" s="5"/>
-      <c r="Z197" s="5"/>
-      <c r="AA197" s="4"/>
+      <c r="G197" s="3"/>
+      <c r="H197" s="29"/>
+      <c r="I197" s="29"/>
+      <c r="J197" s="29"/>
+      <c r="K197" s="29"/>
+      <c r="L197" s="29"/>
+      <c r="M197" s="29"/>
+      <c r="N197" s="29"/>
+      <c r="O197" s="29"/>
+      <c r="P197" s="29"/>
+      <c r="Q197" s="29"/>
+      <c r="R197" s="29"/>
+      <c r="S197" s="29"/>
+      <c r="T197" s="29"/>
+      <c r="U197" s="29"/>
+      <c r="V197" s="29"/>
+      <c r="W197" s="29"/>
+      <c r="X197" s="29"/>
+      <c r="Y197" s="29"/>
+      <c r="Z197" s="29"/>
+      <c r="AA197" s="3"/>
       <c r="AB197" s="16"/>
       <c r="AC197" s="1"/>
       <c r="AD197" s="1"/>
       <c r="AE197" s="1"/>
     </row>
-    <row r="198" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:31" ht="9.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A198" s="1"/>
       <c r="B198" s="33" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C198" s="73">
-        <f>C$190</f>
-        <v>5</v>
-      </c>
-      <c r="D198" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
-      <c r="G198" s="4"/>
-      <c r="H198" s="5"/>
-      <c r="I198" s="5"/>
-      <c r="J198" s="5"/>
-      <c r="K198" s="5"/>
-      <c r="L198" s="5"/>
-      <c r="M198" s="5"/>
-      <c r="N198" s="5"/>
-      <c r="O198" s="5"/>
-      <c r="P198" s="5"/>
-      <c r="Q198" s="5"/>
-      <c r="R198" s="5"/>
-      <c r="S198" s="5"/>
-      <c r="T198" s="5"/>
-      <c r="U198" s="5"/>
-      <c r="V198" s="5"/>
-      <c r="W198" s="5"/>
-      <c r="X198" s="5"/>
-      <c r="Y198" s="5"/>
-      <c r="Z198" s="5"/>
-      <c r="AA198" s="4"/>
+        <f>INT($C$193)+2.01</f>
+        <v>3.01</v>
+      </c>
+      <c r="D198" s="3"/>
+      <c r="E198" s="3"/>
+      <c r="F198" s="3"/>
+      <c r="G198" s="3"/>
+      <c r="H198" s="29"/>
+      <c r="I198" s="29"/>
+      <c r="J198" s="29"/>
+      <c r="K198" s="29"/>
+      <c r="L198" s="29"/>
+      <c r="M198" s="29"/>
+      <c r="N198" s="29"/>
+      <c r="O198" s="29"/>
+      <c r="P198" s="29"/>
+      <c r="Q198" s="29"/>
+      <c r="R198" s="29"/>
+      <c r="S198" s="29"/>
+      <c r="T198" s="29"/>
+      <c r="U198" s="29"/>
+      <c r="V198" s="29"/>
+      <c r="W198" s="29"/>
+      <c r="X198" s="29"/>
+      <c r="Y198" s="29"/>
+      <c r="Z198" s="29"/>
+      <c r="AA198" s="3"/>
       <c r="AB198" s="16"/>
       <c r="AC198" s="1"/>
       <c r="AD198" s="1"/>
       <c r="AE198" s="1"/>
     </row>
-    <row r="199" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A199" s="1"/>
       <c r="B199" s="33"/>
       <c r="C199" s="73">
-        <f>INT($C$191)+2.005</f>
-        <v>3.0049999999999999</v>
-      </c>
-      <c r="D199" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E199" s="4"/>
-      <c r="F199" s="4"/>
+        <f>C$192</f>
+        <v>5</v>
+      </c>
+      <c r="D199" s="4"/>
+      <c r="E199" s="5"/>
+      <c r="F199" s="5"/>
       <c r="G199" s="4"/>
-      <c r="H199" s="58"/>
-      <c r="I199" s="58"/>
-      <c r="J199" s="58"/>
-      <c r="K199" s="58"/>
-      <c r="L199" s="58"/>
-      <c r="M199" s="58"/>
-      <c r="N199" s="58"/>
-      <c r="O199" s="58"/>
-      <c r="P199" s="58"/>
-      <c r="Q199" s="58"/>
-      <c r="R199" s="58"/>
-      <c r="S199" s="58"/>
-      <c r="T199" s="58"/>
-      <c r="U199" s="58"/>
-      <c r="V199" s="58"/>
-      <c r="W199" s="58"/>
-      <c r="X199" s="82"/>
-      <c r="Y199" s="82"/>
-      <c r="Z199" s="82"/>
+      <c r="H199" s="5"/>
+      <c r="I199" s="5"/>
+      <c r="J199" s="5"/>
+      <c r="K199" s="5"/>
+      <c r="L199" s="5"/>
+      <c r="M199" s="5"/>
+      <c r="N199" s="5"/>
+      <c r="O199" s="5"/>
+      <c r="P199" s="5"/>
+      <c r="Q199" s="5"/>
+      <c r="R199" s="5"/>
+      <c r="S199" s="5"/>
+      <c r="T199" s="5"/>
+      <c r="U199" s="5"/>
+      <c r="V199" s="5"/>
+      <c r="W199" s="5"/>
+      <c r="X199" s="5"/>
+      <c r="Y199" s="5"/>
+      <c r="Z199" s="5"/>
       <c r="AA199" s="4"/>
       <c r="AB199" s="16"/>
       <c r="AC199" s="1"/>
       <c r="AD199" s="1"/>
       <c r="AE199" s="1"/>
     </row>
-    <row r="200" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A200" s="1"/>
-      <c r="B200" s="33"/>
+      <c r="B200" s="33" t="s">
+        <v>19</v>
+      </c>
       <c r="C200" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D200" s="4"/>
+        <f>C$192</f>
+        <v>5</v>
+      </c>
+      <c r="D200" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
       <c r="G200" s="4"/>
-      <c r="H200" s="64" t="s">
-        <v>287</v>
-      </c>
-      <c r="I200" s="31">
-        <v>4</v>
-      </c>
-      <c r="J200" s="158" t="s">
-        <v>291</v>
-      </c>
-      <c r="K200" s="2"/>
-      <c r="L200" s="2"/>
-      <c r="M200" s="2"/>
-      <c r="N200" s="2"/>
-      <c r="O200" s="2"/>
-      <c r="P200" s="2"/>
-      <c r="Q200" s="2"/>
-      <c r="R200" s="2"/>
-      <c r="S200" s="2"/>
-      <c r="T200" s="2"/>
-      <c r="U200" s="2"/>
-      <c r="V200" s="2"/>
-      <c r="W200" s="2"/>
-      <c r="X200" s="2"/>
-      <c r="Y200" s="2"/>
-      <c r="Z200" s="2"/>
+      <c r="H200" s="5"/>
+      <c r="I200" s="5"/>
+      <c r="J200" s="5"/>
+      <c r="K200" s="5"/>
+      <c r="L200" s="5"/>
+      <c r="M200" s="5"/>
+      <c r="N200" s="5"/>
+      <c r="O200" s="5"/>
+      <c r="P200" s="5"/>
+      <c r="Q200" s="5"/>
+      <c r="R200" s="5"/>
+      <c r="S200" s="5"/>
+      <c r="T200" s="5"/>
+      <c r="U200" s="5"/>
+      <c r="V200" s="5"/>
+      <c r="W200" s="5"/>
+      <c r="X200" s="5"/>
+      <c r="Y200" s="5"/>
+      <c r="Z200" s="5"/>
       <c r="AA200" s="4"/>
       <c r="AB200" s="16"/>
       <c r="AC200" s="1"/>
       <c r="AD200" s="1"/>
       <c r="AE200" s="1"/>
     </row>
-    <row r="201" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A201" s="1"/>
       <c r="B201" s="33"/>
       <c r="C201" s="73">
-        <f>INT($C$191)+3</f>
-        <v>4</v>
-      </c>
-      <c r="D201" s="4"/>
-      <c r="E201" s="5"/>
-      <c r="F201" s="5"/>
+        <f>INT($C$193)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D201" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E201" s="4"/>
+      <c r="F201" s="4"/>
       <c r="G201" s="4"/>
-      <c r="H201" s="157"/>
-      <c r="I201" s="2"/>
-      <c r="J201" s="2"/>
-      <c r="K201" s="2"/>
-      <c r="L201" s="2"/>
-      <c r="M201" s="2"/>
-      <c r="N201" s="2"/>
-      <c r="O201" s="2"/>
-      <c r="P201" s="2"/>
-      <c r="Q201" s="2"/>
-      <c r="R201" s="2"/>
-      <c r="S201" s="2"/>
-      <c r="T201" s="2"/>
-      <c r="U201" s="2"/>
-      <c r="V201" s="2"/>
-      <c r="W201" s="2"/>
-      <c r="X201" s="2"/>
-      <c r="Y201" s="2"/>
-      <c r="Z201" s="2"/>
+      <c r="H201" s="58"/>
+      <c r="I201" s="58"/>
+      <c r="J201" s="58"/>
+      <c r="K201" s="58"/>
+      <c r="L201" s="58"/>
+      <c r="M201" s="58"/>
+      <c r="N201" s="58"/>
+      <c r="O201" s="58"/>
+      <c r="P201" s="58"/>
+      <c r="Q201" s="58"/>
+      <c r="R201" s="58"/>
+      <c r="S201" s="58"/>
+      <c r="T201" s="58"/>
+      <c r="U201" s="58"/>
+      <c r="V201" s="58"/>
+      <c r="W201" s="58"/>
+      <c r="X201" s="82"/>
+      <c r="Y201" s="82"/>
+      <c r="Z201" s="82"/>
       <c r="AA201" s="4"/>
       <c r="AB201" s="16"/>
       <c r="AC201" s="1"/>
       <c r="AD201" s="1"/>
       <c r="AE201" s="1"/>
     </row>
-    <row r="202" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A202" s="1"/>
       <c r="B202" s="33"/>
       <c r="C202" s="73">
-        <f>INT(C$191+3)</f>
-        <v>4</v>
+        <f>INT($C$193)+2</f>
+        <v>3</v>
       </c>
       <c r="D202" s="4"/>
       <c r="E202" s="5"/>
       <c r="F202" s="5"/>
       <c r="G202" s="4"/>
-      <c r="H202" s="148"/>
-      <c r="I202" s="148"/>
-      <c r="J202" s="148"/>
-      <c r="K202" s="148"/>
-      <c r="L202" s="148"/>
-      <c r="M202" s="148"/>
-      <c r="N202" s="148"/>
-      <c r="O202" s="148"/>
-      <c r="P202" s="148"/>
-      <c r="Q202" s="148"/>
-      <c r="R202" s="148"/>
+      <c r="H202" s="64" t="s">
+        <v>287</v>
+      </c>
+      <c r="I202" s="31">
+        <v>4</v>
+      </c>
+      <c r="J202" s="158" t="s">
+        <v>291</v>
+      </c>
+      <c r="K202" s="2"/>
+      <c r="L202" s="2"/>
+      <c r="M202" s="2"/>
+      <c r="N202" s="2"/>
+      <c r="O202" s="2"/>
+      <c r="P202" s="2"/>
+      <c r="Q202" s="2"/>
+      <c r="R202" s="2"/>
       <c r="S202" s="2"/>
       <c r="T202" s="2"/>
       <c r="U202" s="2"/>
@@ -35689,227 +35859,233 @@
       <c r="AD202" s="1"/>
       <c r="AE202" s="1"/>
     </row>
-    <row r="203" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
       <c r="B203" s="33"/>
       <c r="C203" s="73">
-        <f>INT($C$191)+3.005</f>
-        <v>4.0049999999999999</v>
+        <f>INT($C$193)+3</f>
+        <v>4</v>
       </c>
       <c r="D203" s="4"/>
-      <c r="E203" s="4"/>
-      <c r="F203" s="4"/>
+      <c r="E203" s="5"/>
+      <c r="F203" s="5"/>
       <c r="G203" s="4"/>
-      <c r="H203" s="4"/>
-      <c r="I203" s="4"/>
-      <c r="J203" s="4"/>
-      <c r="K203" s="4"/>
-      <c r="L203" s="4"/>
-      <c r="M203" s="4"/>
-      <c r="N203" s="4"/>
-      <c r="O203" s="4"/>
-      <c r="P203" s="4"/>
-      <c r="Q203" s="4"/>
-      <c r="R203" s="4"/>
-      <c r="S203" s="4"/>
-      <c r="T203" s="4"/>
-      <c r="U203" s="4"/>
-      <c r="V203" s="4"/>
-      <c r="W203" s="4"/>
-      <c r="X203" s="4"/>
-      <c r="Y203" s="4"/>
-      <c r="Z203" s="4"/>
-      <c r="AA203" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="H203" s="157"/>
+      <c r="I203" s="2"/>
+      <c r="J203" s="2"/>
+      <c r="K203" s="2"/>
+      <c r="L203" s="2"/>
+      <c r="M203" s="2"/>
+      <c r="N203" s="2"/>
+      <c r="O203" s="2"/>
+      <c r="P203" s="2"/>
+      <c r="Q203" s="2"/>
+      <c r="R203" s="2"/>
+      <c r="S203" s="2"/>
+      <c r="T203" s="2"/>
+      <c r="U203" s="2"/>
+      <c r="V203" s="2"/>
+      <c r="W203" s="2"/>
+      <c r="X203" s="2"/>
+      <c r="Y203" s="2"/>
+      <c r="Z203" s="2"/>
+      <c r="AA203" s="4"/>
       <c r="AB203" s="16"/>
       <c r="AC203" s="1"/>
       <c r="AD203" s="1"/>
       <c r="AE203" s="1"/>
     </row>
-    <row r="204" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A204" s="1"/>
       <c r="B204" s="33"/>
       <c r="C204" s="73">
-        <f>INT($C$191)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>INT(C$193+3)</f>
+        <v>4</v>
       </c>
       <c r="D204" s="4"/>
-      <c r="E204" s="4"/>
-      <c r="F204" s="4"/>
+      <c r="E204" s="5"/>
+      <c r="F204" s="5"/>
       <c r="G204" s="4"/>
-      <c r="H204" s="4"/>
-      <c r="I204" s="4"/>
-      <c r="J204" s="4"/>
-      <c r="K204" s="4"/>
-      <c r="L204" s="4"/>
-      <c r="M204" s="4"/>
-      <c r="N204" s="4"/>
-      <c r="O204" s="4"/>
-      <c r="P204" s="4"/>
-      <c r="Q204" s="4"/>
-      <c r="R204" s="4"/>
-      <c r="S204" s="4"/>
-      <c r="T204" s="4"/>
-      <c r="U204" s="4"/>
-      <c r="V204" s="4"/>
-      <c r="W204" s="4"/>
-      <c r="X204" s="4"/>
-      <c r="Y204" s="4"/>
-      <c r="Z204" s="4"/>
+      <c r="H204" s="148"/>
+      <c r="I204" s="148"/>
+      <c r="J204" s="148"/>
+      <c r="K204" s="148"/>
+      <c r="L204" s="148"/>
+      <c r="M204" s="148"/>
+      <c r="N204" s="148"/>
+      <c r="O204" s="148"/>
+      <c r="P204" s="148"/>
+      <c r="Q204" s="148"/>
+      <c r="R204" s="148"/>
+      <c r="S204" s="2"/>
+      <c r="T204" s="2"/>
+      <c r="U204" s="2"/>
+      <c r="V204" s="2"/>
+      <c r="W204" s="2"/>
+      <c r="X204" s="2"/>
+      <c r="Y204" s="2"/>
+      <c r="Z204" s="2"/>
       <c r="AA204" s="4"/>
       <c r="AB204" s="16"/>
       <c r="AC204" s="1"/>
       <c r="AD204" s="1"/>
       <c r="AE204" s="1"/>
     </row>
-    <row r="205" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
-      <c r="B205" s="35"/>
-      <c r="C205" s="76">
-        <f>INT($C$191)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D205" s="17"/>
-      <c r="E205" s="17"/>
-      <c r="F205" s="17"/>
-      <c r="G205" s="17"/>
-      <c r="H205" s="17"/>
-      <c r="I205" s="17"/>
-      <c r="J205" s="17"/>
-      <c r="K205" s="17"/>
-      <c r="L205" s="17"/>
-      <c r="M205" s="17"/>
-      <c r="N205" s="17"/>
-      <c r="O205" s="17"/>
-      <c r="P205" s="17"/>
-      <c r="Q205" s="17"/>
-      <c r="R205" s="17"/>
-      <c r="S205" s="17"/>
-      <c r="T205" s="17"/>
-      <c r="U205" s="17"/>
-      <c r="V205" s="17"/>
-      <c r="W205" s="17"/>
-      <c r="X205" s="17"/>
-      <c r="Y205" s="17"/>
-      <c r="Z205" s="17"/>
-      <c r="AA205" s="17"/>
-      <c r="AB205" s="18" t="s">
-        <v>1</v>
-      </c>
+      <c r="B205" s="33"/>
+      <c r="C205" s="73">
+        <f>INT($C$193)+3.005</f>
+        <v>4.0049999999999999</v>
+      </c>
+      <c r="D205" s="4"/>
+      <c r="E205" s="4"/>
+      <c r="F205" s="4"/>
+      <c r="G205" s="4"/>
+      <c r="H205" s="4"/>
+      <c r="I205" s="4"/>
+      <c r="J205" s="4"/>
+      <c r="K205" s="4"/>
+      <c r="L205" s="4"/>
+      <c r="M205" s="4"/>
+      <c r="N205" s="4"/>
+      <c r="O205" s="4"/>
+      <c r="P205" s="4"/>
+      <c r="Q205" s="4"/>
+      <c r="R205" s="4"/>
+      <c r="S205" s="4"/>
+      <c r="T205" s="4"/>
+      <c r="U205" s="4"/>
+      <c r="V205" s="4"/>
+      <c r="W205" s="4"/>
+      <c r="X205" s="4"/>
+      <c r="Y205" s="4"/>
+      <c r="Z205" s="4"/>
+      <c r="AA205" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB205" s="16"/>
       <c r="AC205" s="1"/>
       <c r="AD205" s="1"/>
       <c r="AE205" s="1"/>
     </row>
-    <row r="206" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A206" s="1"/>
-      <c r="B206" s="19"/>
-      <c r="C206" s="77">
-        <f>INT($C$191)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D206" s="19"/>
-      <c r="E206" s="19"/>
-      <c r="F206" s="19"/>
-      <c r="G206" s="19"/>
-      <c r="H206" s="19"/>
-      <c r="I206" s="19"/>
-      <c r="J206" s="19"/>
-      <c r="K206" s="19"/>
-      <c r="L206" s="19"/>
-      <c r="M206" s="19"/>
-      <c r="N206" s="19"/>
-      <c r="O206" s="19"/>
-      <c r="P206" s="19"/>
-      <c r="Q206" s="19"/>
-      <c r="R206" s="19"/>
-      <c r="S206" s="19"/>
-      <c r="T206" s="19"/>
-      <c r="U206" s="19"/>
-      <c r="V206" s="19"/>
-      <c r="W206" s="19"/>
-      <c r="X206" s="19"/>
-      <c r="Y206" s="19"/>
-      <c r="Z206" s="19"/>
-      <c r="AA206" s="19"/>
-      <c r="AB206" s="19"/>
+      <c r="B206" s="33"/>
+      <c r="C206" s="73">
+        <f>INT($C$193)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D206" s="4"/>
+      <c r="E206" s="4"/>
+      <c r="F206" s="4"/>
+      <c r="G206" s="4"/>
+      <c r="H206" s="4"/>
+      <c r="I206" s="4"/>
+      <c r="J206" s="4"/>
+      <c r="K206" s="4"/>
+      <c r="L206" s="4"/>
+      <c r="M206" s="4"/>
+      <c r="N206" s="4"/>
+      <c r="O206" s="4"/>
+      <c r="P206" s="4"/>
+      <c r="Q206" s="4"/>
+      <c r="R206" s="4"/>
+      <c r="S206" s="4"/>
+      <c r="T206" s="4"/>
+      <c r="U206" s="4"/>
+      <c r="V206" s="4"/>
+      <c r="W206" s="4"/>
+      <c r="X206" s="4"/>
+      <c r="Y206" s="4"/>
+      <c r="Z206" s="4"/>
+      <c r="AA206" s="4"/>
+      <c r="AB206" s="16"/>
       <c r="AC206" s="1"/>
       <c r="AD206" s="1"/>
       <c r="AE206" s="1"/>
     </row>
-    <row r="207" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1"/>
-      <c r="B207" s="1"/>
-      <c r="C207" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D207" s="1"/>
-      <c r="E207" s="1"/>
-      <c r="F207" s="1"/>
-      <c r="G207" s="1"/>
-      <c r="H207" s="1"/>
-      <c r="I207" s="1"/>
-      <c r="J207" s="1"/>
-      <c r="K207" s="1"/>
-      <c r="L207" s="1"/>
-      <c r="M207" s="1"/>
-      <c r="N207" s="1"/>
-      <c r="O207" s="1"/>
-      <c r="P207" s="1"/>
-      <c r="Q207" s="1"/>
-      <c r="R207" s="1"/>
-      <c r="S207" s="1"/>
-      <c r="T207" s="1"/>
-      <c r="U207" s="1"/>
-      <c r="V207" s="1"/>
-      <c r="W207" s="1"/>
-      <c r="X207" s="1"/>
-      <c r="Y207" s="1"/>
-      <c r="Z207" s="1"/>
-      <c r="AA207" s="1"/>
-      <c r="AB207" s="1"/>
+      <c r="B207" s="35"/>
+      <c r="C207" s="76">
+        <f>INT($C$193)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D207" s="17"/>
+      <c r="E207" s="17"/>
+      <c r="F207" s="17"/>
+      <c r="G207" s="17"/>
+      <c r="H207" s="17"/>
+      <c r="I207" s="17"/>
+      <c r="J207" s="17"/>
+      <c r="K207" s="17"/>
+      <c r="L207" s="17"/>
+      <c r="M207" s="17"/>
+      <c r="N207" s="17"/>
+      <c r="O207" s="17"/>
+      <c r="P207" s="17"/>
+      <c r="Q207" s="17"/>
+      <c r="R207" s="17"/>
+      <c r="S207" s="17"/>
+      <c r="T207" s="17"/>
+      <c r="U207" s="17"/>
+      <c r="V207" s="17"/>
+      <c r="W207" s="17"/>
+      <c r="X207" s="17"/>
+      <c r="Y207" s="17"/>
+      <c r="Z207" s="17"/>
+      <c r="AA207" s="17"/>
+      <c r="AB207" s="18" t="s">
+        <v>1</v>
+      </c>
       <c r="AC207" s="1"/>
       <c r="AD207" s="1"/>
       <c r="AE207" s="1"/>
     </row>
-    <row r="208" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1"/>
-      <c r="B208" s="1"/>
-      <c r="C208" s="66"/>
-      <c r="D208" s="1"/>
-      <c r="E208" s="1"/>
-      <c r="F208" s="1"/>
-      <c r="G208" s="1"/>
-      <c r="H208" s="1"/>
-      <c r="I208" s="1"/>
-      <c r="J208" s="1"/>
-      <c r="K208" s="1"/>
-      <c r="L208" s="1"/>
-      <c r="M208" s="1"/>
-      <c r="N208" s="1"/>
-      <c r="O208" s="1"/>
-      <c r="P208" s="1"/>
-      <c r="Q208" s="1"/>
-      <c r="R208" s="1"/>
-      <c r="S208" s="1"/>
-      <c r="T208" s="1"/>
-      <c r="U208" s="1"/>
-      <c r="V208" s="1"/>
-      <c r="W208" s="1"/>
-      <c r="X208" s="1"/>
-      <c r="Y208" s="1"/>
-      <c r="Z208" s="1"/>
-      <c r="AA208" s="1"/>
-      <c r="AB208" s="1"/>
+      <c r="B208" s="19"/>
+      <c r="C208" s="77">
+        <f>INT($C$193)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D208" s="19"/>
+      <c r="E208" s="19"/>
+      <c r="F208" s="19"/>
+      <c r="G208" s="19"/>
+      <c r="H208" s="19"/>
+      <c r="I208" s="19"/>
+      <c r="J208" s="19"/>
+      <c r="K208" s="19"/>
+      <c r="L208" s="19"/>
+      <c r="M208" s="19"/>
+      <c r="N208" s="19"/>
+      <c r="O208" s="19"/>
+      <c r="P208" s="19"/>
+      <c r="Q208" s="19"/>
+      <c r="R208" s="19"/>
+      <c r="S208" s="19"/>
+      <c r="T208" s="19"/>
+      <c r="U208" s="19"/>
+      <c r="V208" s="19"/>
+      <c r="W208" s="19"/>
+      <c r="X208" s="19"/>
+      <c r="Y208" s="19"/>
+      <c r="Z208" s="19"/>
+      <c r="AA208" s="19"/>
+      <c r="AB208" s="19"/>
       <c r="AC208" s="1"/>
       <c r="AD208" s="1"/>
       <c r="AE208" s="1"/>
     </row>
-    <row r="209" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
-      <c r="C209" s="66"/>
+      <c r="C209" s="73">
+        <f>INT($C$193)+2</f>
+        <v>3</v>
+      </c>
       <c r="D209" s="1"/>
       <c r="E209" s="1"/>
       <c r="F209" s="1"/>
@@ -36072,7 +36248,73 @@
       <c r="AE213" s="1"/>
     </row>
     <row r="214" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="C214" s="72" t="s">
+      <c r="A214" s="1"/>
+      <c r="B214" s="1"/>
+      <c r="C214" s="66"/>
+      <c r="D214" s="1"/>
+      <c r="E214" s="1"/>
+      <c r="F214" s="1"/>
+      <c r="G214" s="1"/>
+      <c r="H214" s="1"/>
+      <c r="I214" s="1"/>
+      <c r="J214" s="1"/>
+      <c r="K214" s="1"/>
+      <c r="L214" s="1"/>
+      <c r="M214" s="1"/>
+      <c r="N214" s="1"/>
+      <c r="O214" s="1"/>
+      <c r="P214" s="1"/>
+      <c r="Q214" s="1"/>
+      <c r="R214" s="1"/>
+      <c r="S214" s="1"/>
+      <c r="T214" s="1"/>
+      <c r="U214" s="1"/>
+      <c r="V214" s="1"/>
+      <c r="W214" s="1"/>
+      <c r="X214" s="1"/>
+      <c r="Y214" s="1"/>
+      <c r="Z214" s="1"/>
+      <c r="AA214" s="1"/>
+      <c r="AB214" s="1"/>
+      <c r="AC214" s="1"/>
+      <c r="AD214" s="1"/>
+      <c r="AE214" s="1"/>
+    </row>
+    <row r="215" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A215" s="1"/>
+      <c r="B215" s="1"/>
+      <c r="C215" s="66"/>
+      <c r="D215" s="1"/>
+      <c r="E215" s="1"/>
+      <c r="F215" s="1"/>
+      <c r="G215" s="1"/>
+      <c r="H215" s="1"/>
+      <c r="I215" s="1"/>
+      <c r="J215" s="1"/>
+      <c r="K215" s="1"/>
+      <c r="L215" s="1"/>
+      <c r="M215" s="1"/>
+      <c r="N215" s="1"/>
+      <c r="O215" s="1"/>
+      <c r="P215" s="1"/>
+      <c r="Q215" s="1"/>
+      <c r="R215" s="1"/>
+      <c r="S215" s="1"/>
+      <c r="T215" s="1"/>
+      <c r="U215" s="1"/>
+      <c r="V215" s="1"/>
+      <c r="W215" s="1"/>
+      <c r="X215" s="1"/>
+      <c r="Y215" s="1"/>
+      <c r="Z215" s="1"/>
+      <c r="AA215" s="1"/>
+      <c r="AB215" s="1"/>
+      <c r="AC215" s="1"/>
+      <c r="AD215" s="1"/>
+      <c r="AE215" s="1"/>
+    </row>
+    <row r="216" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="C216" s="72" t="s">
         <v>4</v>
       </c>
     </row>
@@ -36296,7 +36538,7 @@
       <c r="E7" s="176"/>
       <c r="F7" s="172"/>
       <c r="G7" s="178" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="H7" s="172"/>
       <c r="I7" s="172"/>
@@ -37745,23 +37987,23 @@
       <c r="I18" s="31">
         <v>1</v>
       </c>
-      <c r="J18" s="226" t="s">
+      <c r="J18" s="229" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="226"/>
-      <c r="L18" s="226"/>
-      <c r="M18" s="226"/>
-      <c r="N18" s="226"/>
-      <c r="O18" s="226"/>
-      <c r="P18" s="226"/>
-      <c r="Q18" s="226"/>
-      <c r="R18" s="226"/>
-      <c r="S18" s="226"/>
-      <c r="T18" s="226"/>
-      <c r="U18" s="226"/>
-      <c r="V18" s="226"/>
-      <c r="W18" s="226"/>
-      <c r="X18" s="226"/>
+      <c r="K18" s="229"/>
+      <c r="L18" s="229"/>
+      <c r="M18" s="229"/>
+      <c r="N18" s="229"/>
+      <c r="O18" s="229"/>
+      <c r="P18" s="229"/>
+      <c r="Q18" s="229"/>
+      <c r="R18" s="229"/>
+      <c r="S18" s="229"/>
+      <c r="T18" s="229"/>
+      <c r="U18" s="229"/>
+      <c r="V18" s="229"/>
+      <c r="W18" s="229"/>
+      <c r="X18" s="229"/>
       <c r="Y18" s="2"/>
       <c r="Z18" s="4"/>
       <c r="AA18" s="16"/>
@@ -37856,23 +38098,23 @@
       <c r="I21" s="23">
         <v>1</v>
       </c>
-      <c r="J21" s="224" t="s">
+      <c r="J21" s="227" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="225"/>
-      <c r="L21" s="225"/>
-      <c r="M21" s="225"/>
-      <c r="N21" s="225"/>
-      <c r="O21" s="225"/>
-      <c r="P21" s="225"/>
-      <c r="Q21" s="225"/>
-      <c r="R21" s="225"/>
-      <c r="S21" s="225"/>
-      <c r="T21" s="225"/>
-      <c r="U21" s="225"/>
-      <c r="V21" s="225"/>
-      <c r="W21" s="225"/>
-      <c r="X21" s="227"/>
+      <c r="K21" s="228"/>
+      <c r="L21" s="228"/>
+      <c r="M21" s="228"/>
+      <c r="N21" s="228"/>
+      <c r="O21" s="228"/>
+      <c r="P21" s="228"/>
+      <c r="Q21" s="228"/>
+      <c r="R21" s="228"/>
+      <c r="S21" s="228"/>
+      <c r="T21" s="228"/>
+      <c r="U21" s="228"/>
+      <c r="V21" s="228"/>
+      <c r="W21" s="228"/>
+      <c r="X21" s="230"/>
       <c r="Y21" s="2"/>
       <c r="Z21" s="4"/>
       <c r="AA21" s="16"/>

</xml_diff>

<commit_message>
GEPEP to Dev: Structural.xlsx, change rangename for age stages for REVs to i_rev_age_stage_afo to differentiate from the asbv age stages. Add rangename for geneticist age stages (i_rev_age_stage_asbv) for use by p11 saa. Note: the p11 saa shows full expression between 1/4 and 3/4 of the age stage and expression ramps up and down on either side.
</commit_message>
<xml_diff>
--- a/ExcelInputs/Structural.xlsx
+++ b/ExcelInputs/Structural.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Models\AFO\ExcelInputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127C0B2D-B85A-4E4F-98F9-BA86FE1B5B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AA76A62-DC41-4944-96A6-32EDCF7AC316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="240" windowWidth="25950" windowHeight="15555" tabRatio="678" activeTab="1" xr2:uid="{0842FB8C-088A-42F9-B075-24D0619777A0}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="678" activeTab="2" xr2:uid="{0842FB8C-088A-42F9-B075-24D0619777A0}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="24" r:id="rId1"/>
@@ -92,7 +92,7 @@
     <definedName name="i_lag_organs">Stock!$I$70</definedName>
     <definedName name="i_lag_wool">Stock!$I$69</definedName>
     <definedName name="i_landuse_is_dual" localSheetId="0">General!$Q$79:$Q$110</definedName>
-    <definedName name="i_len_f">StructuralSA!$I$200</definedName>
+    <definedName name="i_len_f">StructuralSA!$I$202</definedName>
     <definedName name="i_len_l">Stock!$M$159</definedName>
     <definedName name="i_len_m">Stock!$L$159</definedName>
     <definedName name="i_len_planning_horizon" localSheetId="2">StructuralSA!$M$46</definedName>
@@ -129,10 +129,11 @@
     <definedName name="i_prejoin_offset">Stock!$I$66</definedName>
     <definedName name="i_progeny_w2_len">StructuralSA!$Q$107</definedName>
     <definedName name="i_r2adjust_inc">StructuralSA!$U$148</definedName>
-    <definedName name="i_rev_age_stage" localSheetId="2">StructuralSA!$N$159:$Z$160</definedName>
+    <definedName name="i_rev_age_stage_afo" localSheetId="2">StructuralSA!$N$161:$Z$162</definedName>
+    <definedName name="i_rev_age_stage_asbv">StructuralSA!$N$160:$Z$160</definedName>
     <definedName name="i_rev_number" localSheetId="2">StructuralSA!$I$150</definedName>
-    <definedName name="i_rev_trait_name" localSheetId="2">StructuralSA!$H$162:$H$181</definedName>
-    <definedName name="i_rev_trait_scenario" localSheetId="2">StructuralSA!$I$162:$I$181</definedName>
+    <definedName name="i_rev_trait_name" localSheetId="2">StructuralSA!$H$164:$H$183</definedName>
+    <definedName name="i_rev_trait_scenario" localSheetId="2">StructuralSA!$I$164:$I$183</definedName>
     <definedName name="i_rev_update" localSheetId="2">StructuralSA!$I$148</definedName>
     <definedName name="i_sim_periods_year">Stock!$I$62</definedName>
     <definedName name="i_store_cs_rep" localSheetId="3">'Report Settings'!$K$18</definedName>
@@ -181,7 +182,7 @@
     <definedName name="ZA.WidthCol" localSheetId="4">Admin!$L$26</definedName>
     <definedName name="ZA.ZoomSheet" localSheetId="4">Admin!$O$26</definedName>
   </definedNames>
-  <calcPr calcId="191029" refMode="R1C1" iterate="1"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2213,7 +2214,79 @@
         </r>
       </text>
     </comment>
-    <comment ref="H161" authorId="1" shapeId="0" xr:uid="{FD0151C6-9F6F-4723-995E-804A9122F39A}">
+    <comment ref="N159" authorId="2" shapeId="0" xr:uid="{D52B6350-79DA-43ED-9DD3-35AB8C8E2C20}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>John:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+When using geneticist age stages adult and whole of life are allocated to the individual age stages. So age is not used.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y159" authorId="2" shapeId="0" xr:uid="{006B6E62-3675-41C9-9A10-C71798B4F55A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>John:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+When using geneticist age stages adult and whole of life are allocated to the individual age stages. So age is not used.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N160" authorId="2" shapeId="0" xr:uid="{E3693196-A31F-4656-BCF8-B8AE6FB68901}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>John:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Although not used this value needs to be 0 so that the np.roll works correctly</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H163" authorId="1" shapeId="0" xr:uid="{FD0151C6-9F6F-4723-995E-804A9122F39A}">
       <text>
         <r>
           <rPr>
@@ -2239,7 +2312,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I161" authorId="2" shapeId="0" xr:uid="{533029ED-41A1-487B-BDF7-AC2146E10D21}">
+    <comment ref="I163" authorId="2" shapeId="0" xr:uid="{533029ED-41A1-487B-BDF7-AC2146E10D21}">
       <text>
         <r>
           <rPr>
@@ -2264,7 +2337,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H165" authorId="2" shapeId="0" xr:uid="{A12E8373-CBF7-4301-8BBE-54FB2CD3F999}">
+    <comment ref="H167" authorId="2" shapeId="0" xr:uid="{A12E8373-CBF7-4301-8BBE-54FB2CD3F999}">
       <text>
         <r>
           <rPr>
@@ -2288,7 +2361,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H166" authorId="2" shapeId="0" xr:uid="{ADD99B78-258B-4112-BEFE-ACD7C132C257}">
+    <comment ref="H168" authorId="2" shapeId="0" xr:uid="{ADD99B78-258B-4112-BEFE-ACD7C132C257}">
       <text>
         <r>
           <rPr>
@@ -2312,7 +2385,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H167" authorId="2" shapeId="0" xr:uid="{F4A4ECC6-7846-4162-9607-F6E572F33EDF}">
+    <comment ref="H169" authorId="2" shapeId="0" xr:uid="{F4A4ECC6-7846-4162-9607-F6E572F33EDF}">
       <text>
         <r>
           <rPr>
@@ -2336,7 +2409,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H168" authorId="2" shapeId="0" xr:uid="{4C2B1933-42FC-4263-B576-C6A05675CBF9}">
+    <comment ref="H170" authorId="2" shapeId="0" xr:uid="{4C2B1933-42FC-4263-B576-C6A05675CBF9}">
       <text>
         <r>
           <rPr>
@@ -2360,7 +2433,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H174" authorId="1" shapeId="0" xr:uid="{658A1575-7B6D-49A0-9205-9DD14E053E41}">
+    <comment ref="H176" authorId="1" shapeId="0" xr:uid="{658A1575-7B6D-49A0-9205-9DD14E053E41}">
       <text>
         <r>
           <rPr>
@@ -2384,7 +2457,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H179" authorId="2" shapeId="0" xr:uid="{7D72CFA0-EF47-40D9-9D6F-9FDC3F1C19F9}">
+    <comment ref="H181" authorId="2" shapeId="0" xr:uid="{7D72CFA0-EF47-40D9-9D6F-9FDC3F1C19F9}">
       <text>
         <r>
           <rPr>
@@ -2408,7 +2481,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H200" authorId="2" shapeId="0" xr:uid="{B39EFDC6-7ABB-4808-93B1-2819F2755236}">
+    <comment ref="H202" authorId="2" shapeId="0" xr:uid="{B39EFDC6-7ABB-4808-93B1-2819F2755236}">
       <text>
         <r>
           <rPr>
@@ -2471,7 +2544,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="450">
   <si>
     <t>Controls for this worksheet</t>
   </si>
@@ -3813,9 +3886,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Available trait timing (for information only)</t>
-  </si>
-  <si>
     <t>Geneticist definition (age)</t>
   </si>
   <si>
@@ -3887,7 +3957,52 @@
     <t>rr</t>
   </si>
   <si>
-    <t>31Jan26: Removed the Cutoff levels for the NV pools that have been moved to Property.xlsx
+    <t>Some arrays used for reporting are very big so the default is not to store them. This is the default settings which can be overwritten using sensitivity values</t>
+  </si>
+  <si>
+    <t>22Feb26: Change the value of Prejoining intial repro proportion to 100% in the 11 slice (was 100% in NM)
+20Jul22: Change i_chill_adj_b1 so that chill of the singles is increased (had been no change)
+19Jan22: Fix error in i_mask_g1g3 that included True for [BMT,BM]
+2Dec21 remove min numbers b1. it wasnt doing anything in the code.
+8Jun21: Change definition of the 'k2 input cluster' to include NM so these animals can be differentially fed.
+                 Add comments about difference between 'k2 input cluster' and 'k2 post processing cluster'
+                 Added comment about including the axis length inputs in the first table
+16May21: Remove heading user defined date
+14Apr21: MRY changes for EV pools and confinement (removed about confinement patterns being included)
+12Apr21: Change back to 3N for analysis
+                  1N for LW profile comparisons
+10Apr21: Altered k2 cluster for scan 0 to allocate all ewes to the 11 slice
+                   Changed inputs for GBAL because it can't be represented in the matrix
+4Apr21: Change to 3FVP with 3N
+2Apr21: Change to 3N for dams &amp; 5FVP
+31Mar21: Change the index for the k2 cluster (for the seasonality model)
+29Mar21: Changed to FVP3, 1N for dams, 3N for Offs
+22Mar21: Alter the initial weight &amp; wool spread for the weaners
+1: 1Apr19-Blank worksheet</t>
+  </si>
+  <si>
+    <t>22Feb26: Delete 'Prejoining initial repro propn' from Associatons table
+                   Change the order of the axes postion inputs so that they are in axis order rather than alphabetical order
+3May23: Convert chill adjustment scalars for GBAL slices to a formula (still needs work on the 11, 22 &amp; 33 slices)
+17Jun22: Add a chill adjustment scalar with a b1 axis (to scale Property.xlsx!i_chill_adj)
+11Jul21: dvp/fvp updates 
+27Apr21: Split fvp inputs
+25Apr21: Deleted range names i_w1_len &amp; w3
+9Apr21: Fix formatting (box) around k2 cluster definition.
+30Mar21: Added inputs for % dry and number dams mated
+2: 17Jul20-Added structural inputs table
+1: 1Apr19-Created the version control table</t>
+  </si>
+  <si>
+    <t>Available trait timing (REV trait / Model inversion) - for information only</t>
+  </si>
+  <si>
+    <t>Still to connect the FYI on model inversion traits</t>
+  </si>
+  <si>
+    <t>3May26: Change geneticist age stage named range to only include end and renamed to i_rev_age_stage_asbv
+17Apr29: Added details for geneticist age stage to calculate the midpoint. Converted adults to a 364 day year step
+31Jan26: Removed the Cutoff levels for the NV pools that have been moved to Property.xlsx
 9Dec25: Added sl &amp; rr as REV traits. Expanded era and rr to be available at all individual adult age stages not just overall.
 26Sep24: Add cfat (carcase fat depth) trait
 6Sep24: Alter order of age stages so that whole of life is [0] - which is the default in the code.
@@ -3919,43 +4034,6 @@
                    Moved FVP &amp; N inputs from Stock
 1: 1Apr19-Created the version control table</t>
   </si>
-  <si>
-    <t>Some arrays used for reporting are very big so the default is not to store them. This is the default settings which can be overwritten using sensitivity values</t>
-  </si>
-  <si>
-    <t>22Feb26: Change the value of Prejoining intial repro proportion to 100% in the 11 slice (was 100% in NM)
-20Jul22: Change i_chill_adj_b1 so that chill of the singles is increased (had been no change)
-19Jan22: Fix error in i_mask_g1g3 that included True for [BMT,BM]
-2Dec21 remove min numbers b1. it wasnt doing anything in the code.
-8Jun21: Change definition of the 'k2 input cluster' to include NM so these animals can be differentially fed.
-                 Add comments about difference between 'k2 input cluster' and 'k2 post processing cluster'
-                 Added comment about including the axis length inputs in the first table
-16May21: Remove heading user defined date
-14Apr21: MRY changes for EV pools and confinement (removed about confinement patterns being included)
-12Apr21: Change back to 3N for analysis
-                  1N for LW profile comparisons
-10Apr21: Altered k2 cluster for scan 0 to allocate all ewes to the 11 slice
-                   Changed inputs for GBAL because it can't be represented in the matrix
-4Apr21: Change to 3FVP with 3N
-2Apr21: Change to 3N for dams &amp; 5FVP
-31Mar21: Change the index for the k2 cluster (for the seasonality model)
-29Mar21: Changed to FVP3, 1N for dams, 3N for Offs
-22Mar21: Alter the initial weight &amp; wool spread for the weaners
-1: 1Apr19-Blank worksheet</t>
-  </si>
-  <si>
-    <t>22Feb26: Delete 'Prejoining initial repro propn' from Associatons table
-                   Change the order of the axes postion inputs so that they are in axis order rather than alphabetical order
-3May23: Convert chill adjustment scalars for GBAL slices to a formula (still needs work on the 11, 22 &amp; 33 slices)
-17Jun22: Add a chill adjustment scalar with a b1 axis (to scale Property.xlsx!i_chill_adj)
-11Jul21: dvp/fvp updates 
-27Apr21: Split fvp inputs
-25Apr21: Deleted range names i_w1_len &amp; w3
-9Apr21: Fix formatting (box) around k2 cluster definition.
-30Mar21: Added inputs for % dry and number dams mated
-2: 17Jul20-Added structural inputs table
-1: 1Apr19-Created the version control table</t>
-  </si>
 </sst>
 </file>
 
@@ -3967,7 +4045,7 @@
     <numFmt numFmtId="166" formatCode="0.00_)"/>
     <numFmt numFmtId="167" formatCode="[$-C09]dd\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4186,6 +4264,25 @@
       <color rgb="FF0000CC"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="40">
@@ -5370,7 +5467,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="228">
+  <cellXfs count="231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="25" xfId="3">
@@ -5959,6 +6056,15 @@
     <xf numFmtId="1" fontId="32" fillId="39" borderId="22" xfId="44" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="50" xfId="13" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="24" xfId="16" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="38" xfId="12" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -7125,19 +7231,19 @@
       <c r="I13" s="126">
         <v>44371.659649305599</v>
       </c>
-      <c r="J13" s="221" t="s">
+      <c r="J13" s="224" t="s">
         <v>293</v>
       </c>
-      <c r="K13" s="222"/>
-      <c r="L13" s="222"/>
-      <c r="M13" s="222"/>
-      <c r="N13" s="222"/>
-      <c r="O13" s="222"/>
-      <c r="P13" s="222"/>
-      <c r="Q13" s="222"/>
-      <c r="R13" s="222"/>
-      <c r="S13" s="222"/>
-      <c r="T13" s="223"/>
+      <c r="K13" s="225"/>
+      <c r="L13" s="225"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="225"/>
+      <c r="O13" s="225"/>
+      <c r="P13" s="225"/>
+      <c r="Q13" s="225"/>
+      <c r="R13" s="225"/>
+      <c r="S13" s="225"/>
+      <c r="T13" s="226"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
@@ -7164,19 +7270,19 @@
       <c r="I14" s="125">
         <v>44719.411846643503</v>
       </c>
-      <c r="J14" s="224" t="s">
+      <c r="J14" s="227" t="s">
         <v>352</v>
       </c>
-      <c r="K14" s="225"/>
-      <c r="L14" s="225"/>
-      <c r="M14" s="225"/>
-      <c r="N14" s="225"/>
-      <c r="O14" s="225"/>
-      <c r="P14" s="225"/>
-      <c r="Q14" s="225"/>
-      <c r="R14" s="225"/>
-      <c r="S14" s="225"/>
-      <c r="T14" s="225"/>
+      <c r="K14" s="228"/>
+      <c r="L14" s="228"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="228"/>
+      <c r="O14" s="228"/>
+      <c r="P14" s="228"/>
+      <c r="Q14" s="228"/>
+      <c r="R14" s="228"/>
+      <c r="S14" s="228"/>
+      <c r="T14" s="228"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -9793,7 +9899,7 @@
       <c r="G86" s="4"/>
       <c r="H86" s="148"/>
       <c r="I86" s="162" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="J86" s="162" t="b">
         <v>0</v>
@@ -9978,13 +10084,13 @@
       <c r="N90" s="164"/>
       <c r="O90" s="164"/>
       <c r="P90" s="162" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q90" s="162" t="b">
         <v>0</v>
       </c>
       <c r="R90" s="206" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
@@ -11813,19 +11919,19 @@
       <c r="I13" s="126">
         <v>46075.691937152798</v>
       </c>
-      <c r="J13" s="221" t="s">
-        <v>448</v>
-      </c>
-      <c r="K13" s="222"/>
-      <c r="L13" s="222"/>
-      <c r="M13" s="222"/>
-      <c r="N13" s="222"/>
-      <c r="O13" s="222"/>
-      <c r="P13" s="222"/>
-      <c r="Q13" s="222"/>
-      <c r="R13" s="222"/>
-      <c r="S13" s="222"/>
-      <c r="T13" s="223"/>
+      <c r="J13" s="224" t="s">
+        <v>446</v>
+      </c>
+      <c r="K13" s="225"/>
+      <c r="L13" s="225"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="225"/>
+      <c r="O13" s="225"/>
+      <c r="P13" s="225"/>
+      <c r="Q13" s="225"/>
+      <c r="R13" s="225"/>
+      <c r="S13" s="225"/>
+      <c r="T13" s="226"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
@@ -11852,19 +11958,19 @@
       <c r="I14" s="125">
         <v>46075.710698379597</v>
       </c>
-      <c r="J14" s="224" t="s">
-        <v>447</v>
-      </c>
-      <c r="K14" s="225"/>
-      <c r="L14" s="225"/>
-      <c r="M14" s="225"/>
-      <c r="N14" s="225"/>
-      <c r="O14" s="225"/>
-      <c r="P14" s="225"/>
-      <c r="Q14" s="225"/>
-      <c r="R14" s="225"/>
-      <c r="S14" s="225"/>
-      <c r="T14" s="225"/>
+      <c r="J14" s="227" t="s">
+        <v>445</v>
+      </c>
+      <c r="K14" s="228"/>
+      <c r="L14" s="228"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="228"/>
+      <c r="O14" s="228"/>
+      <c r="P14" s="228"/>
+      <c r="Q14" s="228"/>
+      <c r="R14" s="228"/>
+      <c r="S14" s="228"/>
+      <c r="T14" s="228"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -27026,7 +27132,7 @@
   <sheetPr codeName="Sheet3">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AE214"/>
+  <dimension ref="A1:AE216"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -27555,21 +27661,21 @@
         <v>16</v>
       </c>
       <c r="I13" s="126">
-        <v>46053.6384755787</v>
-      </c>
-      <c r="J13" s="221" t="s">
-        <v>445</v>
-      </c>
-      <c r="K13" s="222"/>
-      <c r="L13" s="222"/>
-      <c r="M13" s="222"/>
-      <c r="N13" s="222"/>
-      <c r="O13" s="222"/>
-      <c r="P13" s="222"/>
-      <c r="Q13" s="222"/>
-      <c r="R13" s="222"/>
-      <c r="S13" s="222"/>
-      <c r="T13" s="223"/>
+        <v>46145.506140277801</v>
+      </c>
+      <c r="J13" s="224" t="s">
+        <v>449</v>
+      </c>
+      <c r="K13" s="225"/>
+      <c r="L13" s="225"/>
+      <c r="M13" s="225"/>
+      <c r="N13" s="225"/>
+      <c r="O13" s="225"/>
+      <c r="P13" s="225"/>
+      <c r="Q13" s="225"/>
+      <c r="R13" s="225"/>
+      <c r="S13" s="225"/>
+      <c r="T13" s="226"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
@@ -27599,19 +27705,19 @@
       <c r="I14" s="125">
         <v>45593.407781134301</v>
       </c>
-      <c r="J14" s="224" t="s">
-        <v>441</v>
-      </c>
-      <c r="K14" s="225"/>
-      <c r="L14" s="225"/>
-      <c r="M14" s="225"/>
-      <c r="N14" s="225"/>
-      <c r="O14" s="225"/>
-      <c r="P14" s="225"/>
-      <c r="Q14" s="225"/>
-      <c r="R14" s="225"/>
-      <c r="S14" s="225"/>
-      <c r="T14" s="225"/>
+      <c r="J14" s="227" t="s">
+        <v>440</v>
+      </c>
+      <c r="K14" s="228"/>
+      <c r="L14" s="228"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="228"/>
+      <c r="O14" s="228"/>
+      <c r="P14" s="228"/>
+      <c r="Q14" s="228"/>
+      <c r="R14" s="228"/>
+      <c r="S14" s="228"/>
+      <c r="T14" s="228"/>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -28846,7 +28952,7 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="26" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="M46" s="220">
         <v>100</v>
@@ -28888,7 +28994,7 @@
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
       <c r="L47" s="26" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="M47" s="212" t="b">
         <v>0</v>
@@ -32852,7 +32958,7 @@
       <c r="A139" s="1"/>
       <c r="B139" s="33"/>
       <c r="C139" s="73">
-        <f>INT(MAX($C$147:$C$182))+1</f>
+        <f>INT(MAX($C$147:$C$184))+1</f>
         <v>5</v>
       </c>
       <c r="D139" s="3"/>
@@ -33536,7 +33642,7 @@
         <v>398</v>
       </c>
       <c r="N156" s="36" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="O156" s="56" t="s">
         <v>401</v>
@@ -33599,37 +33705,37 @@
         <v>0</v>
       </c>
       <c r="O157" s="56" t="s">
+        <v>426</v>
+      </c>
+      <c r="P157" s="56" t="s">
         <v>427</v>
       </c>
-      <c r="P157" s="56" t="s">
+      <c r="Q157" s="56" t="s">
         <v>428</v>
       </c>
-      <c r="Q157" s="56" t="s">
+      <c r="R157" s="56" t="s">
         <v>429</v>
       </c>
-      <c r="R157" s="56" t="s">
+      <c r="S157" s="56" t="s">
         <v>430</v>
       </c>
-      <c r="S157" s="56" t="s">
+      <c r="T157" s="36" t="s">
         <v>431</v>
       </c>
-      <c r="T157" s="36" t="s">
+      <c r="U157" s="36" t="s">
         <v>432</v>
       </c>
-      <c r="U157" s="36" t="s">
+      <c r="V157" s="36" t="s">
         <v>433</v>
       </c>
-      <c r="V157" s="36" t="s">
+      <c r="W157" s="36" t="s">
         <v>434</v>
       </c>
-      <c r="W157" s="36" t="s">
+      <c r="X157" s="36" t="s">
         <v>435</v>
       </c>
-      <c r="X157" s="36" t="s">
+      <c r="Y157" s="36" t="s">
         <v>436</v>
-      </c>
-      <c r="Y157" s="36" t="s">
-        <v>437</v>
       </c>
       <c r="Z157" s="36">
         <v>12</v>
@@ -33644,7 +33750,7 @@
       <c r="A158" s="1"/>
       <c r="B158" s="33"/>
       <c r="C158" s="73">
-        <f t="shared" ref="C158:C160" si="11">INT(C$140+3)</f>
+        <f t="shared" ref="C158:C162" si="11">INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D158" s="4"/>
@@ -33656,7 +33762,7 @@
       <c r="J158" s="148"/>
       <c r="K158" s="148"/>
       <c r="L158" s="26" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="M158" s="52"/>
       <c r="N158" s="36"/>
@@ -33715,59 +33821,47 @@
       <c r="I159" s="148"/>
       <c r="J159" s="148"/>
       <c r="K159" s="148"/>
-      <c r="L159" s="151" t="s">
-        <v>425</v>
-      </c>
-      <c r="M159" s="151" t="s">
+      <c r="L159" s="148"/>
+      <c r="M159" s="52" t="s">
         <v>399</v>
       </c>
-      <c r="N159" s="31">
-        <v>0</v>
-      </c>
+      <c r="N159" s="36"/>
       <c r="O159" s="31">
         <v>0</v>
       </c>
       <c r="P159" s="31">
-        <f>O160+1</f>
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="Q159" s="31">
-        <f t="shared" ref="Q159" si="12">P160+1</f>
-        <v>101</v>
+        <v>150</v>
       </c>
       <c r="R159" s="31">
-        <f>P160+1</f>
-        <v>101</v>
+        <v>300</v>
       </c>
       <c r="S159" s="31">
-        <f>Q160+1</f>
-        <v>184</v>
+        <v>450</v>
       </c>
       <c r="T159" s="31">
-        <f>Y159</f>
-        <v>549</v>
-      </c>
-      <c r="U159" s="31">
-        <f t="shared" ref="U159" si="13">T160+1</f>
-        <v>914</v>
-      </c>
-      <c r="V159" s="31">
-        <f t="shared" ref="V159" si="14">U160+1</f>
-        <v>1279</v>
-      </c>
-      <c r="W159" s="31">
-        <f t="shared" ref="W159" si="15">V160+1</f>
-        <v>1644</v>
-      </c>
-      <c r="X159" s="31">
-        <f t="shared" ref="X159" si="16">W160+1</f>
-        <v>2009</v>
-      </c>
-      <c r="Y159" s="31">
-        <f>S160+1</f>
-        <v>549</v>
-      </c>
-      <c r="Z159" s="31"/>
+        <v>660</v>
+      </c>
+      <c r="U159" s="221">
+        <f>T159+364</f>
+        <v>1024</v>
+      </c>
+      <c r="V159" s="221">
+        <f t="shared" ref="V159:X159" si="12">U159+364</f>
+        <v>1388</v>
+      </c>
+      <c r="W159" s="221">
+        <f t="shared" si="12"/>
+        <v>1752</v>
+      </c>
+      <c r="X159" s="221">
+        <f t="shared" si="12"/>
+        <v>2116</v>
+      </c>
+      <c r="Y159" s="36"/>
+      <c r="Z159" s="36"/>
       <c r="AA159" s="4"/>
       <c r="AB159" s="16"/>
       <c r="AC159" s="1"/>
@@ -33790,210 +33884,246 @@
       <c r="J160" s="148"/>
       <c r="K160" s="148"/>
       <c r="L160" s="148"/>
-      <c r="M160" s="151" t="s">
+      <c r="M160" s="52" t="s">
         <v>400</v>
       </c>
-      <c r="N160" s="31">
-        <v>99999</v>
+      <c r="N160" s="36">
+        <v>0</v>
       </c>
       <c r="O160" s="31">
         <v>1</v>
       </c>
       <c r="P160" s="31">
-        <v>100</v>
+        <v>149</v>
       </c>
       <c r="Q160" s="31">
-        <v>183</v>
+        <v>299</v>
       </c>
       <c r="R160" s="31">
-        <v>425</v>
+        <v>449</v>
       </c>
       <c r="S160" s="31">
-        <f>S159+364</f>
-        <v>548</v>
+        <v>659</v>
       </c>
       <c r="T160" s="31">
-        <f>T159+364</f>
-        <v>913</v>
-      </c>
-      <c r="U160" s="31">
-        <f t="shared" ref="U160:X160" si="17">U159+364</f>
-        <v>1278</v>
-      </c>
-      <c r="V160" s="31">
-        <f t="shared" si="17"/>
-        <v>1643</v>
-      </c>
-      <c r="W160" s="31">
-        <f t="shared" si="17"/>
-        <v>2008</v>
-      </c>
-      <c r="X160" s="31">
-        <f t="shared" si="17"/>
-        <v>2373</v>
-      </c>
-      <c r="Y160" s="31">
-        <f>X160</f>
-        <v>2373</v>
-      </c>
-      <c r="Z160" s="31"/>
+        <v>1024</v>
+      </c>
+      <c r="U160" s="221">
+        <f t="shared" ref="U160:X160" si="13">T160+364</f>
+        <v>1388</v>
+      </c>
+      <c r="V160" s="221">
+        <f t="shared" si="13"/>
+        <v>1752</v>
+      </c>
+      <c r="W160" s="221">
+        <f t="shared" si="13"/>
+        <v>2116</v>
+      </c>
+      <c r="X160" s="221">
+        <f t="shared" si="13"/>
+        <v>2480</v>
+      </c>
+      <c r="Y160" s="36">
+        <v>0</v>
+      </c>
+      <c r="Z160" s="36">
+        <v>0</v>
+      </c>
       <c r="AA160" s="4"/>
       <c r="AB160" s="16"/>
       <c r="AC160" s="1"/>
       <c r="AD160" s="1"/>
       <c r="AE160" s="1"/>
     </row>
-    <row r="161" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
       <c r="B161" s="33"/>
       <c r="C161" s="73">
-        <f>INT($C$140)+2</f>
-        <v>3</v>
+        <f t="shared" si="11"/>
+        <v>4</v>
       </c>
       <c r="D161" s="4"/>
       <c r="E161" s="5"/>
       <c r="F161" s="5"/>
       <c r="G161" s="4"/>
-      <c r="H161" s="64" t="s">
-        <v>257</v>
-      </c>
-      <c r="I161" s="64" t="s">
-        <v>370</v>
-      </c>
-      <c r="J161" s="2"/>
-      <c r="K161" s="2"/>
-      <c r="L161" s="148"/>
-      <c r="M161" s="148"/>
-      <c r="N161" s="214"/>
-      <c r="O161" s="214"/>
-      <c r="P161" s="214"/>
-      <c r="Q161" s="160"/>
-      <c r="R161" s="160"/>
-      <c r="S161" s="160"/>
-      <c r="T161" s="160"/>
-      <c r="U161" s="160"/>
-      <c r="V161" s="160"/>
-      <c r="W161" s="160"/>
-      <c r="X161" s="160"/>
-      <c r="Y161" s="160"/>
-      <c r="Z161" s="160"/>
+      <c r="H161" s="148"/>
+      <c r="I161" s="148"/>
+      <c r="J161" s="148"/>
+      <c r="K161" s="148"/>
+      <c r="L161" s="151" t="s">
+        <v>424</v>
+      </c>
+      <c r="M161" s="151" t="s">
+        <v>399</v>
+      </c>
+      <c r="N161" s="31">
+        <v>0</v>
+      </c>
+      <c r="O161" s="31">
+        <v>0</v>
+      </c>
+      <c r="P161" s="31">
+        <f>O162+1</f>
+        <v>2</v>
+      </c>
+      <c r="Q161" s="31">
+        <f t="shared" ref="Q161" si="14">P162+1</f>
+        <v>101</v>
+      </c>
+      <c r="R161" s="31">
+        <f>P162+1</f>
+        <v>101</v>
+      </c>
+      <c r="S161" s="31">
+        <f>Q162+1</f>
+        <v>184</v>
+      </c>
+      <c r="T161" s="31">
+        <f t="shared" ref="T161" si="15">S162+1</f>
+        <v>549</v>
+      </c>
+      <c r="U161" s="221">
+        <f>T161+364</f>
+        <v>913</v>
+      </c>
+      <c r="V161" s="221">
+        <f t="shared" ref="V161:X161" si="16">U161+364</f>
+        <v>1277</v>
+      </c>
+      <c r="W161" s="221">
+        <f t="shared" si="16"/>
+        <v>1641</v>
+      </c>
+      <c r="X161" s="221">
+        <f t="shared" si="16"/>
+        <v>2005</v>
+      </c>
+      <c r="Y161" s="222">
+        <f>T161</f>
+        <v>549</v>
+      </c>
+      <c r="Z161" s="31">
+        <v>0</v>
+      </c>
       <c r="AA161" s="4"/>
       <c r="AB161" s="16"/>
       <c r="AC161" s="1"/>
       <c r="AD161" s="1"/>
       <c r="AE161" s="1"/>
     </row>
-    <row r="162" spans="1:31" outlineLevel="3" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
       <c r="B162" s="33"/>
       <c r="C162" s="73">
-        <f>INT($C$140)+3</f>
+        <f t="shared" si="11"/>
         <v>4</v>
       </c>
       <c r="D162" s="4"/>
-      <c r="E162" s="5">
-        <v>0</v>
-      </c>
+      <c r="E162" s="5"/>
       <c r="F162" s="5"/>
       <c r="G162" s="4"/>
-      <c r="H162" s="31" t="s">
-        <v>266</v>
-      </c>
-      <c r="I162" s="31">
-        <v>0</v>
-      </c>
+      <c r="H162" s="148"/>
+      <c r="I162" s="148"/>
       <c r="J162" s="148"/>
       <c r="K162" s="148"/>
       <c r="L162" s="148"/>
-      <c r="M162" s="148"/>
-      <c r="N162" s="218" t="s">
-        <v>423</v>
-      </c>
-      <c r="O162" s="218"/>
-      <c r="P162" s="218"/>
-      <c r="Q162" s="218"/>
-      <c r="R162" s="218"/>
-      <c r="S162" s="219"/>
-      <c r="T162" s="219"/>
-      <c r="U162" s="219"/>
-      <c r="V162" s="219"/>
-      <c r="W162" s="219"/>
-      <c r="X162" s="219"/>
-      <c r="Y162" s="219"/>
-      <c r="Z162" s="219"/>
+      <c r="M162" s="151" t="s">
+        <v>400</v>
+      </c>
+      <c r="N162" s="31">
+        <v>99999</v>
+      </c>
+      <c r="O162" s="31">
+        <v>1</v>
+      </c>
+      <c r="P162" s="31">
+        <v>100</v>
+      </c>
+      <c r="Q162" s="31">
+        <v>183</v>
+      </c>
+      <c r="R162" s="31">
+        <v>425</v>
+      </c>
+      <c r="S162" s="31">
+        <f>S161+364</f>
+        <v>548</v>
+      </c>
+      <c r="T162" s="31">
+        <f>T161+364</f>
+        <v>913</v>
+      </c>
+      <c r="U162" s="221">
+        <f t="shared" ref="U162:X162" si="17">T162+364</f>
+        <v>1277</v>
+      </c>
+      <c r="V162" s="221">
+        <f t="shared" si="17"/>
+        <v>1641</v>
+      </c>
+      <c r="W162" s="221">
+        <f t="shared" si="17"/>
+        <v>2005</v>
+      </c>
+      <c r="X162" s="221">
+        <f t="shared" si="17"/>
+        <v>2369</v>
+      </c>
+      <c r="Y162" s="222">
+        <f>X162</f>
+        <v>2369</v>
+      </c>
+      <c r="Z162" s="31">
+        <v>0</v>
+      </c>
       <c r="AA162" s="4"/>
       <c r="AB162" s="16"/>
       <c r="AC162" s="1"/>
       <c r="AD162" s="1"/>
       <c r="AE162" s="1"/>
     </row>
-    <row r="163" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="33"/>
       <c r="C163" s="73">
-        <f t="shared" ref="C163:C179" si="18">INT(C$140+3)</f>
-        <v>4</v>
+        <f>INT($C$140)+2</f>
+        <v>3</v>
       </c>
       <c r="D163" s="4"/>
-      <c r="E163" s="5">
-        <v>1</v>
-      </c>
+      <c r="E163" s="5"/>
       <c r="F163" s="5"/>
       <c r="G163" s="4"/>
-      <c r="H163" s="31" t="s">
-        <v>265</v>
-      </c>
-      <c r="I163" s="31">
-        <v>0</v>
-      </c>
-      <c r="J163" s="148"/>
-      <c r="K163" s="148"/>
+      <c r="H163" s="64" t="s">
+        <v>257</v>
+      </c>
+      <c r="I163" s="64" t="s">
+        <v>370</v>
+      </c>
+      <c r="J163" s="2"/>
+      <c r="K163" s="2"/>
       <c r="L163" s="148"/>
       <c r="M163" s="148"/>
-      <c r="N163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="O163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="P163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="Q163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="R163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="S163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="T163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="U163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="V163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="W163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="X163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="Y163" s="217" t="s">
-        <v>422</v>
-      </c>
-      <c r="Z163" s="217"/>
+      <c r="N163" s="214"/>
+      <c r="O163" s="214"/>
+      <c r="P163" s="214"/>
+      <c r="Q163" s="160"/>
+      <c r="R163" s="160"/>
+      <c r="S163" s="160"/>
+      <c r="T163" s="160"/>
+      <c r="U163" s="160"/>
+      <c r="V163" s="160"/>
+      <c r="W163" s="160"/>
+      <c r="X163" s="160"/>
+      <c r="Y163" s="160"/>
+      <c r="Z163" s="160"/>
       <c r="AA163" s="4"/>
       <c r="AB163" s="16"/>
       <c r="AC163" s="1"/>
       <c r="AD163" s="1"/>
       <c r="AE163" s="1"/>
     </row>
-    <row r="164" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:31" outlineLevel="3" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="33"/>
       <c r="C164" s="73">
@@ -34002,12 +34132,12 @@
       </c>
       <c r="D164" s="4"/>
       <c r="E164" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F164" s="5"/>
       <c r="G164" s="4"/>
       <c r="H164" s="31" t="s">
-        <v>372</v>
+        <v>266</v>
       </c>
       <c r="I164" s="31">
         <v>0</v>
@@ -34015,20 +34145,24 @@
       <c r="J164" s="148"/>
       <c r="K164" s="148"/>
       <c r="L164" s="148"/>
-      <c r="M164" s="148"/>
-      <c r="N164" s="148"/>
-      <c r="O164" s="148"/>
-      <c r="P164" s="148"/>
-      <c r="Q164" s="148"/>
-      <c r="R164" s="148"/>
-      <c r="S164" s="148"/>
-      <c r="T164" s="2"/>
-      <c r="U164" s="2"/>
-      <c r="V164" s="2"/>
-      <c r="W164" s="2"/>
-      <c r="X164" s="2"/>
-      <c r="Y164" s="2"/>
-      <c r="Z164" s="2"/>
+      <c r="M164" s="223" t="s">
+        <v>448</v>
+      </c>
+      <c r="N164" s="218" t="s">
+        <v>447</v>
+      </c>
+      <c r="O164" s="218"/>
+      <c r="P164" s="218"/>
+      <c r="Q164" s="218"/>
+      <c r="R164" s="218"/>
+      <c r="S164" s="219"/>
+      <c r="T164" s="219"/>
+      <c r="U164" s="219"/>
+      <c r="V164" s="219"/>
+      <c r="W164" s="219"/>
+      <c r="X164" s="219"/>
+      <c r="Y164" s="219"/>
+      <c r="Z164" s="219"/>
       <c r="AA164" s="4"/>
       <c r="AB164" s="16"/>
       <c r="AC164" s="1"/>
@@ -34039,17 +34173,17 @@
       <c r="A165" s="1"/>
       <c r="B165" s="33"/>
       <c r="C165" s="73">
-        <f>INT($C$140)+3</f>
+        <f t="shared" ref="C165:C181" si="18">INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D165" s="4"/>
       <c r="E165" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F165" s="5"/>
       <c r="G165" s="4"/>
       <c r="H165" s="31" t="s">
-        <v>373</v>
+        <v>265</v>
       </c>
       <c r="I165" s="31">
         <v>0</v>
@@ -34058,21 +34192,43 @@
       <c r="K165" s="148"/>
       <c r="L165" s="148"/>
       <c r="M165" s="148"/>
-      <c r="N165" s="56" t="s">
+      <c r="N165" s="217" t="s">
         <v>422</v>
       </c>
-      <c r="O165" s="148"/>
-      <c r="P165" s="148"/>
-      <c r="Q165" s="148"/>
-      <c r="R165" s="148"/>
-      <c r="S165" s="148"/>
-      <c r="T165" s="2"/>
-      <c r="U165" s="2"/>
-      <c r="V165" s="2"/>
-      <c r="W165" s="2"/>
-      <c r="X165" s="2"/>
-      <c r="Y165" s="2"/>
-      <c r="Z165" s="2"/>
+      <c r="O165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="P165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="Q165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="R165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="S165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="T165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="U165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="V165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="W165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="X165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y165" s="217" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z165" s="217"/>
       <c r="AA165" s="4"/>
       <c r="AB165" s="16"/>
       <c r="AC165" s="1"/>
@@ -34083,17 +34239,17 @@
       <c r="A166" s="1"/>
       <c r="B166" s="33"/>
       <c r="C166" s="73">
-        <f>INT(C$140+3)</f>
+        <f>INT($C$140)+3</f>
         <v>4</v>
       </c>
       <c r="D166" s="4"/>
       <c r="E166" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F166" s="5"/>
       <c r="G166" s="4"/>
       <c r="H166" s="31" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="I166" s="31">
         <v>0</v>
@@ -34102,9 +34258,7 @@
       <c r="K166" s="148"/>
       <c r="L166" s="148"/>
       <c r="M166" s="148"/>
-      <c r="N166" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N166" s="148"/>
       <c r="O166" s="148"/>
       <c r="P166" s="148"/>
       <c r="Q166" s="148"/>
@@ -34127,17 +34281,17 @@
       <c r="A167" s="1"/>
       <c r="B167" s="33"/>
       <c r="C167" s="73">
-        <f>INT(C$140+3)</f>
+        <f>INT($C$140)+3</f>
         <v>4</v>
       </c>
       <c r="D167" s="4"/>
       <c r="E167" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F167" s="5"/>
       <c r="G167" s="4"/>
       <c r="H167" s="31" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="I167" s="31">
         <v>0</v>
@@ -34171,17 +34325,17 @@
       <c r="A168" s="1"/>
       <c r="B168" s="33"/>
       <c r="C168" s="73">
-        <f t="shared" si="18"/>
+        <f>INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D168" s="4"/>
       <c r="E168" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F168" s="5"/>
       <c r="G168" s="4"/>
       <c r="H168" s="31" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="I168" s="31">
         <v>0</v>
@@ -34215,17 +34369,17 @@
       <c r="A169" s="1"/>
       <c r="B169" s="33"/>
       <c r="C169" s="73">
-        <f t="shared" si="18"/>
+        <f>INT(C$140+3)</f>
         <v>4</v>
       </c>
       <c r="D169" s="4"/>
       <c r="E169" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F169" s="5"/>
       <c r="G169" s="4"/>
       <c r="H169" s="31" t="s">
-        <v>397</v>
+        <v>375</v>
       </c>
       <c r="I169" s="31">
         <v>0</v>
@@ -34264,12 +34418,12 @@
       </c>
       <c r="D170" s="4"/>
       <c r="E170" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F170" s="5"/>
       <c r="G170" s="4"/>
       <c r="H170" s="31" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="I170" s="31">
         <v>0</v>
@@ -34278,7 +34432,9 @@
       <c r="K170" s="148"/>
       <c r="L170" s="148"/>
       <c r="M170" s="148"/>
-      <c r="N170" s="148"/>
+      <c r="N170" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="O170" s="148"/>
       <c r="P170" s="148"/>
       <c r="Q170" s="148"/>
@@ -34306,12 +34462,12 @@
       </c>
       <c r="D171" s="4"/>
       <c r="E171" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F171" s="5"/>
       <c r="G171" s="4"/>
       <c r="H171" s="31" t="s">
-        <v>377</v>
+        <v>397</v>
       </c>
       <c r="I171" s="31">
         <v>0</v>
@@ -34320,7 +34476,9 @@
       <c r="K171" s="148"/>
       <c r="L171" s="148"/>
       <c r="M171" s="148"/>
-      <c r="N171" s="148"/>
+      <c r="N171" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="O171" s="148"/>
       <c r="P171" s="148"/>
       <c r="Q171" s="148"/>
@@ -34348,12 +34506,12 @@
       </c>
       <c r="D172" s="4"/>
       <c r="E172" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F172" s="5"/>
       <c r="G172" s="4"/>
       <c r="H172" s="31" t="s">
-        <v>260</v>
+        <v>376</v>
       </c>
       <c r="I172" s="31">
         <v>0</v>
@@ -34362,24 +34520,18 @@
       <c r="K172" s="148"/>
       <c r="L172" s="148"/>
       <c r="M172" s="148"/>
-      <c r="N172" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N172" s="148"/>
       <c r="O172" s="148"/>
       <c r="P172" s="148"/>
       <c r="Q172" s="148"/>
-      <c r="R172" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="R172" s="148"/>
       <c r="S172" s="148"/>
       <c r="T172" s="2"/>
       <c r="U172" s="2"/>
       <c r="V172" s="2"/>
       <c r="W172" s="2"/>
       <c r="X172" s="2"/>
-      <c r="Y172" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="Y172" s="2"/>
       <c r="Z172" s="2"/>
       <c r="AA172" s="4"/>
       <c r="AB172" s="16"/>
@@ -34396,12 +34548,12 @@
       </c>
       <c r="D173" s="4"/>
       <c r="E173" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F173" s="5"/>
       <c r="G173" s="4"/>
       <c r="H173" s="31" t="s">
-        <v>261</v>
+        <v>377</v>
       </c>
       <c r="I173" s="31">
         <v>0</v>
@@ -34410,24 +34562,18 @@
       <c r="K173" s="148"/>
       <c r="L173" s="148"/>
       <c r="M173" s="148"/>
-      <c r="N173" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N173" s="148"/>
       <c r="O173" s="148"/>
       <c r="P173" s="148"/>
       <c r="Q173" s="148"/>
-      <c r="R173" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="R173" s="148"/>
       <c r="S173" s="148"/>
       <c r="T173" s="2"/>
       <c r="U173" s="2"/>
       <c r="V173" s="2"/>
       <c r="W173" s="2"/>
       <c r="X173" s="2"/>
-      <c r="Y173" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="Y173" s="2"/>
       <c r="Z173" s="2"/>
       <c r="AA173" s="4"/>
       <c r="AB173" s="16"/>
@@ -34444,12 +34590,12 @@
       </c>
       <c r="D174" s="4"/>
       <c r="E174" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F174" s="5"/>
       <c r="G174" s="4"/>
       <c r="H174" s="31" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I174" s="31">
         <v>0</v>
@@ -34468,21 +34614,11 @@
         <v>422</v>
       </c>
       <c r="S174" s="148"/>
-      <c r="T174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="U174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="V174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="W174" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="X174" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="T174" s="2"/>
+      <c r="U174" s="2"/>
+      <c r="V174" s="2"/>
+      <c r="W174" s="2"/>
+      <c r="X174" s="2"/>
       <c r="Y174" s="56" t="s">
         <v>422</v>
       </c>
@@ -34502,12 +34638,12 @@
       </c>
       <c r="D175" s="4"/>
       <c r="E175" s="5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F175" s="5"/>
       <c r="G175" s="4"/>
       <c r="H175" s="31" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="I175" s="31">
         <v>0</v>
@@ -34516,18 +34652,24 @@
       <c r="K175" s="148"/>
       <c r="L175" s="148"/>
       <c r="M175" s="148"/>
-      <c r="N175" s="148"/>
+      <c r="N175" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="O175" s="148"/>
       <c r="P175" s="148"/>
       <c r="Q175" s="148"/>
-      <c r="R175" s="148"/>
+      <c r="R175" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="S175" s="148"/>
       <c r="T175" s="2"/>
       <c r="U175" s="2"/>
       <c r="V175" s="2"/>
       <c r="W175" s="2"/>
       <c r="X175" s="2"/>
-      <c r="Y175" s="2"/>
+      <c r="Y175" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="Z175" s="2"/>
       <c r="AA175" s="4"/>
       <c r="AB175" s="16"/>
@@ -34544,12 +34686,12 @@
       </c>
       <c r="D176" s="4"/>
       <c r="E176" s="5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F176" s="5"/>
       <c r="G176" s="4"/>
       <c r="H176" s="31" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="I176" s="31">
         <v>0</v>
@@ -34563,15 +34705,11 @@
       </c>
       <c r="O176" s="148"/>
       <c r="P176" s="148"/>
-      <c r="Q176" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="Q176" s="148"/>
       <c r="R176" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="S176" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="S176" s="148"/>
       <c r="T176" s="56" t="s">
         <v>422</v>
       </c>
@@ -34590,7 +34728,7 @@
       <c r="Y176" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Z176" s="56"/>
+      <c r="Z176" s="2"/>
       <c r="AA176" s="4"/>
       <c r="AB176" s="16"/>
       <c r="AC176" s="1"/>
@@ -34606,12 +34744,12 @@
       </c>
       <c r="D177" s="4"/>
       <c r="E177" s="5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F177" s="5"/>
       <c r="G177" s="4"/>
       <c r="H177" s="31" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="I177" s="31">
         <v>0</v>
@@ -34620,39 +34758,19 @@
       <c r="K177" s="148"/>
       <c r="L177" s="148"/>
       <c r="M177" s="148"/>
-      <c r="N177" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="N177" s="148"/>
       <c r="O177" s="148"/>
       <c r="P177" s="148"/>
-      <c r="Q177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="R177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="S177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="T177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="U177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="V177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="W177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="X177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="Y177" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="Z177" s="56"/>
+      <c r="Q177" s="148"/>
+      <c r="R177" s="148"/>
+      <c r="S177" s="148"/>
+      <c r="T177" s="2"/>
+      <c r="U177" s="2"/>
+      <c r="V177" s="2"/>
+      <c r="W177" s="2"/>
+      <c r="X177" s="2"/>
+      <c r="Y177" s="2"/>
+      <c r="Z177" s="2"/>
       <c r="AA177" s="4"/>
       <c r="AB177" s="16"/>
       <c r="AC177" s="1"/>
@@ -34668,12 +34786,12 @@
       </c>
       <c r="D178" s="4"/>
       <c r="E178" s="5">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F178" s="5"/>
       <c r="G178" s="4"/>
       <c r="H178" s="31" t="s">
-        <v>371</v>
+        <v>258</v>
       </c>
       <c r="I178" s="31">
         <v>0</v>
@@ -34730,12 +34848,12 @@
       </c>
       <c r="D179" s="4"/>
       <c r="E179" s="5">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F179" s="5"/>
       <c r="G179" s="4"/>
       <c r="H179" s="31" t="s">
-        <v>438</v>
+        <v>259</v>
       </c>
       <c r="I179" s="31">
         <v>0</v>
@@ -34787,17 +34905,17 @@
       <c r="A180" s="1"/>
       <c r="B180" s="33"/>
       <c r="C180" s="73">
-        <f>INT(C$140+3)</f>
+        <f t="shared" si="18"/>
         <v>4</v>
       </c>
       <c r="D180" s="4"/>
       <c r="E180" s="5">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F180" s="5"/>
       <c r="G180" s="4"/>
       <c r="H180" s="31" t="s">
-        <v>443</v>
+        <v>371</v>
       </c>
       <c r="I180" s="31">
         <v>0</v>
@@ -34849,17 +34967,17 @@
       <c r="A181" s="1"/>
       <c r="B181" s="33"/>
       <c r="C181" s="73">
-        <f>INT(C$140+3)</f>
+        <f t="shared" si="18"/>
         <v>4</v>
       </c>
       <c r="D181" s="4"/>
       <c r="E181" s="5">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F181" s="5"/>
       <c r="G181" s="4"/>
       <c r="H181" s="31" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="I181" s="31">
         <v>0</v>
@@ -34868,573 +34986,623 @@
       <c r="K181" s="148"/>
       <c r="L181" s="148"/>
       <c r="M181" s="148"/>
-      <c r="N181" s="216" t="s">
+      <c r="N181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="O181" s="215"/>
-      <c r="P181" s="215"/>
-      <c r="Q181" s="215"/>
-      <c r="R181" s="216" t="s">
+      <c r="O181" s="148"/>
+      <c r="P181" s="148"/>
+      <c r="Q181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="S181" s="215"/>
-      <c r="T181" s="216" t="s">
+      <c r="R181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="U181" s="216" t="s">
+      <c r="S181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="V181" s="216" t="s">
+      <c r="T181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="W181" s="216" t="s">
+      <c r="U181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="X181" s="216" t="s">
+      <c r="V181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Y181" s="216" t="s">
+      <c r="W181" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Z181" s="216"/>
+      <c r="X181" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y181" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z181" s="56"/>
       <c r="AA181" s="4"/>
       <c r="AB181" s="16"/>
       <c r="AC181" s="1"/>
       <c r="AD181" s="1"/>
       <c r="AE181" s="1"/>
     </row>
-    <row r="182" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A182" s="1"/>
       <c r="B182" s="33"/>
       <c r="C182" s="73">
-        <f>INT($C$140)+3.005</f>
-        <v>4.0049999999999999</v>
+        <f>INT(C$140+3)</f>
+        <v>4</v>
       </c>
       <c r="D182" s="4"/>
-      <c r="E182" s="4"/>
-      <c r="F182" s="4"/>
+      <c r="E182" s="5">
+        <v>18</v>
+      </c>
+      <c r="F182" s="5"/>
       <c r="G182" s="4"/>
-      <c r="H182" s="4"/>
-      <c r="I182" s="4"/>
-      <c r="J182" s="4"/>
-      <c r="K182" s="4"/>
-      <c r="L182" s="4"/>
-      <c r="M182" s="4"/>
-      <c r="N182" s="4"/>
-      <c r="O182" s="4"/>
-      <c r="P182" s="4"/>
-      <c r="Q182" s="4"/>
-      <c r="R182" s="4"/>
-      <c r="S182" s="4"/>
-      <c r="T182" s="4"/>
-      <c r="U182" s="4"/>
-      <c r="V182" s="4"/>
-      <c r="W182" s="4"/>
-      <c r="X182" s="4"/>
-      <c r="Y182" s="4"/>
-      <c r="Z182" s="4"/>
-      <c r="AA182" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="H182" s="31" t="s">
+        <v>442</v>
+      </c>
+      <c r="I182" s="31">
+        <v>0</v>
+      </c>
+      <c r="J182" s="148"/>
+      <c r="K182" s="148"/>
+      <c r="L182" s="148"/>
+      <c r="M182" s="148"/>
+      <c r="N182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="O182" s="148"/>
+      <c r="P182" s="148"/>
+      <c r="Q182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="R182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="S182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="T182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="U182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="V182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="W182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="X182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y182" s="56" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z182" s="56"/>
+      <c r="AA182" s="4"/>
       <c r="AB182" s="16"/>
       <c r="AC182" s="1"/>
       <c r="AD182" s="1"/>
       <c r="AE182" s="1"/>
     </row>
-    <row r="183" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A183" s="1"/>
       <c r="B183" s="33"/>
       <c r="C183" s="73">
-        <f>INT($C$140)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>INT(C$140+3)</f>
+        <v>4</v>
       </c>
       <c r="D183" s="4"/>
-      <c r="E183" s="4"/>
-      <c r="F183" s="4"/>
+      <c r="E183" s="5">
+        <v>19</v>
+      </c>
+      <c r="F183" s="5"/>
       <c r="G183" s="4"/>
-      <c r="H183" s="4"/>
-      <c r="I183" s="4"/>
-      <c r="J183" s="4"/>
-      <c r="K183" s="4"/>
-      <c r="L183" s="4"/>
-      <c r="M183" s="4"/>
-      <c r="N183" s="4"/>
-      <c r="O183" s="4"/>
-      <c r="P183" s="4"/>
-      <c r="Q183" s="4"/>
-      <c r="R183" s="4"/>
-      <c r="S183" s="4"/>
-      <c r="T183" s="4"/>
-      <c r="U183" s="4"/>
-      <c r="V183" s="4"/>
-      <c r="W183" s="4"/>
-      <c r="X183" s="4"/>
-      <c r="Y183" s="4"/>
-      <c r="Z183" s="4"/>
+      <c r="H183" s="31" t="s">
+        <v>443</v>
+      </c>
+      <c r="I183" s="31">
+        <v>0</v>
+      </c>
+      <c r="J183" s="148"/>
+      <c r="K183" s="148"/>
+      <c r="L183" s="148"/>
+      <c r="M183" s="148"/>
+      <c r="N183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="O183" s="215"/>
+      <c r="P183" s="215"/>
+      <c r="Q183" s="215"/>
+      <c r="R183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="S183" s="215"/>
+      <c r="T183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="U183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="V183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="W183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="X183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y183" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z183" s="216"/>
       <c r="AA183" s="4"/>
       <c r="AB183" s="16"/>
       <c r="AC183" s="1"/>
       <c r="AD183" s="1"/>
       <c r="AE183" s="1"/>
     </row>
-    <row r="184" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
-      <c r="B184" s="35"/>
-      <c r="C184" s="76">
-        <f>INT($C$140)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D184" s="17"/>
-      <c r="E184" s="17"/>
-      <c r="F184" s="17"/>
-      <c r="G184" s="17"/>
-      <c r="H184" s="17"/>
-      <c r="I184" s="17"/>
-      <c r="J184" s="17"/>
-      <c r="K184" s="17"/>
-      <c r="L184" s="17"/>
-      <c r="M184" s="17"/>
-      <c r="N184" s="17"/>
-      <c r="O184" s="17"/>
-      <c r="P184" s="17"/>
-      <c r="Q184" s="17"/>
-      <c r="R184" s="17"/>
-      <c r="S184" s="17"/>
-      <c r="T184" s="17"/>
-      <c r="U184" s="17"/>
-      <c r="V184" s="17"/>
-      <c r="W184" s="17"/>
-      <c r="X184" s="17"/>
-      <c r="Y184" s="17"/>
-      <c r="Z184" s="17"/>
-      <c r="AA184" s="17"/>
-      <c r="AB184" s="18" t="s">
-        <v>1</v>
-      </c>
+      <c r="B184" s="33"/>
+      <c r="C184" s="73">
+        <f>INT($C$140)+3.005</f>
+        <v>4.0049999999999999</v>
+      </c>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+      <c r="H184" s="4"/>
+      <c r="I184" s="4"/>
+      <c r="J184" s="4"/>
+      <c r="K184" s="4"/>
+      <c r="L184" s="4"/>
+      <c r="M184" s="4"/>
+      <c r="N184" s="4"/>
+      <c r="O184" s="4"/>
+      <c r="P184" s="4"/>
+      <c r="Q184" s="4"/>
+      <c r="R184" s="4"/>
+      <c r="S184" s="4"/>
+      <c r="T184" s="4"/>
+      <c r="U184" s="4"/>
+      <c r="V184" s="4"/>
+      <c r="W184" s="4"/>
+      <c r="X184" s="4"/>
+      <c r="Y184" s="4"/>
+      <c r="Z184" s="4"/>
+      <c r="AA184" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB184" s="16"/>
       <c r="AC184" s="1"/>
       <c r="AD184" s="1"/>
       <c r="AE184" s="1"/>
     </row>
-    <row r="185" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
-      <c r="B185" s="19"/>
-      <c r="C185" s="77">
-        <f>INT($C$140)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D185" s="19"/>
-      <c r="E185" s="19"/>
-      <c r="F185" s="19"/>
-      <c r="G185" s="19"/>
-      <c r="H185" s="19"/>
-      <c r="I185" s="19"/>
-      <c r="J185" s="19"/>
-      <c r="K185" s="19"/>
-      <c r="L185" s="19"/>
-      <c r="M185" s="19"/>
-      <c r="N185" s="19"/>
-      <c r="O185" s="19"/>
-      <c r="P185" s="19"/>
-      <c r="Q185" s="19"/>
-      <c r="R185" s="19"/>
-      <c r="S185" s="19"/>
-      <c r="T185" s="19"/>
-      <c r="U185" s="19"/>
-      <c r="V185" s="19"/>
-      <c r="W185" s="19"/>
-      <c r="X185" s="19"/>
-      <c r="Y185" s="19"/>
-      <c r="Z185" s="19"/>
-      <c r="AA185" s="19"/>
-      <c r="AB185" s="19"/>
+      <c r="B185" s="33"/>
+      <c r="C185" s="73">
+        <f>INT($C$140)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D185" s="4"/>
+      <c r="E185" s="4"/>
+      <c r="F185" s="4"/>
+      <c r="G185" s="4"/>
+      <c r="H185" s="4"/>
+      <c r="I185" s="4"/>
+      <c r="J185" s="4"/>
+      <c r="K185" s="4"/>
+      <c r="L185" s="4"/>
+      <c r="M185" s="4"/>
+      <c r="N185" s="4"/>
+      <c r="O185" s="4"/>
+      <c r="P185" s="4"/>
+      <c r="Q185" s="4"/>
+      <c r="R185" s="4"/>
+      <c r="S185" s="4"/>
+      <c r="T185" s="4"/>
+      <c r="U185" s="4"/>
+      <c r="V185" s="4"/>
+      <c r="W185" s="4"/>
+      <c r="X185" s="4"/>
+      <c r="Y185" s="4"/>
+      <c r="Z185" s="4"/>
+      <c r="AA185" s="4"/>
+      <c r="AB185" s="16"/>
       <c r="AC185" s="1"/>
       <c r="AD185" s="1"/>
       <c r="AE185" s="1"/>
     </row>
-    <row r="186" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
-      <c r="B186" s="1"/>
-      <c r="C186" s="73">
-        <f>INT($C$140)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D186" s="1"/>
-      <c r="E186" s="1"/>
-      <c r="F186" s="1"/>
-      <c r="G186" s="1"/>
-      <c r="H186" s="1"/>
-      <c r="I186" s="1"/>
-      <c r="J186" s="1"/>
-      <c r="K186" s="1"/>
-      <c r="L186" s="1"/>
-      <c r="M186" s="1"/>
-      <c r="N186" s="1"/>
-      <c r="O186" s="1"/>
-      <c r="P186" s="1"/>
-      <c r="Q186" s="1"/>
-      <c r="R186" s="1"/>
-      <c r="S186" s="1"/>
-      <c r="T186" s="1"/>
-      <c r="U186" s="1"/>
-      <c r="V186" s="1"/>
-      <c r="W186" s="1"/>
-      <c r="X186" s="1"/>
-      <c r="Y186" s="1"/>
-      <c r="Z186" s="1"/>
-      <c r="AA186" s="1"/>
-      <c r="AB186" s="1"/>
+      <c r="B186" s="35"/>
+      <c r="C186" s="76">
+        <f>INT($C$140)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D186" s="17"/>
+      <c r="E186" s="17"/>
+      <c r="F186" s="17"/>
+      <c r="G186" s="17"/>
+      <c r="H186" s="17"/>
+      <c r="I186" s="17"/>
+      <c r="J186" s="17"/>
+      <c r="K186" s="17"/>
+      <c r="L186" s="17"/>
+      <c r="M186" s="17"/>
+      <c r="N186" s="17"/>
+      <c r="O186" s="17"/>
+      <c r="P186" s="17"/>
+      <c r="Q186" s="17"/>
+      <c r="R186" s="17"/>
+      <c r="S186" s="17"/>
+      <c r="T186" s="17"/>
+      <c r="U186" s="17"/>
+      <c r="V186" s="17"/>
+      <c r="W186" s="17"/>
+      <c r="X186" s="17"/>
+      <c r="Y186" s="17"/>
+      <c r="Z186" s="17"/>
+      <c r="AA186" s="17"/>
+      <c r="AB186" s="18" t="s">
+        <v>1</v>
+      </c>
       <c r="AC186" s="1"/>
       <c r="AD186" s="1"/>
       <c r="AE186" s="1"/>
     </row>
-    <row r="187" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
-      <c r="B187" s="1"/>
-      <c r="C187" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D187" s="1"/>
-      <c r="E187" s="1"/>
-      <c r="F187" s="1"/>
-      <c r="G187" s="1"/>
-      <c r="H187" s="1"/>
-      <c r="I187" s="1"/>
-      <c r="J187" s="1"/>
-      <c r="K187" s="1"/>
-      <c r="L187" s="1"/>
-      <c r="M187" s="1"/>
-      <c r="N187" s="1"/>
-      <c r="O187" s="1"/>
-      <c r="P187" s="1"/>
-      <c r="Q187" s="1"/>
-      <c r="R187" s="1"/>
-      <c r="S187" s="1"/>
-      <c r="T187" s="1"/>
-      <c r="U187" s="1"/>
-      <c r="V187" s="1"/>
-      <c r="W187" s="1"/>
-      <c r="X187" s="1"/>
-      <c r="Y187" s="1"/>
-      <c r="Z187" s="1"/>
-      <c r="AA187" s="1"/>
-      <c r="AB187" s="1"/>
+      <c r="B187" s="19"/>
+      <c r="C187" s="77">
+        <f>INT($C$140)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D187" s="19"/>
+      <c r="E187" s="19"/>
+      <c r="F187" s="19"/>
+      <c r="G187" s="19"/>
+      <c r="H187" s="19"/>
+      <c r="I187" s="19"/>
+      <c r="J187" s="19"/>
+      <c r="K187" s="19"/>
+      <c r="L187" s="19"/>
+      <c r="M187" s="19"/>
+      <c r="N187" s="19"/>
+      <c r="O187" s="19"/>
+      <c r="P187" s="19"/>
+      <c r="Q187" s="19"/>
+      <c r="R187" s="19"/>
+      <c r="S187" s="19"/>
+      <c r="T187" s="19"/>
+      <c r="U187" s="19"/>
+      <c r="V187" s="19"/>
+      <c r="W187" s="19"/>
+      <c r="X187" s="19"/>
+      <c r="Y187" s="19"/>
+      <c r="Z187" s="19"/>
+      <c r="AA187" s="19"/>
+      <c r="AB187" s="19"/>
       <c r="AC187" s="1"/>
       <c r="AD187" s="1"/>
       <c r="AE187" s="1"/>
     </row>
-    <row r="188" spans="1:31" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
-      <c r="B188" s="20"/>
-      <c r="C188" s="74">
-        <f>INT($C$191)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D188" s="20"/>
-      <c r="E188" s="20"/>
-      <c r="F188" s="20"/>
-      <c r="G188" s="20"/>
-      <c r="H188" s="20"/>
-      <c r="I188" s="20"/>
-      <c r="J188" s="20"/>
-      <c r="K188" s="20"/>
-      <c r="L188" s="20"/>
-      <c r="M188" s="20"/>
-      <c r="N188" s="20"/>
-      <c r="O188" s="20"/>
-      <c r="P188" s="20"/>
-      <c r="Q188" s="20"/>
-      <c r="R188" s="20"/>
-      <c r="S188" s="20"/>
-      <c r="T188" s="20"/>
-      <c r="U188" s="20"/>
-      <c r="V188" s="20"/>
-      <c r="W188" s="20"/>
-      <c r="X188" s="20"/>
-      <c r="Y188" s="20"/>
-      <c r="Z188" s="20"/>
-      <c r="AA188" s="20"/>
-      <c r="AB188" s="20"/>
+      <c r="B188" s="1"/>
+      <c r="C188" s="73">
+        <f>INT($C$140)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D188" s="1"/>
+      <c r="E188" s="1"/>
+      <c r="F188" s="1"/>
+      <c r="G188" s="1"/>
+      <c r="H188" s="1"/>
+      <c r="I188" s="1"/>
+      <c r="J188" s="1"/>
+      <c r="K188" s="1"/>
+      <c r="L188" s="1"/>
+      <c r="M188" s="1"/>
+      <c r="N188" s="1"/>
+      <c r="O188" s="1"/>
+      <c r="P188" s="1"/>
+      <c r="Q188" s="1"/>
+      <c r="R188" s="1"/>
+      <c r="S188" s="1"/>
+      <c r="T188" s="1"/>
+      <c r="U188" s="1"/>
+      <c r="V188" s="1"/>
+      <c r="W188" s="1"/>
+      <c r="X188" s="1"/>
+      <c r="Y188" s="1"/>
+      <c r="Z188" s="1"/>
+      <c r="AA188" s="1"/>
+      <c r="AB188" s="1"/>
       <c r="AC188" s="1"/>
       <c r="AD188" s="1"/>
       <c r="AE188" s="1"/>
     </row>
-    <row r="189" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A189" s="1"/>
-      <c r="B189" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="C189" s="75">
-        <f>INT($C$191)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D189" s="14"/>
-      <c r="E189" s="14"/>
-      <c r="F189" s="14"/>
-      <c r="G189" s="14"/>
-      <c r="H189" s="14"/>
-      <c r="I189" s="14"/>
-      <c r="J189" s="14"/>
-      <c r="K189" s="14"/>
-      <c r="L189" s="14"/>
-      <c r="M189" s="14"/>
-      <c r="N189" s="14"/>
-      <c r="O189" s="14"/>
-      <c r="P189" s="14"/>
-      <c r="Q189" s="14"/>
-      <c r="R189" s="14"/>
-      <c r="S189" s="14"/>
-      <c r="T189" s="14"/>
-      <c r="U189" s="14"/>
-      <c r="V189" s="14"/>
-      <c r="W189" s="14"/>
-      <c r="X189" s="14"/>
-      <c r="Y189" s="14"/>
-      <c r="Z189" s="14"/>
-      <c r="AA189" s="14"/>
-      <c r="AB189" s="15"/>
+      <c r="B189" s="1"/>
+      <c r="C189" s="73">
+        <f>INT($C$193)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D189" s="1"/>
+      <c r="E189" s="1"/>
+      <c r="F189" s="1"/>
+      <c r="G189" s="1"/>
+      <c r="H189" s="1"/>
+      <c r="I189" s="1"/>
+      <c r="J189" s="1"/>
+      <c r="K189" s="1"/>
+      <c r="L189" s="1"/>
+      <c r="M189" s="1"/>
+      <c r="N189" s="1"/>
+      <c r="O189" s="1"/>
+      <c r="P189" s="1"/>
+      <c r="Q189" s="1"/>
+      <c r="R189" s="1"/>
+      <c r="S189" s="1"/>
+      <c r="T189" s="1"/>
+      <c r="U189" s="1"/>
+      <c r="V189" s="1"/>
+      <c r="W189" s="1"/>
+      <c r="X189" s="1"/>
+      <c r="Y189" s="1"/>
+      <c r="Z189" s="1"/>
+      <c r="AA189" s="1"/>
+      <c r="AB189" s="1"/>
       <c r="AC189" s="1"/>
       <c r="AD189" s="1"/>
       <c r="AE189" s="1"/>
     </row>
-    <row r="190" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:31" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A190" s="1"/>
-      <c r="B190" s="33"/>
-      <c r="C190" s="73">
-        <f>INT(MAX($C$199:$C$203))+1</f>
-        <v>5</v>
-      </c>
-      <c r="D190" s="3"/>
-      <c r="E190" s="3"/>
-      <c r="F190" s="3"/>
-      <c r="G190" s="3"/>
-      <c r="H190" s="27"/>
-      <c r="I190" s="27"/>
-      <c r="J190" s="27"/>
-      <c r="K190" s="27"/>
-      <c r="L190" s="27"/>
-      <c r="M190" s="27"/>
-      <c r="N190" s="27"/>
-      <c r="O190" s="27"/>
-      <c r="P190" s="27"/>
-      <c r="Q190" s="27"/>
-      <c r="R190" s="27"/>
-      <c r="S190" s="27"/>
-      <c r="T190" s="27"/>
-      <c r="U190" s="27"/>
-      <c r="V190" s="27"/>
-      <c r="W190" s="27"/>
-      <c r="X190" s="27"/>
-      <c r="Y190" s="27"/>
-      <c r="Z190" s="27"/>
-      <c r="AA190" s="3"/>
-      <c r="AB190" s="16"/>
+      <c r="B190" s="20"/>
+      <c r="C190" s="74">
+        <f>INT($C$193)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D190" s="20"/>
+      <c r="E190" s="20"/>
+      <c r="F190" s="20"/>
+      <c r="G190" s="20"/>
+      <c r="H190" s="20"/>
+      <c r="I190" s="20"/>
+      <c r="J190" s="20"/>
+      <c r="K190" s="20"/>
+      <c r="L190" s="20"/>
+      <c r="M190" s="20"/>
+      <c r="N190" s="20"/>
+      <c r="O190" s="20"/>
+      <c r="P190" s="20"/>
+      <c r="Q190" s="20"/>
+      <c r="R190" s="20"/>
+      <c r="S190" s="20"/>
+      <c r="T190" s="20"/>
+      <c r="U190" s="20"/>
+      <c r="V190" s="20"/>
+      <c r="W190" s="20"/>
+      <c r="X190" s="20"/>
+      <c r="Y190" s="20"/>
+      <c r="Z190" s="20"/>
+      <c r="AA190" s="20"/>
+      <c r="AB190" s="20"/>
       <c r="AC190" s="1"/>
       <c r="AD190" s="1"/>
       <c r="AE190" s="1"/>
     </row>
-    <row r="191" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1"/>
-      <c r="B191" s="33"/>
-      <c r="C191" s="73">
-        <v>1.02</v>
-      </c>
-      <c r="D191" s="21"/>
-      <c r="E191" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="F191" s="25"/>
-      <c r="G191" s="12"/>
-      <c r="H191" s="147" t="str">
-        <f>COUNTIFS($B$1:$B191, "«")&amp;" Feed Pool definitions"</f>
-        <v>6 Feed Pool definitions</v>
-      </c>
-      <c r="I191" s="6"/>
-      <c r="J191" s="6"/>
-      <c r="K191" s="6"/>
-      <c r="L191" s="6"/>
-      <c r="M191" s="6"/>
-      <c r="N191" s="6"/>
-      <c r="O191" s="6"/>
-      <c r="P191" s="6"/>
-      <c r="Q191" s="6"/>
-      <c r="R191" s="6"/>
-      <c r="S191" s="6"/>
-      <c r="T191" s="6"/>
-      <c r="U191" s="6"/>
-      <c r="V191" s="6"/>
-      <c r="W191" s="6"/>
-      <c r="X191" s="6"/>
-      <c r="Y191" s="6"/>
-      <c r="Z191" s="6"/>
-      <c r="AA191" s="10"/>
-      <c r="AB191" s="16"/>
+      <c r="B191" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C191" s="75">
+        <f>INT($C$193)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D191" s="14"/>
+      <c r="E191" s="14"/>
+      <c r="F191" s="14"/>
+      <c r="G191" s="14"/>
+      <c r="H191" s="14"/>
+      <c r="I191" s="14"/>
+      <c r="J191" s="14"/>
+      <c r="K191" s="14"/>
+      <c r="L191" s="14"/>
+      <c r="M191" s="14"/>
+      <c r="N191" s="14"/>
+      <c r="O191" s="14"/>
+      <c r="P191" s="14"/>
+      <c r="Q191" s="14"/>
+      <c r="R191" s="14"/>
+      <c r="S191" s="14"/>
+      <c r="T191" s="14"/>
+      <c r="U191" s="14"/>
+      <c r="V191" s="14"/>
+      <c r="W191" s="14"/>
+      <c r="X191" s="14"/>
+      <c r="Y191" s="14"/>
+      <c r="Z191" s="14"/>
+      <c r="AA191" s="14"/>
+      <c r="AB191" s="15"/>
       <c r="AC191" s="1"/>
       <c r="AD191" s="1"/>
       <c r="AE191" s="1"/>
     </row>
-    <row r="192" spans="1:31" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
       <c r="B192" s="33"/>
       <c r="C192" s="73">
-        <f>INT($C$191)+1.02</f>
-        <v>2.02</v>
-      </c>
-      <c r="D192" s="21"/>
-      <c r="E192" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="F192" s="28">
-        <v>1</v>
-      </c>
-      <c r="G192" s="13"/>
-      <c r="H192" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="I192" s="7"/>
-      <c r="J192" s="7"/>
-      <c r="K192" s="7"/>
-      <c r="L192" s="7"/>
-      <c r="M192" s="7"/>
-      <c r="N192" s="7"/>
-      <c r="O192" s="7"/>
-      <c r="P192" s="7"/>
-      <c r="Q192" s="7"/>
-      <c r="R192" s="7"/>
-      <c r="S192" s="7"/>
-      <c r="T192" s="7"/>
-      <c r="U192" s="7"/>
-      <c r="V192" s="7"/>
-      <c r="W192" s="7"/>
-      <c r="X192" s="7"/>
-      <c r="Y192" s="7"/>
-      <c r="Z192" s="7"/>
-      <c r="AA192" s="11"/>
+        <f>INT(MAX($C$201:$C$205))+1</f>
+        <v>5</v>
+      </c>
+      <c r="D192" s="3"/>
+      <c r="E192" s="3"/>
+      <c r="F192" s="3"/>
+      <c r="G192" s="3"/>
+      <c r="H192" s="27"/>
+      <c r="I192" s="27"/>
+      <c r="J192" s="27"/>
+      <c r="K192" s="27"/>
+      <c r="L192" s="27"/>
+      <c r="M192" s="27"/>
+      <c r="N192" s="27"/>
+      <c r="O192" s="27"/>
+      <c r="P192" s="27"/>
+      <c r="Q192" s="27"/>
+      <c r="R192" s="27"/>
+      <c r="S192" s="27"/>
+      <c r="T192" s="27"/>
+      <c r="U192" s="27"/>
+      <c r="V192" s="27"/>
+      <c r="W192" s="27"/>
+      <c r="X192" s="27"/>
+      <c r="Y192" s="27"/>
+      <c r="Z192" s="27"/>
+      <c r="AA192" s="3"/>
       <c r="AB192" s="16"/>
       <c r="AC192" s="1"/>
       <c r="AD192" s="1"/>
       <c r="AE192" s="1"/>
     </row>
-    <row r="193" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
       <c r="B193" s="33"/>
       <c r="C193" s="73">
-        <f>INT($C$191)+2.005</f>
-        <v>3.0049999999999999</v>
-      </c>
-      <c r="D193" s="3"/>
-      <c r="E193" s="3"/>
-      <c r="F193" s="3"/>
-      <c r="G193" s="3"/>
-      <c r="H193" s="3"/>
-      <c r="I193" s="3"/>
-      <c r="J193" s="3"/>
-      <c r="K193" s="3"/>
-      <c r="L193" s="3"/>
-      <c r="M193" s="3"/>
-      <c r="N193" s="3"/>
-      <c r="O193" s="3"/>
-      <c r="P193" s="3"/>
-      <c r="Q193" s="3"/>
-      <c r="R193" s="3"/>
-      <c r="S193" s="3"/>
-      <c r="T193" s="3"/>
-      <c r="U193" s="3"/>
-      <c r="V193" s="3"/>
-      <c r="W193" s="3"/>
-      <c r="X193" s="3"/>
-      <c r="Y193" s="3"/>
-      <c r="Z193" s="3"/>
-      <c r="AA193" s="3"/>
+        <v>1.02</v>
+      </c>
+      <c r="D193" s="21"/>
+      <c r="E193" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="F193" s="25"/>
+      <c r="G193" s="12"/>
+      <c r="H193" s="147" t="str">
+        <f>COUNTIFS($B$1:$B193, "«")&amp;" Feed Pool definitions"</f>
+        <v>6 Feed Pool definitions</v>
+      </c>
+      <c r="I193" s="6"/>
+      <c r="J193" s="6"/>
+      <c r="K193" s="6"/>
+      <c r="L193" s="6"/>
+      <c r="M193" s="6"/>
+      <c r="N193" s="6"/>
+      <c r="O193" s="6"/>
+      <c r="P193" s="6"/>
+      <c r="Q193" s="6"/>
+      <c r="R193" s="6"/>
+      <c r="S193" s="6"/>
+      <c r="T193" s="6"/>
+      <c r="U193" s="6"/>
+      <c r="V193" s="6"/>
+      <c r="W193" s="6"/>
+      <c r="X193" s="6"/>
+      <c r="Y193" s="6"/>
+      <c r="Z193" s="6"/>
+      <c r="AA193" s="10"/>
       <c r="AB193" s="16"/>
       <c r="AC193" s="1"/>
       <c r="AD193" s="1"/>
       <c r="AE193" s="1"/>
     </row>
-    <row r="194" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:31" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
       <c r="B194" s="33"/>
       <c r="C194" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D194" s="3"/>
-      <c r="E194" s="5"/>
-      <c r="F194" s="5"/>
-      <c r="G194" s="3"/>
-      <c r="H194" s="29"/>
-      <c r="I194" s="29"/>
-      <c r="J194" s="29"/>
-      <c r="K194" s="29"/>
-      <c r="L194" s="29"/>
-      <c r="M194" s="29"/>
-      <c r="N194" s="29"/>
-      <c r="O194" s="29"/>
-      <c r="P194" s="29"/>
-      <c r="Q194" s="29"/>
-      <c r="R194" s="29"/>
-      <c r="S194" s="29"/>
-      <c r="T194" s="29"/>
-      <c r="U194" s="29"/>
-      <c r="V194" s="29"/>
-      <c r="W194" s="29"/>
-      <c r="X194" s="29"/>
-      <c r="Y194" s="29"/>
-      <c r="Z194" s="29"/>
-      <c r="AA194" s="3"/>
+        <f>INT($C$193)+1.02</f>
+        <v>2.02</v>
+      </c>
+      <c r="D194" s="21"/>
+      <c r="E194" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F194" s="28">
+        <v>1</v>
+      </c>
+      <c r="G194" s="13"/>
+      <c r="H194" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="I194" s="7"/>
+      <c r="J194" s="7"/>
+      <c r="K194" s="7"/>
+      <c r="L194" s="7"/>
+      <c r="M194" s="7"/>
+      <c r="N194" s="7"/>
+      <c r="O194" s="7"/>
+      <c r="P194" s="7"/>
+      <c r="Q194" s="7"/>
+      <c r="R194" s="7"/>
+      <c r="S194" s="7"/>
+      <c r="T194" s="7"/>
+      <c r="U194" s="7"/>
+      <c r="V194" s="7"/>
+      <c r="W194" s="7"/>
+      <c r="X194" s="7"/>
+      <c r="Y194" s="7"/>
+      <c r="Z194" s="7"/>
+      <c r="AA194" s="11"/>
       <c r="AB194" s="16"/>
       <c r="AC194" s="1"/>
       <c r="AD194" s="1"/>
       <c r="AE194" s="1"/>
     </row>
-    <row r="195" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
       <c r="B195" s="33"/>
       <c r="C195" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
+        <f>INT($C$193)+2.005</f>
+        <v>3.0049999999999999</v>
       </c>
       <c r="D195" s="3"/>
-      <c r="E195" s="5"/>
-      <c r="F195" s="5"/>
+      <c r="E195" s="3"/>
+      <c r="F195" s="3"/>
       <c r="G195" s="3"/>
-      <c r="H195" s="29"/>
-      <c r="I195" s="29"/>
-      <c r="J195" s="29"/>
-      <c r="K195" s="29"/>
-      <c r="L195" s="29"/>
-      <c r="M195" s="29"/>
-      <c r="N195" s="29"/>
-      <c r="O195" s="29"/>
-      <c r="P195" s="29"/>
-      <c r="Q195" s="29"/>
-      <c r="R195" s="29"/>
-      <c r="S195" s="29"/>
-      <c r="T195" s="29"/>
-      <c r="U195" s="29"/>
-      <c r="V195" s="29"/>
-      <c r="W195" s="29"/>
-      <c r="X195" s="29"/>
-      <c r="Y195" s="29"/>
-      <c r="Z195" s="29"/>
+      <c r="H195" s="3"/>
+      <c r="I195" s="3"/>
+      <c r="J195" s="3"/>
+      <c r="K195" s="3"/>
+      <c r="L195" s="3"/>
+      <c r="M195" s="3"/>
+      <c r="N195" s="3"/>
+      <c r="O195" s="3"/>
+      <c r="P195" s="3"/>
+      <c r="Q195" s="3"/>
+      <c r="R195" s="3"/>
+      <c r="S195" s="3"/>
+      <c r="T195" s="3"/>
+      <c r="U195" s="3"/>
+      <c r="V195" s="3"/>
+      <c r="W195" s="3"/>
+      <c r="X195" s="3"/>
+      <c r="Y195" s="3"/>
+      <c r="Z195" s="3"/>
       <c r="AA195" s="3"/>
       <c r="AB195" s="16"/>
       <c r="AC195" s="1"/>
       <c r="AD195" s="1"/>
       <c r="AE195" s="1"/>
     </row>
-    <row r="196" spans="1:31" ht="9.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A196" s="1"/>
-      <c r="B196" s="33" t="s">
-        <v>20</v>
-      </c>
+      <c r="B196" s="33"/>
       <c r="C196" s="73">
-        <f>INT($C$191)+2.01</f>
-        <v>3.01</v>
+        <f>INT($C$193)+2</f>
+        <v>3</v>
       </c>
       <c r="D196" s="3"/>
-      <c r="E196" s="3"/>
-      <c r="F196" s="3"/>
+      <c r="E196" s="5"/>
+      <c r="F196" s="5"/>
       <c r="G196" s="3"/>
       <c r="H196" s="29"/>
       <c r="I196" s="29"/>
@@ -35461,220 +35629,222 @@
       <c r="AD196" s="1"/>
       <c r="AE196" s="1"/>
     </row>
-    <row r="197" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A197" s="1"/>
       <c r="B197" s="33"/>
       <c r="C197" s="73">
-        <f>C$190</f>
-        <v>5</v>
-      </c>
-      <c r="D197" s="4"/>
+        <f>INT($C$193)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D197" s="3"/>
       <c r="E197" s="5"/>
       <c r="F197" s="5"/>
-      <c r="G197" s="4"/>
-      <c r="H197" s="5"/>
-      <c r="I197" s="5"/>
-      <c r="J197" s="5"/>
-      <c r="K197" s="5"/>
-      <c r="L197" s="5"/>
-      <c r="M197" s="5"/>
-      <c r="N197" s="5"/>
-      <c r="O197" s="5"/>
-      <c r="P197" s="5"/>
-      <c r="Q197" s="5"/>
-      <c r="R197" s="5"/>
-      <c r="S197" s="5"/>
-      <c r="T197" s="5"/>
-      <c r="U197" s="5"/>
-      <c r="V197" s="5"/>
-      <c r="W197" s="5"/>
-      <c r="X197" s="5"/>
-      <c r="Y197" s="5"/>
-      <c r="Z197" s="5"/>
-      <c r="AA197" s="4"/>
+      <c r="G197" s="3"/>
+      <c r="H197" s="29"/>
+      <c r="I197" s="29"/>
+      <c r="J197" s="29"/>
+      <c r="K197" s="29"/>
+      <c r="L197" s="29"/>
+      <c r="M197" s="29"/>
+      <c r="N197" s="29"/>
+      <c r="O197" s="29"/>
+      <c r="P197" s="29"/>
+      <c r="Q197" s="29"/>
+      <c r="R197" s="29"/>
+      <c r="S197" s="29"/>
+      <c r="T197" s="29"/>
+      <c r="U197" s="29"/>
+      <c r="V197" s="29"/>
+      <c r="W197" s="29"/>
+      <c r="X197" s="29"/>
+      <c r="Y197" s="29"/>
+      <c r="Z197" s="29"/>
+      <c r="AA197" s="3"/>
       <c r="AB197" s="16"/>
       <c r="AC197" s="1"/>
       <c r="AD197" s="1"/>
       <c r="AE197" s="1"/>
     </row>
-    <row r="198" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:31" ht="9.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A198" s="1"/>
       <c r="B198" s="33" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C198" s="73">
-        <f>C$190</f>
-        <v>5</v>
-      </c>
-      <c r="D198" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
-      <c r="G198" s="4"/>
-      <c r="H198" s="5"/>
-      <c r="I198" s="5"/>
-      <c r="J198" s="5"/>
-      <c r="K198" s="5"/>
-      <c r="L198" s="5"/>
-      <c r="M198" s="5"/>
-      <c r="N198" s="5"/>
-      <c r="O198" s="5"/>
-      <c r="P198" s="5"/>
-      <c r="Q198" s="5"/>
-      <c r="R198" s="5"/>
-      <c r="S198" s="5"/>
-      <c r="T198" s="5"/>
-      <c r="U198" s="5"/>
-      <c r="V198" s="5"/>
-      <c r="W198" s="5"/>
-      <c r="X198" s="5"/>
-      <c r="Y198" s="5"/>
-      <c r="Z198" s="5"/>
-      <c r="AA198" s="4"/>
+        <f>INT($C$193)+2.01</f>
+        <v>3.01</v>
+      </c>
+      <c r="D198" s="3"/>
+      <c r="E198" s="3"/>
+      <c r="F198" s="3"/>
+      <c r="G198" s="3"/>
+      <c r="H198" s="29"/>
+      <c r="I198" s="29"/>
+      <c r="J198" s="29"/>
+      <c r="K198" s="29"/>
+      <c r="L198" s="29"/>
+      <c r="M198" s="29"/>
+      <c r="N198" s="29"/>
+      <c r="O198" s="29"/>
+      <c r="P198" s="29"/>
+      <c r="Q198" s="29"/>
+      <c r="R198" s="29"/>
+      <c r="S198" s="29"/>
+      <c r="T198" s="29"/>
+      <c r="U198" s="29"/>
+      <c r="V198" s="29"/>
+      <c r="W198" s="29"/>
+      <c r="X198" s="29"/>
+      <c r="Y198" s="29"/>
+      <c r="Z198" s="29"/>
+      <c r="AA198" s="3"/>
       <c r="AB198" s="16"/>
       <c r="AC198" s="1"/>
       <c r="AD198" s="1"/>
       <c r="AE198" s="1"/>
     </row>
-    <row r="199" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A199" s="1"/>
       <c r="B199" s="33"/>
       <c r="C199" s="73">
-        <f>INT($C$191)+2.005</f>
-        <v>3.0049999999999999</v>
-      </c>
-      <c r="D199" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E199" s="4"/>
-      <c r="F199" s="4"/>
+        <f>C$192</f>
+        <v>5</v>
+      </c>
+      <c r="D199" s="4"/>
+      <c r="E199" s="5"/>
+      <c r="F199" s="5"/>
       <c r="G199" s="4"/>
-      <c r="H199" s="58"/>
-      <c r="I199" s="58"/>
-      <c r="J199" s="58"/>
-      <c r="K199" s="58"/>
-      <c r="L199" s="58"/>
-      <c r="M199" s="58"/>
-      <c r="N199" s="58"/>
-      <c r="O199" s="58"/>
-      <c r="P199" s="58"/>
-      <c r="Q199" s="58"/>
-      <c r="R199" s="58"/>
-      <c r="S199" s="58"/>
-      <c r="T199" s="58"/>
-      <c r="U199" s="58"/>
-      <c r="V199" s="58"/>
-      <c r="W199" s="58"/>
-      <c r="X199" s="82"/>
-      <c r="Y199" s="82"/>
-      <c r="Z199" s="82"/>
+      <c r="H199" s="5"/>
+      <c r="I199" s="5"/>
+      <c r="J199" s="5"/>
+      <c r="K199" s="5"/>
+      <c r="L199" s="5"/>
+      <c r="M199" s="5"/>
+      <c r="N199" s="5"/>
+      <c r="O199" s="5"/>
+      <c r="P199" s="5"/>
+      <c r="Q199" s="5"/>
+      <c r="R199" s="5"/>
+      <c r="S199" s="5"/>
+      <c r="T199" s="5"/>
+      <c r="U199" s="5"/>
+      <c r="V199" s="5"/>
+      <c r="W199" s="5"/>
+      <c r="X199" s="5"/>
+      <c r="Y199" s="5"/>
+      <c r="Z199" s="5"/>
       <c r="AA199" s="4"/>
       <c r="AB199" s="16"/>
       <c r="AC199" s="1"/>
       <c r="AD199" s="1"/>
       <c r="AE199" s="1"/>
     </row>
-    <row r="200" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A200" s="1"/>
-      <c r="B200" s="33"/>
+      <c r="B200" s="33" t="s">
+        <v>19</v>
+      </c>
       <c r="C200" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D200" s="4"/>
+        <f>C$192</f>
+        <v>5</v>
+      </c>
+      <c r="D200" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
       <c r="G200" s="4"/>
-      <c r="H200" s="64" t="s">
-        <v>287</v>
-      </c>
-      <c r="I200" s="31">
-        <v>4</v>
-      </c>
-      <c r="J200" s="158" t="s">
-        <v>291</v>
-      </c>
-      <c r="K200" s="2"/>
-      <c r="L200" s="2"/>
-      <c r="M200" s="2"/>
-      <c r="N200" s="2"/>
-      <c r="O200" s="2"/>
-      <c r="P200" s="2"/>
-      <c r="Q200" s="2"/>
-      <c r="R200" s="2"/>
-      <c r="S200" s="2"/>
-      <c r="T200" s="2"/>
-      <c r="U200" s="2"/>
-      <c r="V200" s="2"/>
-      <c r="W200" s="2"/>
-      <c r="X200" s="2"/>
-      <c r="Y200" s="2"/>
-      <c r="Z200" s="2"/>
+      <c r="H200" s="5"/>
+      <c r="I200" s="5"/>
+      <c r="J200" s="5"/>
+      <c r="K200" s="5"/>
+      <c r="L200" s="5"/>
+      <c r="M200" s="5"/>
+      <c r="N200" s="5"/>
+      <c r="O200" s="5"/>
+      <c r="P200" s="5"/>
+      <c r="Q200" s="5"/>
+      <c r="R200" s="5"/>
+      <c r="S200" s="5"/>
+      <c r="T200" s="5"/>
+      <c r="U200" s="5"/>
+      <c r="V200" s="5"/>
+      <c r="W200" s="5"/>
+      <c r="X200" s="5"/>
+      <c r="Y200" s="5"/>
+      <c r="Z200" s="5"/>
       <c r="AA200" s="4"/>
       <c r="AB200" s="16"/>
       <c r="AC200" s="1"/>
       <c r="AD200" s="1"/>
       <c r="AE200" s="1"/>
     </row>
-    <row r="201" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A201" s="1"/>
       <c r="B201" s="33"/>
       <c r="C201" s="73">
-        <f>INT($C$191)+3</f>
-        <v>4</v>
-      </c>
-      <c r="D201" s="4"/>
-      <c r="E201" s="5"/>
-      <c r="F201" s="5"/>
+        <f>INT($C$193)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D201" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E201" s="4"/>
+      <c r="F201" s="4"/>
       <c r="G201" s="4"/>
-      <c r="H201" s="157"/>
-      <c r="I201" s="2"/>
-      <c r="J201" s="2"/>
-      <c r="K201" s="2"/>
-      <c r="L201" s="2"/>
-      <c r="M201" s="2"/>
-      <c r="N201" s="2"/>
-      <c r="O201" s="2"/>
-      <c r="P201" s="2"/>
-      <c r="Q201" s="2"/>
-      <c r="R201" s="2"/>
-      <c r="S201" s="2"/>
-      <c r="T201" s="2"/>
-      <c r="U201" s="2"/>
-      <c r="V201" s="2"/>
-      <c r="W201" s="2"/>
-      <c r="X201" s="2"/>
-      <c r="Y201" s="2"/>
-      <c r="Z201" s="2"/>
+      <c r="H201" s="58"/>
+      <c r="I201" s="58"/>
+      <c r="J201" s="58"/>
+      <c r="K201" s="58"/>
+      <c r="L201" s="58"/>
+      <c r="M201" s="58"/>
+      <c r="N201" s="58"/>
+      <c r="O201" s="58"/>
+      <c r="P201" s="58"/>
+      <c r="Q201" s="58"/>
+      <c r="R201" s="58"/>
+      <c r="S201" s="58"/>
+      <c r="T201" s="58"/>
+      <c r="U201" s="58"/>
+      <c r="V201" s="58"/>
+      <c r="W201" s="58"/>
+      <c r="X201" s="82"/>
+      <c r="Y201" s="82"/>
+      <c r="Z201" s="82"/>
       <c r="AA201" s="4"/>
       <c r="AB201" s="16"/>
       <c r="AC201" s="1"/>
       <c r="AD201" s="1"/>
       <c r="AE201" s="1"/>
     </row>
-    <row r="202" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A202" s="1"/>
       <c r="B202" s="33"/>
       <c r="C202" s="73">
-        <f>INT(C$191+3)</f>
-        <v>4</v>
+        <f>INT($C$193)+2</f>
+        <v>3</v>
       </c>
       <c r="D202" s="4"/>
       <c r="E202" s="5"/>
       <c r="F202" s="5"/>
       <c r="G202" s="4"/>
-      <c r="H202" s="148"/>
-      <c r="I202" s="148"/>
-      <c r="J202" s="148"/>
-      <c r="K202" s="148"/>
-      <c r="L202" s="148"/>
-      <c r="M202" s="148"/>
-      <c r="N202" s="148"/>
-      <c r="O202" s="148"/>
-      <c r="P202" s="148"/>
-      <c r="Q202" s="148"/>
-      <c r="R202" s="148"/>
+      <c r="H202" s="64" t="s">
+        <v>287</v>
+      </c>
+      <c r="I202" s="31">
+        <v>4</v>
+      </c>
+      <c r="J202" s="158" t="s">
+        <v>291</v>
+      </c>
+      <c r="K202" s="2"/>
+      <c r="L202" s="2"/>
+      <c r="M202" s="2"/>
+      <c r="N202" s="2"/>
+      <c r="O202" s="2"/>
+      <c r="P202" s="2"/>
+      <c r="Q202" s="2"/>
+      <c r="R202" s="2"/>
       <c r="S202" s="2"/>
       <c r="T202" s="2"/>
       <c r="U202" s="2"/>
@@ -35689,227 +35859,233 @@
       <c r="AD202" s="1"/>
       <c r="AE202" s="1"/>
     </row>
-    <row r="203" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
       <c r="B203" s="33"/>
       <c r="C203" s="73">
-        <f>INT($C$191)+3.005</f>
-        <v>4.0049999999999999</v>
+        <f>INT($C$193)+3</f>
+        <v>4</v>
       </c>
       <c r="D203" s="4"/>
-      <c r="E203" s="4"/>
-      <c r="F203" s="4"/>
+      <c r="E203" s="5"/>
+      <c r="F203" s="5"/>
       <c r="G203" s="4"/>
-      <c r="H203" s="4"/>
-      <c r="I203" s="4"/>
-      <c r="J203" s="4"/>
-      <c r="K203" s="4"/>
-      <c r="L203" s="4"/>
-      <c r="M203" s="4"/>
-      <c r="N203" s="4"/>
-      <c r="O203" s="4"/>
-      <c r="P203" s="4"/>
-      <c r="Q203" s="4"/>
-      <c r="R203" s="4"/>
-      <c r="S203" s="4"/>
-      <c r="T203" s="4"/>
-      <c r="U203" s="4"/>
-      <c r="V203" s="4"/>
-      <c r="W203" s="4"/>
-      <c r="X203" s="4"/>
-      <c r="Y203" s="4"/>
-      <c r="Z203" s="4"/>
-      <c r="AA203" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="H203" s="157"/>
+      <c r="I203" s="2"/>
+      <c r="J203" s="2"/>
+      <c r="K203" s="2"/>
+      <c r="L203" s="2"/>
+      <c r="M203" s="2"/>
+      <c r="N203" s="2"/>
+      <c r="O203" s="2"/>
+      <c r="P203" s="2"/>
+      <c r="Q203" s="2"/>
+      <c r="R203" s="2"/>
+      <c r="S203" s="2"/>
+      <c r="T203" s="2"/>
+      <c r="U203" s="2"/>
+      <c r="V203" s="2"/>
+      <c r="W203" s="2"/>
+      <c r="X203" s="2"/>
+      <c r="Y203" s="2"/>
+      <c r="Z203" s="2"/>
+      <c r="AA203" s="4"/>
       <c r="AB203" s="16"/>
       <c r="AC203" s="1"/>
       <c r="AD203" s="1"/>
       <c r="AE203" s="1"/>
     </row>
-    <row r="204" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A204" s="1"/>
       <c r="B204" s="33"/>
       <c r="C204" s="73">
-        <f>INT($C$191)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>INT(C$193+3)</f>
+        <v>4</v>
       </c>
       <c r="D204" s="4"/>
-      <c r="E204" s="4"/>
-      <c r="F204" s="4"/>
+      <c r="E204" s="5"/>
+      <c r="F204" s="5"/>
       <c r="G204" s="4"/>
-      <c r="H204" s="4"/>
-      <c r="I204" s="4"/>
-      <c r="J204" s="4"/>
-      <c r="K204" s="4"/>
-      <c r="L204" s="4"/>
-      <c r="M204" s="4"/>
-      <c r="N204" s="4"/>
-      <c r="O204" s="4"/>
-      <c r="P204" s="4"/>
-      <c r="Q204" s="4"/>
-      <c r="R204" s="4"/>
-      <c r="S204" s="4"/>
-      <c r="T204" s="4"/>
-      <c r="U204" s="4"/>
-      <c r="V204" s="4"/>
-      <c r="W204" s="4"/>
-      <c r="X204" s="4"/>
-      <c r="Y204" s="4"/>
-      <c r="Z204" s="4"/>
+      <c r="H204" s="148"/>
+      <c r="I204" s="148"/>
+      <c r="J204" s="148"/>
+      <c r="K204" s="148"/>
+      <c r="L204" s="148"/>
+      <c r="M204" s="148"/>
+      <c r="N204" s="148"/>
+      <c r="O204" s="148"/>
+      <c r="P204" s="148"/>
+      <c r="Q204" s="148"/>
+      <c r="R204" s="148"/>
+      <c r="S204" s="2"/>
+      <c r="T204" s="2"/>
+      <c r="U204" s="2"/>
+      <c r="V204" s="2"/>
+      <c r="W204" s="2"/>
+      <c r="X204" s="2"/>
+      <c r="Y204" s="2"/>
+      <c r="Z204" s="2"/>
       <c r="AA204" s="4"/>
       <c r="AB204" s="16"/>
       <c r="AC204" s="1"/>
       <c r="AD204" s="1"/>
       <c r="AE204" s="1"/>
     </row>
-    <row r="205" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
-      <c r="B205" s="35"/>
-      <c r="C205" s="76">
-        <f>INT($C$191)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D205" s="17"/>
-      <c r="E205" s="17"/>
-      <c r="F205" s="17"/>
-      <c r="G205" s="17"/>
-      <c r="H205" s="17"/>
-      <c r="I205" s="17"/>
-      <c r="J205" s="17"/>
-      <c r="K205" s="17"/>
-      <c r="L205" s="17"/>
-      <c r="M205" s="17"/>
-      <c r="N205" s="17"/>
-      <c r="O205" s="17"/>
-      <c r="P205" s="17"/>
-      <c r="Q205" s="17"/>
-      <c r="R205" s="17"/>
-      <c r="S205" s="17"/>
-      <c r="T205" s="17"/>
-      <c r="U205" s="17"/>
-      <c r="V205" s="17"/>
-      <c r="W205" s="17"/>
-      <c r="X205" s="17"/>
-      <c r="Y205" s="17"/>
-      <c r="Z205" s="17"/>
-      <c r="AA205" s="17"/>
-      <c r="AB205" s="18" t="s">
-        <v>1</v>
-      </c>
+      <c r="B205" s="33"/>
+      <c r="C205" s="73">
+        <f>INT($C$193)+3.005</f>
+        <v>4.0049999999999999</v>
+      </c>
+      <c r="D205" s="4"/>
+      <c r="E205" s="4"/>
+      <c r="F205" s="4"/>
+      <c r="G205" s="4"/>
+      <c r="H205" s="4"/>
+      <c r="I205" s="4"/>
+      <c r="J205" s="4"/>
+      <c r="K205" s="4"/>
+      <c r="L205" s="4"/>
+      <c r="M205" s="4"/>
+      <c r="N205" s="4"/>
+      <c r="O205" s="4"/>
+      <c r="P205" s="4"/>
+      <c r="Q205" s="4"/>
+      <c r="R205" s="4"/>
+      <c r="S205" s="4"/>
+      <c r="T205" s="4"/>
+      <c r="U205" s="4"/>
+      <c r="V205" s="4"/>
+      <c r="W205" s="4"/>
+      <c r="X205" s="4"/>
+      <c r="Y205" s="4"/>
+      <c r="Z205" s="4"/>
+      <c r="AA205" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB205" s="16"/>
       <c r="AC205" s="1"/>
       <c r="AD205" s="1"/>
       <c r="AE205" s="1"/>
     </row>
-    <row r="206" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A206" s="1"/>
-      <c r="B206" s="19"/>
-      <c r="C206" s="77">
-        <f>INT($C$191)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D206" s="19"/>
-      <c r="E206" s="19"/>
-      <c r="F206" s="19"/>
-      <c r="G206" s="19"/>
-      <c r="H206" s="19"/>
-      <c r="I206" s="19"/>
-      <c r="J206" s="19"/>
-      <c r="K206" s="19"/>
-      <c r="L206" s="19"/>
-      <c r="M206" s="19"/>
-      <c r="N206" s="19"/>
-      <c r="O206" s="19"/>
-      <c r="P206" s="19"/>
-      <c r="Q206" s="19"/>
-      <c r="R206" s="19"/>
-      <c r="S206" s="19"/>
-      <c r="T206" s="19"/>
-      <c r="U206" s="19"/>
-      <c r="V206" s="19"/>
-      <c r="W206" s="19"/>
-      <c r="X206" s="19"/>
-      <c r="Y206" s="19"/>
-      <c r="Z206" s="19"/>
-      <c r="AA206" s="19"/>
-      <c r="AB206" s="19"/>
+      <c r="B206" s="33"/>
+      <c r="C206" s="73">
+        <f>INT($C$193)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D206" s="4"/>
+      <c r="E206" s="4"/>
+      <c r="F206" s="4"/>
+      <c r="G206" s="4"/>
+      <c r="H206" s="4"/>
+      <c r="I206" s="4"/>
+      <c r="J206" s="4"/>
+      <c r="K206" s="4"/>
+      <c r="L206" s="4"/>
+      <c r="M206" s="4"/>
+      <c r="N206" s="4"/>
+      <c r="O206" s="4"/>
+      <c r="P206" s="4"/>
+      <c r="Q206" s="4"/>
+      <c r="R206" s="4"/>
+      <c r="S206" s="4"/>
+      <c r="T206" s="4"/>
+      <c r="U206" s="4"/>
+      <c r="V206" s="4"/>
+      <c r="W206" s="4"/>
+      <c r="X206" s="4"/>
+      <c r="Y206" s="4"/>
+      <c r="Z206" s="4"/>
+      <c r="AA206" s="4"/>
+      <c r="AB206" s="16"/>
       <c r="AC206" s="1"/>
       <c r="AD206" s="1"/>
       <c r="AE206" s="1"/>
     </row>
-    <row r="207" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A207" s="1"/>
-      <c r="B207" s="1"/>
-      <c r="C207" s="73">
-        <f>INT($C$191)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D207" s="1"/>
-      <c r="E207" s="1"/>
-      <c r="F207" s="1"/>
-      <c r="G207" s="1"/>
-      <c r="H207" s="1"/>
-      <c r="I207" s="1"/>
-      <c r="J207" s="1"/>
-      <c r="K207" s="1"/>
-      <c r="L207" s="1"/>
-      <c r="M207" s="1"/>
-      <c r="N207" s="1"/>
-      <c r="O207" s="1"/>
-      <c r="P207" s="1"/>
-      <c r="Q207" s="1"/>
-      <c r="R207" s="1"/>
-      <c r="S207" s="1"/>
-      <c r="T207" s="1"/>
-      <c r="U207" s="1"/>
-      <c r="V207" s="1"/>
-      <c r="W207" s="1"/>
-      <c r="X207" s="1"/>
-      <c r="Y207" s="1"/>
-      <c r="Z207" s="1"/>
-      <c r="AA207" s="1"/>
-      <c r="AB207" s="1"/>
+      <c r="B207" s="35"/>
+      <c r="C207" s="76">
+        <f>INT($C$193)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D207" s="17"/>
+      <c r="E207" s="17"/>
+      <c r="F207" s="17"/>
+      <c r="G207" s="17"/>
+      <c r="H207" s="17"/>
+      <c r="I207" s="17"/>
+      <c r="J207" s="17"/>
+      <c r="K207" s="17"/>
+      <c r="L207" s="17"/>
+      <c r="M207" s="17"/>
+      <c r="N207" s="17"/>
+      <c r="O207" s="17"/>
+      <c r="P207" s="17"/>
+      <c r="Q207" s="17"/>
+      <c r="R207" s="17"/>
+      <c r="S207" s="17"/>
+      <c r="T207" s="17"/>
+      <c r="U207" s="17"/>
+      <c r="V207" s="17"/>
+      <c r="W207" s="17"/>
+      <c r="X207" s="17"/>
+      <c r="Y207" s="17"/>
+      <c r="Z207" s="17"/>
+      <c r="AA207" s="17"/>
+      <c r="AB207" s="18" t="s">
+        <v>1</v>
+      </c>
       <c r="AC207" s="1"/>
       <c r="AD207" s="1"/>
       <c r="AE207" s="1"/>
     </row>
-    <row r="208" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1"/>
-      <c r="B208" s="1"/>
-      <c r="C208" s="66"/>
-      <c r="D208" s="1"/>
-      <c r="E208" s="1"/>
-      <c r="F208" s="1"/>
-      <c r="G208" s="1"/>
-      <c r="H208" s="1"/>
-      <c r="I208" s="1"/>
-      <c r="J208" s="1"/>
-      <c r="K208" s="1"/>
-      <c r="L208" s="1"/>
-      <c r="M208" s="1"/>
-      <c r="N208" s="1"/>
-      <c r="O208" s="1"/>
-      <c r="P208" s="1"/>
-      <c r="Q208" s="1"/>
-      <c r="R208" s="1"/>
-      <c r="S208" s="1"/>
-      <c r="T208" s="1"/>
-      <c r="U208" s="1"/>
-      <c r="V208" s="1"/>
-      <c r="W208" s="1"/>
-      <c r="X208" s="1"/>
-      <c r="Y208" s="1"/>
-      <c r="Z208" s="1"/>
-      <c r="AA208" s="1"/>
-      <c r="AB208" s="1"/>
+      <c r="B208" s="19"/>
+      <c r="C208" s="77">
+        <f>INT($C$193)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D208" s="19"/>
+      <c r="E208" s="19"/>
+      <c r="F208" s="19"/>
+      <c r="G208" s="19"/>
+      <c r="H208" s="19"/>
+      <c r="I208" s="19"/>
+      <c r="J208" s="19"/>
+      <c r="K208" s="19"/>
+      <c r="L208" s="19"/>
+      <c r="M208" s="19"/>
+      <c r="N208" s="19"/>
+      <c r="O208" s="19"/>
+      <c r="P208" s="19"/>
+      <c r="Q208" s="19"/>
+      <c r="R208" s="19"/>
+      <c r="S208" s="19"/>
+      <c r="T208" s="19"/>
+      <c r="U208" s="19"/>
+      <c r="V208" s="19"/>
+      <c r="W208" s="19"/>
+      <c r="X208" s="19"/>
+      <c r="Y208" s="19"/>
+      <c r="Z208" s="19"/>
+      <c r="AA208" s="19"/>
+      <c r="AB208" s="19"/>
       <c r="AC208" s="1"/>
       <c r="AD208" s="1"/>
       <c r="AE208" s="1"/>
     </row>
-    <row r="209" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
-      <c r="C209" s="66"/>
+      <c r="C209" s="73">
+        <f>INT($C$193)+2</f>
+        <v>3</v>
+      </c>
       <c r="D209" s="1"/>
       <c r="E209" s="1"/>
       <c r="F209" s="1"/>
@@ -36072,7 +36248,73 @@
       <c r="AE213" s="1"/>
     </row>
     <row r="214" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="C214" s="72" t="s">
+      <c r="A214" s="1"/>
+      <c r="B214" s="1"/>
+      <c r="C214" s="66"/>
+      <c r="D214" s="1"/>
+      <c r="E214" s="1"/>
+      <c r="F214" s="1"/>
+      <c r="G214" s="1"/>
+      <c r="H214" s="1"/>
+      <c r="I214" s="1"/>
+      <c r="J214" s="1"/>
+      <c r="K214" s="1"/>
+      <c r="L214" s="1"/>
+      <c r="M214" s="1"/>
+      <c r="N214" s="1"/>
+      <c r="O214" s="1"/>
+      <c r="P214" s="1"/>
+      <c r="Q214" s="1"/>
+      <c r="R214" s="1"/>
+      <c r="S214" s="1"/>
+      <c r="T214" s="1"/>
+      <c r="U214" s="1"/>
+      <c r="V214" s="1"/>
+      <c r="W214" s="1"/>
+      <c r="X214" s="1"/>
+      <c r="Y214" s="1"/>
+      <c r="Z214" s="1"/>
+      <c r="AA214" s="1"/>
+      <c r="AB214" s="1"/>
+      <c r="AC214" s="1"/>
+      <c r="AD214" s="1"/>
+      <c r="AE214" s="1"/>
+    </row>
+    <row r="215" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A215" s="1"/>
+      <c r="B215" s="1"/>
+      <c r="C215" s="66"/>
+      <c r="D215" s="1"/>
+      <c r="E215" s="1"/>
+      <c r="F215" s="1"/>
+      <c r="G215" s="1"/>
+      <c r="H215" s="1"/>
+      <c r="I215" s="1"/>
+      <c r="J215" s="1"/>
+      <c r="K215" s="1"/>
+      <c r="L215" s="1"/>
+      <c r="M215" s="1"/>
+      <c r="N215" s="1"/>
+      <c r="O215" s="1"/>
+      <c r="P215" s="1"/>
+      <c r="Q215" s="1"/>
+      <c r="R215" s="1"/>
+      <c r="S215" s="1"/>
+      <c r="T215" s="1"/>
+      <c r="U215" s="1"/>
+      <c r="V215" s="1"/>
+      <c r="W215" s="1"/>
+      <c r="X215" s="1"/>
+      <c r="Y215" s="1"/>
+      <c r="Z215" s="1"/>
+      <c r="AA215" s="1"/>
+      <c r="AB215" s="1"/>
+      <c r="AC215" s="1"/>
+      <c r="AD215" s="1"/>
+      <c r="AE215" s="1"/>
+    </row>
+    <row r="216" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="C216" s="72" t="s">
         <v>4</v>
       </c>
     </row>
@@ -36296,7 +36538,7 @@
       <c r="E7" s="176"/>
       <c r="F7" s="172"/>
       <c r="G7" s="178" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="H7" s="172"/>
       <c r="I7" s="172"/>
@@ -37745,23 +37987,23 @@
       <c r="I18" s="31">
         <v>1</v>
       </c>
-      <c r="J18" s="226" t="s">
+      <c r="J18" s="229" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="226"/>
-      <c r="L18" s="226"/>
-      <c r="M18" s="226"/>
-      <c r="N18" s="226"/>
-      <c r="O18" s="226"/>
-      <c r="P18" s="226"/>
-      <c r="Q18" s="226"/>
-      <c r="R18" s="226"/>
-      <c r="S18" s="226"/>
-      <c r="T18" s="226"/>
-      <c r="U18" s="226"/>
-      <c r="V18" s="226"/>
-      <c r="W18" s="226"/>
-      <c r="X18" s="226"/>
+      <c r="K18" s="229"/>
+      <c r="L18" s="229"/>
+      <c r="M18" s="229"/>
+      <c r="N18" s="229"/>
+      <c r="O18" s="229"/>
+      <c r="P18" s="229"/>
+      <c r="Q18" s="229"/>
+      <c r="R18" s="229"/>
+      <c r="S18" s="229"/>
+      <c r="T18" s="229"/>
+      <c r="U18" s="229"/>
+      <c r="V18" s="229"/>
+      <c r="W18" s="229"/>
+      <c r="X18" s="229"/>
       <c r="Y18" s="2"/>
       <c r="Z18" s="4"/>
       <c r="AA18" s="16"/>
@@ -37856,23 +38098,23 @@
       <c r="I21" s="23">
         <v>1</v>
       </c>
-      <c r="J21" s="224" t="s">
+      <c r="J21" s="227" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="225"/>
-      <c r="L21" s="225"/>
-      <c r="M21" s="225"/>
-      <c r="N21" s="225"/>
-      <c r="O21" s="225"/>
-      <c r="P21" s="225"/>
-      <c r="Q21" s="225"/>
-      <c r="R21" s="225"/>
-      <c r="S21" s="225"/>
-      <c r="T21" s="225"/>
-      <c r="U21" s="225"/>
-      <c r="V21" s="225"/>
-      <c r="W21" s="225"/>
-      <c r="X21" s="227"/>
+      <c r="K21" s="228"/>
+      <c r="L21" s="228"/>
+      <c r="M21" s="228"/>
+      <c r="N21" s="228"/>
+      <c r="O21" s="228"/>
+      <c r="P21" s="228"/>
+      <c r="Q21" s="228"/>
+      <c r="R21" s="228"/>
+      <c r="S21" s="228"/>
+      <c r="T21" s="228"/>
+      <c r="U21" s="228"/>
+      <c r="V21" s="228"/>
+      <c r="W21" s="228"/>
+      <c r="X21" s="230"/>
       <c r="Y21" s="2"/>
       <c r="Z21" s="4"/>
       <c r="AA21" s="16"/>

</xml_diff>

<commit_message>
Add output variables required for the genotype calibration. Add CS as a genotype trait in Structural
</commit_message>
<xml_diff>
--- a/ExcelInputs/Structural.xlsx
+++ b/ExcelInputs/Structural.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Models\AFO\ExcelInputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AA76A62-DC41-4944-96A6-32EDCF7AC316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8265F8A-6332-4AF9-945A-0E84E88507C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="28110" windowHeight="16440" tabRatio="678" activeTab="2" xr2:uid="{0842FB8C-088A-42F9-B075-24D0619777A0}"/>
   </bookViews>
@@ -92,7 +92,7 @@
     <definedName name="i_lag_organs">Stock!$I$70</definedName>
     <definedName name="i_lag_wool">Stock!$I$69</definedName>
     <definedName name="i_landuse_is_dual" localSheetId="0">General!$Q$79:$Q$110</definedName>
-    <definedName name="i_len_f">StructuralSA!$I$202</definedName>
+    <definedName name="i_len_f">StructuralSA!$I$203</definedName>
     <definedName name="i_len_l">Stock!$M$159</definedName>
     <definedName name="i_len_m">Stock!$L$159</definedName>
     <definedName name="i_len_planning_horizon" localSheetId="2">StructuralSA!$M$46</definedName>
@@ -2481,7 +2481,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H202" authorId="2" shapeId="0" xr:uid="{B39EFDC6-7ABB-4808-93B1-2819F2755236}">
+    <comment ref="H203" authorId="2" shapeId="0" xr:uid="{B39EFDC6-7ABB-4808-93B1-2819F2755236}">
       <text>
         <r>
           <rPr>
@@ -2544,7 +2544,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="451">
   <si>
     <t>Controls for this worksheet</t>
   </si>
@@ -4000,7 +4000,11 @@
     <t>Still to connect the FYI on model inversion traits</t>
   </si>
   <si>
-    <t>3May26: Change geneticist age stage named range to only include end and renamed to i_rev_age_stage_asbv
+    <t>cs</t>
+  </si>
+  <si>
+    <t>7Jul26: Add CS as a trait in the REV trait table and fix timing of some other traits (AWBE)
+3May26: Change geneticist age stage named range to only include end and renamed to i_rev_age_stage_asbv
 17Apr29: Added details for geneticist age stage to calculate the midpoint. Converted adults to a 364 day year step
 31Jan26: Removed the Cutoff levels for the NV pools that have been moved to Property.xlsx
 9Dec25: Added sl &amp; rr as REV traits. Expanded era and rr to be available at all individual adult age stages not just overall.
@@ -27132,7 +27136,7 @@
   <sheetPr codeName="Sheet3">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AE216"/>
+  <dimension ref="A1:AE217"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -27661,10 +27665,10 @@
         <v>16</v>
       </c>
       <c r="I13" s="126">
-        <v>46145.506140277801</v>
+        <v>46210.320505902797</v>
       </c>
       <c r="J13" s="224" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K13" s="225"/>
       <c r="L13" s="225"/>
@@ -32958,7 +32962,7 @@
       <c r="A139" s="1"/>
       <c r="B139" s="33"/>
       <c r="C139" s="73">
-        <f>INT(MAX($C$147:$C$184))+1</f>
+        <f>INT(MAX($C$147:$C$185))+1</f>
         <v>5</v>
       </c>
       <c r="D139" s="3"/>
@@ -34445,7 +34449,9 @@
       <c r="V170" s="2"/>
       <c r="W170" s="2"/>
       <c r="X170" s="2"/>
-      <c r="Y170" s="2"/>
+      <c r="Y170" s="56" t="s">
+        <v>422</v>
+      </c>
       <c r="Z170" s="2"/>
       <c r="AA170" s="4"/>
       <c r="AB170" s="16"/>
@@ -34614,11 +34620,11 @@
         <v>422</v>
       </c>
       <c r="S174" s="148"/>
-      <c r="T174" s="2"/>
-      <c r="U174" s="2"/>
-      <c r="V174" s="2"/>
-      <c r="W174" s="2"/>
-      <c r="X174" s="2"/>
+      <c r="T174" s="56"/>
+      <c r="U174" s="56"/>
+      <c r="V174" s="56"/>
+      <c r="W174" s="56"/>
+      <c r="X174" s="56"/>
       <c r="Y174" s="56" t="s">
         <v>422</v>
       </c>
@@ -34662,11 +34668,11 @@
         <v>422</v>
       </c>
       <c r="S175" s="148"/>
-      <c r="T175" s="2"/>
-      <c r="U175" s="2"/>
-      <c r="V175" s="2"/>
-      <c r="W175" s="2"/>
-      <c r="X175" s="2"/>
+      <c r="T175" s="56"/>
+      <c r="U175" s="56"/>
+      <c r="V175" s="56"/>
+      <c r="W175" s="56"/>
+      <c r="X175" s="56"/>
       <c r="Y175" s="56" t="s">
         <v>422</v>
       </c>
@@ -34710,21 +34716,11 @@
         <v>422</v>
       </c>
       <c r="S176" s="148"/>
-      <c r="T176" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="U176" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="V176" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="W176" s="56" t="s">
-        <v>422</v>
-      </c>
-      <c r="X176" s="56" t="s">
-        <v>422</v>
-      </c>
+      <c r="T176" s="56"/>
+      <c r="U176" s="56"/>
+      <c r="V176" s="56"/>
+      <c r="W176" s="56"/>
+      <c r="X176" s="56"/>
       <c r="Y176" s="56" t="s">
         <v>422</v>
       </c>
@@ -35110,85 +35106,109 @@
       <c r="K183" s="148"/>
       <c r="L183" s="148"/>
       <c r="M183" s="148"/>
-      <c r="N183" s="216" t="s">
+      <c r="N183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="O183" s="215"/>
-      <c r="P183" s="215"/>
-      <c r="Q183" s="215"/>
-      <c r="R183" s="216" t="s">
+      <c r="O183" s="148"/>
+      <c r="P183" s="148"/>
+      <c r="Q183" s="56"/>
+      <c r="R183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="S183" s="215"/>
-      <c r="T183" s="216" t="s">
+      <c r="S183" s="56"/>
+      <c r="T183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="U183" s="216" t="s">
+      <c r="U183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="V183" s="216" t="s">
+      <c r="V183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="W183" s="216" t="s">
+      <c r="W183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="X183" s="216" t="s">
+      <c r="X183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Y183" s="216" t="s">
+      <c r="Y183" s="56" t="s">
         <v>422</v>
       </c>
-      <c r="Z183" s="216"/>
+      <c r="Z183" s="56"/>
       <c r="AA183" s="4"/>
       <c r="AB183" s="16"/>
       <c r="AC183" s="1"/>
       <c r="AD183" s="1"/>
       <c r="AE183" s="1"/>
     </row>
-    <row r="184" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A184" s="1"/>
       <c r="B184" s="33"/>
       <c r="C184" s="73">
-        <f>INT($C$140)+3.005</f>
-        <v>4.0049999999999999</v>
+        <f>INT(C$140+3)</f>
+        <v>4</v>
       </c>
       <c r="D184" s="4"/>
-      <c r="E184" s="4"/>
-      <c r="F184" s="4"/>
+      <c r="E184" s="5">
+        <v>20</v>
+      </c>
+      <c r="F184" s="5"/>
       <c r="G184" s="4"/>
-      <c r="H184" s="4"/>
-      <c r="I184" s="4"/>
-      <c r="J184" s="4"/>
-      <c r="K184" s="4"/>
-      <c r="L184" s="4"/>
-      <c r="M184" s="4"/>
-      <c r="N184" s="4"/>
-      <c r="O184" s="4"/>
-      <c r="P184" s="4"/>
-      <c r="Q184" s="4"/>
-      <c r="R184" s="4"/>
-      <c r="S184" s="4"/>
-      <c r="T184" s="4"/>
-      <c r="U184" s="4"/>
-      <c r="V184" s="4"/>
-      <c r="W184" s="4"/>
-      <c r="X184" s="4"/>
-      <c r="Y184" s="4"/>
-      <c r="Z184" s="4"/>
-      <c r="AA184" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="H184" s="31" t="s">
+        <v>449</v>
+      </c>
+      <c r="I184" s="31">
+        <v>0</v>
+      </c>
+      <c r="J184" s="148"/>
+      <c r="K184" s="148"/>
+      <c r="L184" s="148"/>
+      <c r="M184" s="148"/>
+      <c r="N184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="O184" s="215"/>
+      <c r="P184" s="215"/>
+      <c r="Q184" s="215" t="s">
+        <v>422</v>
+      </c>
+      <c r="R184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="S184" s="215" t="s">
+        <v>422</v>
+      </c>
+      <c r="T184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="U184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="V184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="W184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="X184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="Y184" s="216" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z184" s="216"/>
+      <c r="AA184" s="4"/>
       <c r="AB184" s="16"/>
       <c r="AC184" s="1"/>
       <c r="AD184" s="1"/>
       <c r="AE184" s="1"/>
     </row>
-    <row r="185" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A185" s="1"/>
       <c r="B185" s="33"/>
       <c r="C185" s="73">
-        <f>INT($C$140)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>INT($C$140)+3.005</f>
+        <v>4.0049999999999999</v>
       </c>
       <c r="D185" s="4"/>
       <c r="E185" s="4"/>
@@ -35213,118 +35233,120 @@
       <c r="X185" s="4"/>
       <c r="Y185" s="4"/>
       <c r="Z185" s="4"/>
-      <c r="AA185" s="4"/>
+      <c r="AA185" s="4" t="s">
+        <v>3</v>
+      </c>
       <c r="AB185" s="16"/>
       <c r="AC185" s="1"/>
       <c r="AD185" s="1"/>
       <c r="AE185" s="1"/>
     </row>
-    <row r="186" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A186" s="1"/>
-      <c r="B186" s="35"/>
-      <c r="C186" s="76">
-        <f>INT($C$140)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D186" s="17"/>
-      <c r="E186" s="17"/>
-      <c r="F186" s="17"/>
-      <c r="G186" s="17"/>
-      <c r="H186" s="17"/>
-      <c r="I186" s="17"/>
-      <c r="J186" s="17"/>
-      <c r="K186" s="17"/>
-      <c r="L186" s="17"/>
-      <c r="M186" s="17"/>
-      <c r="N186" s="17"/>
-      <c r="O186" s="17"/>
-      <c r="P186" s="17"/>
-      <c r="Q186" s="17"/>
-      <c r="R186" s="17"/>
-      <c r="S186" s="17"/>
-      <c r="T186" s="17"/>
-      <c r="U186" s="17"/>
-      <c r="V186" s="17"/>
-      <c r="W186" s="17"/>
-      <c r="X186" s="17"/>
-      <c r="Y186" s="17"/>
-      <c r="Z186" s="17"/>
-      <c r="AA186" s="17"/>
-      <c r="AB186" s="18" t="s">
-        <v>1</v>
-      </c>
+      <c r="B186" s="33"/>
+      <c r="C186" s="73">
+        <f>INT($C$140)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D186" s="4"/>
+      <c r="E186" s="4"/>
+      <c r="F186" s="4"/>
+      <c r="G186" s="4"/>
+      <c r="H186" s="4"/>
+      <c r="I186" s="4"/>
+      <c r="J186" s="4"/>
+      <c r="K186" s="4"/>
+      <c r="L186" s="4"/>
+      <c r="M186" s="4"/>
+      <c r="N186" s="4"/>
+      <c r="O186" s="4"/>
+      <c r="P186" s="4"/>
+      <c r="Q186" s="4"/>
+      <c r="R186" s="4"/>
+      <c r="S186" s="4"/>
+      <c r="T186" s="4"/>
+      <c r="U186" s="4"/>
+      <c r="V186" s="4"/>
+      <c r="W186" s="4"/>
+      <c r="X186" s="4"/>
+      <c r="Y186" s="4"/>
+      <c r="Z186" s="4"/>
+      <c r="AA186" s="4"/>
+      <c r="AB186" s="16"/>
       <c r="AC186" s="1"/>
       <c r="AD186" s="1"/>
       <c r="AE186" s="1"/>
     </row>
-    <row r="187" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1"/>
-      <c r="B187" s="19"/>
-      <c r="C187" s="77">
-        <f>INT($C$140)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D187" s="19"/>
-      <c r="E187" s="19"/>
-      <c r="F187" s="19"/>
-      <c r="G187" s="19"/>
-      <c r="H187" s="19"/>
-      <c r="I187" s="19"/>
-      <c r="J187" s="19"/>
-      <c r="K187" s="19"/>
-      <c r="L187" s="19"/>
-      <c r="M187" s="19"/>
-      <c r="N187" s="19"/>
-      <c r="O187" s="19"/>
-      <c r="P187" s="19"/>
-      <c r="Q187" s="19"/>
-      <c r="R187" s="19"/>
-      <c r="S187" s="19"/>
-      <c r="T187" s="19"/>
-      <c r="U187" s="19"/>
-      <c r="V187" s="19"/>
-      <c r="W187" s="19"/>
-      <c r="X187" s="19"/>
-      <c r="Y187" s="19"/>
-      <c r="Z187" s="19"/>
-      <c r="AA187" s="19"/>
-      <c r="AB187" s="19"/>
+      <c r="B187" s="35"/>
+      <c r="C187" s="76">
+        <f>INT($C$140)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D187" s="17"/>
+      <c r="E187" s="17"/>
+      <c r="F187" s="17"/>
+      <c r="G187" s="17"/>
+      <c r="H187" s="17"/>
+      <c r="I187" s="17"/>
+      <c r="J187" s="17"/>
+      <c r="K187" s="17"/>
+      <c r="L187" s="17"/>
+      <c r="M187" s="17"/>
+      <c r="N187" s="17"/>
+      <c r="O187" s="17"/>
+      <c r="P187" s="17"/>
+      <c r="Q187" s="17"/>
+      <c r="R187" s="17"/>
+      <c r="S187" s="17"/>
+      <c r="T187" s="17"/>
+      <c r="U187" s="17"/>
+      <c r="V187" s="17"/>
+      <c r="W187" s="17"/>
+      <c r="X187" s="17"/>
+      <c r="Y187" s="17"/>
+      <c r="Z187" s="17"/>
+      <c r="AA187" s="17"/>
+      <c r="AB187" s="18" t="s">
+        <v>1</v>
+      </c>
       <c r="AC187" s="1"/>
       <c r="AD187" s="1"/>
       <c r="AE187" s="1"/>
     </row>
-    <row r="188" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1"/>
-      <c r="B188" s="1"/>
-      <c r="C188" s="73">
-        <f>INT($C$140)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D188" s="1"/>
-      <c r="E188" s="1"/>
-      <c r="F188" s="1"/>
-      <c r="G188" s="1"/>
-      <c r="H188" s="1"/>
-      <c r="I188" s="1"/>
-      <c r="J188" s="1"/>
-      <c r="K188" s="1"/>
-      <c r="L188" s="1"/>
-      <c r="M188" s="1"/>
-      <c r="N188" s="1"/>
-      <c r="O188" s="1"/>
-      <c r="P188" s="1"/>
-      <c r="Q188" s="1"/>
-      <c r="R188" s="1"/>
-      <c r="S188" s="1"/>
-      <c r="T188" s="1"/>
-      <c r="U188" s="1"/>
-      <c r="V188" s="1"/>
-      <c r="W188" s="1"/>
-      <c r="X188" s="1"/>
-      <c r="Y188" s="1"/>
-      <c r="Z188" s="1"/>
-      <c r="AA188" s="1"/>
-      <c r="AB188" s="1"/>
+      <c r="B188" s="19"/>
+      <c r="C188" s="77">
+        <f>INT($C$140)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D188" s="19"/>
+      <c r="E188" s="19"/>
+      <c r="F188" s="19"/>
+      <c r="G188" s="19"/>
+      <c r="H188" s="19"/>
+      <c r="I188" s="19"/>
+      <c r="J188" s="19"/>
+      <c r="K188" s="19"/>
+      <c r="L188" s="19"/>
+      <c r="M188" s="19"/>
+      <c r="N188" s="19"/>
+      <c r="O188" s="19"/>
+      <c r="P188" s="19"/>
+      <c r="Q188" s="19"/>
+      <c r="R188" s="19"/>
+      <c r="S188" s="19"/>
+      <c r="T188" s="19"/>
+      <c r="U188" s="19"/>
+      <c r="V188" s="19"/>
+      <c r="W188" s="19"/>
+      <c r="X188" s="19"/>
+      <c r="Y188" s="19"/>
+      <c r="Z188" s="19"/>
+      <c r="AA188" s="19"/>
+      <c r="AB188" s="19"/>
       <c r="AC188" s="1"/>
       <c r="AD188" s="1"/>
       <c r="AE188" s="1"/>
@@ -35333,7 +35355,7 @@
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="73">
-        <f>INT($C$193)+2</f>
+        <f>INT($C$140)+2</f>
         <v>3</v>
       </c>
       <c r="D189" s="1"/>
@@ -35365,264 +35387,264 @@
       <c r="AD189" s="1"/>
       <c r="AE189" s="1"/>
     </row>
-    <row r="190" spans="1:31" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A190" s="1"/>
-      <c r="B190" s="20"/>
-      <c r="C190" s="74">
-        <f>INT($C$193)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D190" s="20"/>
-      <c r="E190" s="20"/>
-      <c r="F190" s="20"/>
-      <c r="G190" s="20"/>
-      <c r="H190" s="20"/>
-      <c r="I190" s="20"/>
-      <c r="J190" s="20"/>
-      <c r="K190" s="20"/>
-      <c r="L190" s="20"/>
-      <c r="M190" s="20"/>
-      <c r="N190" s="20"/>
-      <c r="O190" s="20"/>
-      <c r="P190" s="20"/>
-      <c r="Q190" s="20"/>
-      <c r="R190" s="20"/>
-      <c r="S190" s="20"/>
-      <c r="T190" s="20"/>
-      <c r="U190" s="20"/>
-      <c r="V190" s="20"/>
-      <c r="W190" s="20"/>
-      <c r="X190" s="20"/>
-      <c r="Y190" s="20"/>
-      <c r="Z190" s="20"/>
-      <c r="AA190" s="20"/>
-      <c r="AB190" s="20"/>
+      <c r="B190" s="1"/>
+      <c r="C190" s="73">
+        <f>INT($C$194)+2</f>
+        <v>3</v>
+      </c>
+      <c r="D190" s="1"/>
+      <c r="E190" s="1"/>
+      <c r="F190" s="1"/>
+      <c r="G190" s="1"/>
+      <c r="H190" s="1"/>
+      <c r="I190" s="1"/>
+      <c r="J190" s="1"/>
+      <c r="K190" s="1"/>
+      <c r="L190" s="1"/>
+      <c r="M190" s="1"/>
+      <c r="N190" s="1"/>
+      <c r="O190" s="1"/>
+      <c r="P190" s="1"/>
+      <c r="Q190" s="1"/>
+      <c r="R190" s="1"/>
+      <c r="S190" s="1"/>
+      <c r="T190" s="1"/>
+      <c r="U190" s="1"/>
+      <c r="V190" s="1"/>
+      <c r="W190" s="1"/>
+      <c r="X190" s="1"/>
+      <c r="Y190" s="1"/>
+      <c r="Z190" s="1"/>
+      <c r="AA190" s="1"/>
+      <c r="AB190" s="1"/>
       <c r="AC190" s="1"/>
       <c r="AD190" s="1"/>
       <c r="AE190" s="1"/>
     </row>
-    <row r="191" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:31" ht="5.0999999999999996" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A191" s="1"/>
-      <c r="B191" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="C191" s="75">
-        <f>INT($C$193)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D191" s="14"/>
-      <c r="E191" s="14"/>
-      <c r="F191" s="14"/>
-      <c r="G191" s="14"/>
-      <c r="H191" s="14"/>
-      <c r="I191" s="14"/>
-      <c r="J191" s="14"/>
-      <c r="K191" s="14"/>
-      <c r="L191" s="14"/>
-      <c r="M191" s="14"/>
-      <c r="N191" s="14"/>
-      <c r="O191" s="14"/>
-      <c r="P191" s="14"/>
-      <c r="Q191" s="14"/>
-      <c r="R191" s="14"/>
-      <c r="S191" s="14"/>
-      <c r="T191" s="14"/>
-      <c r="U191" s="14"/>
-      <c r="V191" s="14"/>
-      <c r="W191" s="14"/>
-      <c r="X191" s="14"/>
-      <c r="Y191" s="14"/>
-      <c r="Z191" s="14"/>
-      <c r="AA191" s="14"/>
-      <c r="AB191" s="15"/>
+      <c r="B191" s="20"/>
+      <c r="C191" s="74">
+        <f>INT($C$194)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D191" s="20"/>
+      <c r="E191" s="20"/>
+      <c r="F191" s="20"/>
+      <c r="G191" s="20"/>
+      <c r="H191" s="20"/>
+      <c r="I191" s="20"/>
+      <c r="J191" s="20"/>
+      <c r="K191" s="20"/>
+      <c r="L191" s="20"/>
+      <c r="M191" s="20"/>
+      <c r="N191" s="20"/>
+      <c r="O191" s="20"/>
+      <c r="P191" s="20"/>
+      <c r="Q191" s="20"/>
+      <c r="R191" s="20"/>
+      <c r="S191" s="20"/>
+      <c r="T191" s="20"/>
+      <c r="U191" s="20"/>
+      <c r="V191" s="20"/>
+      <c r="W191" s="20"/>
+      <c r="X191" s="20"/>
+      <c r="Y191" s="20"/>
+      <c r="Z191" s="20"/>
+      <c r="AA191" s="20"/>
+      <c r="AB191" s="20"/>
       <c r="AC191" s="1"/>
       <c r="AD191" s="1"/>
       <c r="AE191" s="1"/>
     </row>
-    <row r="192" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1"/>
-      <c r="B192" s="33"/>
-      <c r="C192" s="73">
-        <f>INT(MAX($C$201:$C$205))+1</f>
-        <v>5</v>
-      </c>
-      <c r="D192" s="3"/>
-      <c r="E192" s="3"/>
-      <c r="F192" s="3"/>
-      <c r="G192" s="3"/>
-      <c r="H192" s="27"/>
-      <c r="I192" s="27"/>
-      <c r="J192" s="27"/>
-      <c r="K192" s="27"/>
-      <c r="L192" s="27"/>
-      <c r="M192" s="27"/>
-      <c r="N192" s="27"/>
-      <c r="O192" s="27"/>
-      <c r="P192" s="27"/>
-      <c r="Q192" s="27"/>
-      <c r="R192" s="27"/>
-      <c r="S192" s="27"/>
-      <c r="T192" s="27"/>
-      <c r="U192" s="27"/>
-      <c r="V192" s="27"/>
-      <c r="W192" s="27"/>
-      <c r="X192" s="27"/>
-      <c r="Y192" s="27"/>
-      <c r="Z192" s="27"/>
-      <c r="AA192" s="3"/>
-      <c r="AB192" s="16"/>
+      <c r="B192" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C192" s="75">
+        <f>INT($C$194)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D192" s="14"/>
+      <c r="E192" s="14"/>
+      <c r="F192" s="14"/>
+      <c r="G192" s="14"/>
+      <c r="H192" s="14"/>
+      <c r="I192" s="14"/>
+      <c r="J192" s="14"/>
+      <c r="K192" s="14"/>
+      <c r="L192" s="14"/>
+      <c r="M192" s="14"/>
+      <c r="N192" s="14"/>
+      <c r="O192" s="14"/>
+      <c r="P192" s="14"/>
+      <c r="Q192" s="14"/>
+      <c r="R192" s="14"/>
+      <c r="S192" s="14"/>
+      <c r="T192" s="14"/>
+      <c r="U192" s="14"/>
+      <c r="V192" s="14"/>
+      <c r="W192" s="14"/>
+      <c r="X192" s="14"/>
+      <c r="Y192" s="14"/>
+      <c r="Z192" s="14"/>
+      <c r="AA192" s="14"/>
+      <c r="AB192" s="15"/>
       <c r="AC192" s="1"/>
       <c r="AD192" s="1"/>
       <c r="AE192" s="1"/>
     </row>
-    <row r="193" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A193" s="1"/>
       <c r="B193" s="33"/>
       <c r="C193" s="73">
-        <v>1.02</v>
-      </c>
-      <c r="D193" s="21"/>
-      <c r="E193" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="F193" s="25"/>
-      <c r="G193" s="12"/>
-      <c r="H193" s="147" t="str">
-        <f>COUNTIFS($B$1:$B193, "«")&amp;" Feed Pool definitions"</f>
-        <v>6 Feed Pool definitions</v>
-      </c>
-      <c r="I193" s="6"/>
-      <c r="J193" s="6"/>
-      <c r="K193" s="6"/>
-      <c r="L193" s="6"/>
-      <c r="M193" s="6"/>
-      <c r="N193" s="6"/>
-      <c r="O193" s="6"/>
-      <c r="P193" s="6"/>
-      <c r="Q193" s="6"/>
-      <c r="R193" s="6"/>
-      <c r="S193" s="6"/>
-      <c r="T193" s="6"/>
-      <c r="U193" s="6"/>
-      <c r="V193" s="6"/>
-      <c r="W193" s="6"/>
-      <c r="X193" s="6"/>
-      <c r="Y193" s="6"/>
-      <c r="Z193" s="6"/>
-      <c r="AA193" s="10"/>
+        <f>INT(MAX($C$202:$C$206))+1</f>
+        <v>5</v>
+      </c>
+      <c r="D193" s="3"/>
+      <c r="E193" s="3"/>
+      <c r="F193" s="3"/>
+      <c r="G193" s="3"/>
+      <c r="H193" s="27"/>
+      <c r="I193" s="27"/>
+      <c r="J193" s="27"/>
+      <c r="K193" s="27"/>
+      <c r="L193" s="27"/>
+      <c r="M193" s="27"/>
+      <c r="N193" s="27"/>
+      <c r="O193" s="27"/>
+      <c r="P193" s="27"/>
+      <c r="Q193" s="27"/>
+      <c r="R193" s="27"/>
+      <c r="S193" s="27"/>
+      <c r="T193" s="27"/>
+      <c r="U193" s="27"/>
+      <c r="V193" s="27"/>
+      <c r="W193" s="27"/>
+      <c r="X193" s="27"/>
+      <c r="Y193" s="27"/>
+      <c r="Z193" s="27"/>
+      <c r="AA193" s="3"/>
       <c r="AB193" s="16"/>
       <c r="AC193" s="1"/>
       <c r="AD193" s="1"/>
       <c r="AE193" s="1"/>
     </row>
-    <row r="194" spans="1:31" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A194" s="1"/>
       <c r="B194" s="33"/>
       <c r="C194" s="73">
-        <f>INT($C$193)+1.02</f>
-        <v>2.02</v>
+        <v>1.02</v>
       </c>
       <c r="D194" s="21"/>
       <c r="E194" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="F194" s="28">
-        <v>1</v>
-      </c>
-      <c r="G194" s="13"/>
-      <c r="H194" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="I194" s="7"/>
-      <c r="J194" s="7"/>
-      <c r="K194" s="7"/>
-      <c r="L194" s="7"/>
-      <c r="M194" s="7"/>
-      <c r="N194" s="7"/>
-      <c r="O194" s="7"/>
-      <c r="P194" s="7"/>
-      <c r="Q194" s="7"/>
-      <c r="R194" s="7"/>
-      <c r="S194" s="7"/>
-      <c r="T194" s="7"/>
-      <c r="U194" s="7"/>
-      <c r="V194" s="7"/>
-      <c r="W194" s="7"/>
-      <c r="X194" s="7"/>
-      <c r="Y194" s="7"/>
-      <c r="Z194" s="7"/>
-      <c r="AA194" s="11"/>
+        <v>6</v>
+      </c>
+      <c r="F194" s="25"/>
+      <c r="G194" s="12"/>
+      <c r="H194" s="147" t="str">
+        <f>COUNTIFS($B$1:$B194, "«")&amp;" Feed Pool definitions"</f>
+        <v>6 Feed Pool definitions</v>
+      </c>
+      <c r="I194" s="6"/>
+      <c r="J194" s="6"/>
+      <c r="K194" s="6"/>
+      <c r="L194" s="6"/>
+      <c r="M194" s="6"/>
+      <c r="N194" s="6"/>
+      <c r="O194" s="6"/>
+      <c r="P194" s="6"/>
+      <c r="Q194" s="6"/>
+      <c r="R194" s="6"/>
+      <c r="S194" s="6"/>
+      <c r="T194" s="6"/>
+      <c r="U194" s="6"/>
+      <c r="V194" s="6"/>
+      <c r="W194" s="6"/>
+      <c r="X194" s="6"/>
+      <c r="Y194" s="6"/>
+      <c r="Z194" s="6"/>
+      <c r="AA194" s="10"/>
       <c r="AB194" s="16"/>
       <c r="AC194" s="1"/>
       <c r="AD194" s="1"/>
       <c r="AE194" s="1"/>
     </row>
-    <row r="195" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:31" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
       <c r="B195" s="33"/>
       <c r="C195" s="73">
-        <f>INT($C$193)+2.005</f>
-        <v>3.0049999999999999</v>
-      </c>
-      <c r="D195" s="3"/>
-      <c r="E195" s="3"/>
-      <c r="F195" s="3"/>
-      <c r="G195" s="3"/>
-      <c r="H195" s="3"/>
-      <c r="I195" s="3"/>
-      <c r="J195" s="3"/>
-      <c r="K195" s="3"/>
-      <c r="L195" s="3"/>
-      <c r="M195" s="3"/>
-      <c r="N195" s="3"/>
-      <c r="O195" s="3"/>
-      <c r="P195" s="3"/>
-      <c r="Q195" s="3"/>
-      <c r="R195" s="3"/>
-      <c r="S195" s="3"/>
-      <c r="T195" s="3"/>
-      <c r="U195" s="3"/>
-      <c r="V195" s="3"/>
-      <c r="W195" s="3"/>
-      <c r="X195" s="3"/>
-      <c r="Y195" s="3"/>
-      <c r="Z195" s="3"/>
-      <c r="AA195" s="3"/>
+        <f>INT($C$194)+1.02</f>
+        <v>2.02</v>
+      </c>
+      <c r="D195" s="21"/>
+      <c r="E195" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F195" s="28">
+        <v>1</v>
+      </c>
+      <c r="G195" s="13"/>
+      <c r="H195" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="I195" s="7"/>
+      <c r="J195" s="7"/>
+      <c r="K195" s="7"/>
+      <c r="L195" s="7"/>
+      <c r="M195" s="7"/>
+      <c r="N195" s="7"/>
+      <c r="O195" s="7"/>
+      <c r="P195" s="7"/>
+      <c r="Q195" s="7"/>
+      <c r="R195" s="7"/>
+      <c r="S195" s="7"/>
+      <c r="T195" s="7"/>
+      <c r="U195" s="7"/>
+      <c r="V195" s="7"/>
+      <c r="W195" s="7"/>
+      <c r="X195" s="7"/>
+      <c r="Y195" s="7"/>
+      <c r="Z195" s="7"/>
+      <c r="AA195" s="11"/>
       <c r="AB195" s="16"/>
       <c r="AC195" s="1"/>
       <c r="AD195" s="1"/>
       <c r="AE195" s="1"/>
     </row>
-    <row r="196" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A196" s="1"/>
       <c r="B196" s="33"/>
       <c r="C196" s="73">
-        <f>INT($C$193)+2</f>
-        <v>3</v>
+        <f>INT($C$194)+2.005</f>
+        <v>3.0049999999999999</v>
       </c>
       <c r="D196" s="3"/>
-      <c r="E196" s="5"/>
-      <c r="F196" s="5"/>
+      <c r="E196" s="3"/>
+      <c r="F196" s="3"/>
       <c r="G196" s="3"/>
-      <c r="H196" s="29"/>
-      <c r="I196" s="29"/>
-      <c r="J196" s="29"/>
-      <c r="K196" s="29"/>
-      <c r="L196" s="29"/>
-      <c r="M196" s="29"/>
-      <c r="N196" s="29"/>
-      <c r="O196" s="29"/>
-      <c r="P196" s="29"/>
-      <c r="Q196" s="29"/>
-      <c r="R196" s="29"/>
-      <c r="S196" s="29"/>
-      <c r="T196" s="29"/>
-      <c r="U196" s="29"/>
-      <c r="V196" s="29"/>
-      <c r="W196" s="29"/>
-      <c r="X196" s="29"/>
-      <c r="Y196" s="29"/>
-      <c r="Z196" s="29"/>
+      <c r="H196" s="3"/>
+      <c r="I196" s="3"/>
+      <c r="J196" s="3"/>
+      <c r="K196" s="3"/>
+      <c r="L196" s="3"/>
+      <c r="M196" s="3"/>
+      <c r="N196" s="3"/>
+      <c r="O196" s="3"/>
+      <c r="P196" s="3"/>
+      <c r="Q196" s="3"/>
+      <c r="R196" s="3"/>
+      <c r="S196" s="3"/>
+      <c r="T196" s="3"/>
+      <c r="U196" s="3"/>
+      <c r="V196" s="3"/>
+      <c r="W196" s="3"/>
+      <c r="X196" s="3"/>
+      <c r="Y196" s="3"/>
+      <c r="Z196" s="3"/>
       <c r="AA196" s="3"/>
       <c r="AB196" s="16"/>
       <c r="AC196" s="1"/>
@@ -35633,7 +35655,7 @@
       <c r="A197" s="1"/>
       <c r="B197" s="33"/>
       <c r="C197" s="73">
-        <f>INT($C$193)+2</f>
+        <f>INT($C$194)+2</f>
         <v>3</v>
       </c>
       <c r="D197" s="3"/>
@@ -35665,18 +35687,16 @@
       <c r="AD197" s="1"/>
       <c r="AE197" s="1"/>
     </row>
-    <row r="198" spans="1:31" ht="9.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A198" s="1"/>
-      <c r="B198" s="33" t="s">
-        <v>20</v>
-      </c>
+      <c r="B198" s="33"/>
       <c r="C198" s="73">
-        <f>INT($C$193)+2.01</f>
-        <v>3.01</v>
+        <f>INT($C$194)+2</f>
+        <v>3</v>
       </c>
       <c r="D198" s="3"/>
-      <c r="E198" s="3"/>
-      <c r="F198" s="3"/>
+      <c r="E198" s="5"/>
+      <c r="F198" s="5"/>
       <c r="G198" s="3"/>
       <c r="H198" s="29"/>
       <c r="I198" s="29"/>
@@ -35703,37 +35723,39 @@
       <c r="AD198" s="1"/>
       <c r="AE198" s="1"/>
     </row>
-    <row r="199" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:31" ht="9.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A199" s="1"/>
-      <c r="B199" s="33"/>
+      <c r="B199" s="33" t="s">
+        <v>20</v>
+      </c>
       <c r="C199" s="73">
-        <f>C$192</f>
-        <v>5</v>
-      </c>
-      <c r="D199" s="4"/>
-      <c r="E199" s="5"/>
-      <c r="F199" s="5"/>
-      <c r="G199" s="4"/>
-      <c r="H199" s="5"/>
-      <c r="I199" s="5"/>
-      <c r="J199" s="5"/>
-      <c r="K199" s="5"/>
-      <c r="L199" s="5"/>
-      <c r="M199" s="5"/>
-      <c r="N199" s="5"/>
-      <c r="O199" s="5"/>
-      <c r="P199" s="5"/>
-      <c r="Q199" s="5"/>
-      <c r="R199" s="5"/>
-      <c r="S199" s="5"/>
-      <c r="T199" s="5"/>
-      <c r="U199" s="5"/>
-      <c r="V199" s="5"/>
-      <c r="W199" s="5"/>
-      <c r="X199" s="5"/>
-      <c r="Y199" s="5"/>
-      <c r="Z199" s="5"/>
-      <c r="AA199" s="4"/>
+        <f>INT($C$194)+2.01</f>
+        <v>3.01</v>
+      </c>
+      <c r="D199" s="3"/>
+      <c r="E199" s="3"/>
+      <c r="F199" s="3"/>
+      <c r="G199" s="3"/>
+      <c r="H199" s="29"/>
+      <c r="I199" s="29"/>
+      <c r="J199" s="29"/>
+      <c r="K199" s="29"/>
+      <c r="L199" s="29"/>
+      <c r="M199" s="29"/>
+      <c r="N199" s="29"/>
+      <c r="O199" s="29"/>
+      <c r="P199" s="29"/>
+      <c r="Q199" s="29"/>
+      <c r="R199" s="29"/>
+      <c r="S199" s="29"/>
+      <c r="T199" s="29"/>
+      <c r="U199" s="29"/>
+      <c r="V199" s="29"/>
+      <c r="W199" s="29"/>
+      <c r="X199" s="29"/>
+      <c r="Y199" s="29"/>
+      <c r="Z199" s="29"/>
+      <c r="AA199" s="3"/>
       <c r="AB199" s="16"/>
       <c r="AC199" s="1"/>
       <c r="AD199" s="1"/>
@@ -35741,16 +35763,12 @@
     </row>
     <row r="200" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A200" s="1"/>
-      <c r="B200" s="33" t="s">
-        <v>19</v>
-      </c>
+      <c r="B200" s="33"/>
       <c r="C200" s="73">
-        <f>C$192</f>
+        <f>C$193</f>
         <v>5</v>
       </c>
-      <c r="D200" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="D200" s="4"/>
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
       <c r="G200" s="4"/>
@@ -35779,100 +35797,104 @@
       <c r="AD200" s="1"/>
       <c r="AE200" s="1"/>
     </row>
-    <row r="201" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:31" outlineLevel="4" x14ac:dyDescent="0.25">
       <c r="A201" s="1"/>
-      <c r="B201" s="33"/>
+      <c r="B201" s="33" t="s">
+        <v>19</v>
+      </c>
       <c r="C201" s="73">
-        <f>INT($C$193)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>C$193</f>
+        <v>5</v>
       </c>
       <c r="D201" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E201" s="4"/>
-      <c r="F201" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="E201" s="5"/>
+      <c r="F201" s="5"/>
       <c r="G201" s="4"/>
-      <c r="H201" s="58"/>
-      <c r="I201" s="58"/>
-      <c r="J201" s="58"/>
-      <c r="K201" s="58"/>
-      <c r="L201" s="58"/>
-      <c r="M201" s="58"/>
-      <c r="N201" s="58"/>
-      <c r="O201" s="58"/>
-      <c r="P201" s="58"/>
-      <c r="Q201" s="58"/>
-      <c r="R201" s="58"/>
-      <c r="S201" s="58"/>
-      <c r="T201" s="58"/>
-      <c r="U201" s="58"/>
-      <c r="V201" s="58"/>
-      <c r="W201" s="58"/>
-      <c r="X201" s="82"/>
-      <c r="Y201" s="82"/>
-      <c r="Z201" s="82"/>
+      <c r="H201" s="5"/>
+      <c r="I201" s="5"/>
+      <c r="J201" s="5"/>
+      <c r="K201" s="5"/>
+      <c r="L201" s="5"/>
+      <c r="M201" s="5"/>
+      <c r="N201" s="5"/>
+      <c r="O201" s="5"/>
+      <c r="P201" s="5"/>
+      <c r="Q201" s="5"/>
+      <c r="R201" s="5"/>
+      <c r="S201" s="5"/>
+      <c r="T201" s="5"/>
+      <c r="U201" s="5"/>
+      <c r="V201" s="5"/>
+      <c r="W201" s="5"/>
+      <c r="X201" s="5"/>
+      <c r="Y201" s="5"/>
+      <c r="Z201" s="5"/>
       <c r="AA201" s="4"/>
       <c r="AB201" s="16"/>
       <c r="AC201" s="1"/>
       <c r="AD201" s="1"/>
       <c r="AE201" s="1"/>
     </row>
-    <row r="202" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A202" s="1"/>
       <c r="B202" s="33"/>
       <c r="C202" s="73">
-        <f>INT($C$193)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D202" s="4"/>
-      <c r="E202" s="5"/>
-      <c r="F202" s="5"/>
+        <f>INT($C$194)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D202" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E202" s="4"/>
+      <c r="F202" s="4"/>
       <c r="G202" s="4"/>
-      <c r="H202" s="64" t="s">
-        <v>287</v>
-      </c>
-      <c r="I202" s="31">
-        <v>4</v>
-      </c>
-      <c r="J202" s="158" t="s">
-        <v>291</v>
-      </c>
-      <c r="K202" s="2"/>
-      <c r="L202" s="2"/>
-      <c r="M202" s="2"/>
-      <c r="N202" s="2"/>
-      <c r="O202" s="2"/>
-      <c r="P202" s="2"/>
-      <c r="Q202" s="2"/>
-      <c r="R202" s="2"/>
-      <c r="S202" s="2"/>
-      <c r="T202" s="2"/>
-      <c r="U202" s="2"/>
-      <c r="V202" s="2"/>
-      <c r="W202" s="2"/>
-      <c r="X202" s="2"/>
-      <c r="Y202" s="2"/>
-      <c r="Z202" s="2"/>
+      <c r="H202" s="58"/>
+      <c r="I202" s="58"/>
+      <c r="J202" s="58"/>
+      <c r="K202" s="58"/>
+      <c r="L202" s="58"/>
+      <c r="M202" s="58"/>
+      <c r="N202" s="58"/>
+      <c r="O202" s="58"/>
+      <c r="P202" s="58"/>
+      <c r="Q202" s="58"/>
+      <c r="R202" s="58"/>
+      <c r="S202" s="58"/>
+      <c r="T202" s="58"/>
+      <c r="U202" s="58"/>
+      <c r="V202" s="58"/>
+      <c r="W202" s="58"/>
+      <c r="X202" s="82"/>
+      <c r="Y202" s="82"/>
+      <c r="Z202" s="82"/>
       <c r="AA202" s="4"/>
       <c r="AB202" s="16"/>
       <c r="AC202" s="1"/>
       <c r="AD202" s="1"/>
       <c r="AE202" s="1"/>
     </row>
-    <row r="203" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
       <c r="B203" s="33"/>
       <c r="C203" s="73">
-        <f>INT($C$193)+3</f>
-        <v>4</v>
+        <f>INT($C$194)+2</f>
+        <v>3</v>
       </c>
       <c r="D203" s="4"/>
       <c r="E203" s="5"/>
       <c r="F203" s="5"/>
       <c r="G203" s="4"/>
-      <c r="H203" s="157"/>
-      <c r="I203" s="2"/>
-      <c r="J203" s="2"/>
+      <c r="H203" s="64" t="s">
+        <v>287</v>
+      </c>
+      <c r="I203" s="31">
+        <v>4</v>
+      </c>
+      <c r="J203" s="158" t="s">
+        <v>291</v>
+      </c>
       <c r="K203" s="2"/>
       <c r="L203" s="2"/>
       <c r="M203" s="2"/>
@@ -35899,24 +35921,24 @@
       <c r="A204" s="1"/>
       <c r="B204" s="33"/>
       <c r="C204" s="73">
-        <f>INT(C$193+3)</f>
+        <f>INT($C$194)+3</f>
         <v>4</v>
       </c>
       <c r="D204" s="4"/>
       <c r="E204" s="5"/>
       <c r="F204" s="5"/>
       <c r="G204" s="4"/>
-      <c r="H204" s="148"/>
-      <c r="I204" s="148"/>
-      <c r="J204" s="148"/>
-      <c r="K204" s="148"/>
-      <c r="L204" s="148"/>
-      <c r="M204" s="148"/>
-      <c r="N204" s="148"/>
-      <c r="O204" s="148"/>
-      <c r="P204" s="148"/>
-      <c r="Q204" s="148"/>
-      <c r="R204" s="148"/>
+      <c r="H204" s="157"/>
+      <c r="I204" s="2"/>
+      <c r="J204" s="2"/>
+      <c r="K204" s="2"/>
+      <c r="L204" s="2"/>
+      <c r="M204" s="2"/>
+      <c r="N204" s="2"/>
+      <c r="O204" s="2"/>
+      <c r="P204" s="2"/>
+      <c r="Q204" s="2"/>
+      <c r="R204" s="2"/>
       <c r="S204" s="2"/>
       <c r="T204" s="2"/>
       <c r="U204" s="2"/>
@@ -35931,50 +35953,48 @@
       <c r="AD204" s="1"/>
       <c r="AE204" s="1"/>
     </row>
-    <row r="205" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:31" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A205" s="1"/>
       <c r="B205" s="33"/>
       <c r="C205" s="73">
-        <f>INT($C$193)+3.005</f>
-        <v>4.0049999999999999</v>
+        <f>INT(C$194+3)</f>
+        <v>4</v>
       </c>
       <c r="D205" s="4"/>
-      <c r="E205" s="4"/>
-      <c r="F205" s="4"/>
+      <c r="E205" s="5"/>
+      <c r="F205" s="5"/>
       <c r="G205" s="4"/>
-      <c r="H205" s="4"/>
-      <c r="I205" s="4"/>
-      <c r="J205" s="4"/>
-      <c r="K205" s="4"/>
-      <c r="L205" s="4"/>
-      <c r="M205" s="4"/>
-      <c r="N205" s="4"/>
-      <c r="O205" s="4"/>
-      <c r="P205" s="4"/>
-      <c r="Q205" s="4"/>
-      <c r="R205" s="4"/>
-      <c r="S205" s="4"/>
-      <c r="T205" s="4"/>
-      <c r="U205" s="4"/>
-      <c r="V205" s="4"/>
-      <c r="W205" s="4"/>
-      <c r="X205" s="4"/>
-      <c r="Y205" s="4"/>
-      <c r="Z205" s="4"/>
-      <c r="AA205" s="4" t="s">
-        <v>3</v>
-      </c>
+      <c r="H205" s="148"/>
+      <c r="I205" s="148"/>
+      <c r="J205" s="148"/>
+      <c r="K205" s="148"/>
+      <c r="L205" s="148"/>
+      <c r="M205" s="148"/>
+      <c r="N205" s="148"/>
+      <c r="O205" s="148"/>
+      <c r="P205" s="148"/>
+      <c r="Q205" s="148"/>
+      <c r="R205" s="148"/>
+      <c r="S205" s="2"/>
+      <c r="T205" s="2"/>
+      <c r="U205" s="2"/>
+      <c r="V205" s="2"/>
+      <c r="W205" s="2"/>
+      <c r="X205" s="2"/>
+      <c r="Y205" s="2"/>
+      <c r="Z205" s="2"/>
+      <c r="AA205" s="4"/>
       <c r="AB205" s="16"/>
       <c r="AC205" s="1"/>
       <c r="AD205" s="1"/>
       <c r="AE205" s="1"/>
     </row>
-    <row r="206" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="3" x14ac:dyDescent="0.25">
       <c r="A206" s="1"/>
       <c r="B206" s="33"/>
       <c r="C206" s="73">
-        <f>INT($C$193)+2.005</f>
-        <v>3.0049999999999999</v>
+        <f>INT($C$194)+3.005</f>
+        <v>4.0049999999999999</v>
       </c>
       <c r="D206" s="4"/>
       <c r="E206" s="4"/>
@@ -35999,126 +36019,131 @@
       <c r="X206" s="4"/>
       <c r="Y206" s="4"/>
       <c r="Z206" s="4"/>
-      <c r="AA206" s="4"/>
+      <c r="AA206" s="4" t="s">
+        <v>3</v>
+      </c>
       <c r="AB206" s="16"/>
       <c r="AC206" s="1"/>
       <c r="AD206" s="1"/>
       <c r="AE206" s="1"/>
     </row>
-    <row r="207" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A207" s="1"/>
-      <c r="B207" s="35"/>
-      <c r="C207" s="76">
-        <f>INT($C$193)+1.005</f>
-        <v>2.0049999999999999</v>
-      </c>
-      <c r="D207" s="17"/>
-      <c r="E207" s="17"/>
-      <c r="F207" s="17"/>
-      <c r="G207" s="17"/>
-      <c r="H207" s="17"/>
-      <c r="I207" s="17"/>
-      <c r="J207" s="17"/>
-      <c r="K207" s="17"/>
-      <c r="L207" s="17"/>
-      <c r="M207" s="17"/>
-      <c r="N207" s="17"/>
-      <c r="O207" s="17"/>
-      <c r="P207" s="17"/>
-      <c r="Q207" s="17"/>
-      <c r="R207" s="17"/>
-      <c r="S207" s="17"/>
-      <c r="T207" s="17"/>
-      <c r="U207" s="17"/>
-      <c r="V207" s="17"/>
-      <c r="W207" s="17"/>
-      <c r="X207" s="17"/>
-      <c r="Y207" s="17"/>
-      <c r="Z207" s="17"/>
-      <c r="AA207" s="17"/>
-      <c r="AB207" s="18" t="s">
-        <v>1</v>
-      </c>
+      <c r="B207" s="33"/>
+      <c r="C207" s="73">
+        <f>INT($C$194)+2.005</f>
+        <v>3.0049999999999999</v>
+      </c>
+      <c r="D207" s="4"/>
+      <c r="E207" s="4"/>
+      <c r="F207" s="4"/>
+      <c r="G207" s="4"/>
+      <c r="H207" s="4"/>
+      <c r="I207" s="4"/>
+      <c r="J207" s="4"/>
+      <c r="K207" s="4"/>
+      <c r="L207" s="4"/>
+      <c r="M207" s="4"/>
+      <c r="N207" s="4"/>
+      <c r="O207" s="4"/>
+      <c r="P207" s="4"/>
+      <c r="Q207" s="4"/>
+      <c r="R207" s="4"/>
+      <c r="S207" s="4"/>
+      <c r="T207" s="4"/>
+      <c r="U207" s="4"/>
+      <c r="V207" s="4"/>
+      <c r="W207" s="4"/>
+      <c r="X207" s="4"/>
+      <c r="Y207" s="4"/>
+      <c r="Z207" s="4"/>
+      <c r="AA207" s="4"/>
+      <c r="AB207" s="16"/>
       <c r="AC207" s="1"/>
       <c r="AD207" s="1"/>
       <c r="AE207" s="1"/>
     </row>
-    <row r="208" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:31" ht="5.0999999999999996" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1"/>
-      <c r="B208" s="19"/>
-      <c r="C208" s="77">
-        <f>INT($C$193)+0.005</f>
-        <v>1.0049999999999999</v>
-      </c>
-      <c r="D208" s="19"/>
-      <c r="E208" s="19"/>
-      <c r="F208" s="19"/>
-      <c r="G208" s="19"/>
-      <c r="H208" s="19"/>
-      <c r="I208" s="19"/>
-      <c r="J208" s="19"/>
-      <c r="K208" s="19"/>
-      <c r="L208" s="19"/>
-      <c r="M208" s="19"/>
-      <c r="N208" s="19"/>
-      <c r="O208" s="19"/>
-      <c r="P208" s="19"/>
-      <c r="Q208" s="19"/>
-      <c r="R208" s="19"/>
-      <c r="S208" s="19"/>
-      <c r="T208" s="19"/>
-      <c r="U208" s="19"/>
-      <c r="V208" s="19"/>
-      <c r="W208" s="19"/>
-      <c r="X208" s="19"/>
-      <c r="Y208" s="19"/>
-      <c r="Z208" s="19"/>
-      <c r="AA208" s="19"/>
-      <c r="AB208" s="19"/>
+      <c r="B208" s="35"/>
+      <c r="C208" s="76">
+        <f>INT($C$194)+1.005</f>
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="D208" s="17"/>
+      <c r="E208" s="17"/>
+      <c r="F208" s="17"/>
+      <c r="G208" s="17"/>
+      <c r="H208" s="17"/>
+      <c r="I208" s="17"/>
+      <c r="J208" s="17"/>
+      <c r="K208" s="17"/>
+      <c r="L208" s="17"/>
+      <c r="M208" s="17"/>
+      <c r="N208" s="17"/>
+      <c r="O208" s="17"/>
+      <c r="P208" s="17"/>
+      <c r="Q208" s="17"/>
+      <c r="R208" s="17"/>
+      <c r="S208" s="17"/>
+      <c r="T208" s="17"/>
+      <c r="U208" s="17"/>
+      <c r="V208" s="17"/>
+      <c r="W208" s="17"/>
+      <c r="X208" s="17"/>
+      <c r="Y208" s="17"/>
+      <c r="Z208" s="17"/>
+      <c r="AA208" s="17"/>
+      <c r="AB208" s="18" t="s">
+        <v>1</v>
+      </c>
       <c r="AC208" s="1"/>
       <c r="AD208" s="1"/>
       <c r="AE208" s="1"/>
     </row>
-    <row r="209" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:31" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="1"/>
-      <c r="B209" s="1"/>
-      <c r="C209" s="73">
-        <f>INT($C$193)+2</f>
-        <v>3</v>
-      </c>
-      <c r="D209" s="1"/>
-      <c r="E209" s="1"/>
-      <c r="F209" s="1"/>
-      <c r="G209" s="1"/>
-      <c r="H209" s="1"/>
-      <c r="I209" s="1"/>
-      <c r="J209" s="1"/>
-      <c r="K209" s="1"/>
-      <c r="L209" s="1"/>
-      <c r="M209" s="1"/>
-      <c r="N209" s="1"/>
-      <c r="O209" s="1"/>
-      <c r="P209" s="1"/>
-      <c r="Q209" s="1"/>
-      <c r="R209" s="1"/>
-      <c r="S209" s="1"/>
-      <c r="T209" s="1"/>
-      <c r="U209" s="1"/>
-      <c r="V209" s="1"/>
-      <c r="W209" s="1"/>
-      <c r="X209" s="1"/>
-      <c r="Y209" s="1"/>
-      <c r="Z209" s="1"/>
-      <c r="AA209" s="1"/>
-      <c r="AB209" s="1"/>
+      <c r="B209" s="19"/>
+      <c r="C209" s="77">
+        <f>INT($C$194)+0.005</f>
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D209" s="19"/>
+      <c r="E209" s="19"/>
+      <c r="F209" s="19"/>
+      <c r="G209" s="19"/>
+      <c r="H209" s="19"/>
+      <c r="I209" s="19"/>
+      <c r="J209" s="19"/>
+      <c r="K209" s="19"/>
+      <c r="L209" s="19"/>
+      <c r="M209" s="19"/>
+      <c r="N209" s="19"/>
+      <c r="O209" s="19"/>
+      <c r="P209" s="19"/>
+      <c r="Q209" s="19"/>
+      <c r="R209" s="19"/>
+      <c r="S209" s="19"/>
+      <c r="T209" s="19"/>
+      <c r="U209" s="19"/>
+      <c r="V209" s="19"/>
+      <c r="W209" s="19"/>
+      <c r="X209" s="19"/>
+      <c r="Y209" s="19"/>
+      <c r="Z209" s="19"/>
+      <c r="AA209" s="19"/>
+      <c r="AB209" s="19"/>
       <c r="AC209" s="1"/>
       <c r="AD209" s="1"/>
       <c r="AE209" s="1"/>
     </row>
-    <row r="210" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:31" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
-      <c r="C210" s="66"/>
+      <c r="C210" s="73">
+        <f>INT($C$194)+2</f>
+        <v>3</v>
+      </c>
       <c r="D210" s="1"/>
       <c r="E210" s="1"/>
       <c r="F210" s="1"/>
@@ -36314,7 +36339,40 @@
       <c r="AE215" s="1"/>
     </row>
     <row r="216" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="C216" s="72" t="s">
+      <c r="A216" s="1"/>
+      <c r="B216" s="1"/>
+      <c r="C216" s="66"/>
+      <c r="D216" s="1"/>
+      <c r="E216" s="1"/>
+      <c r="F216" s="1"/>
+      <c r="G216" s="1"/>
+      <c r="H216" s="1"/>
+      <c r="I216" s="1"/>
+      <c r="J216" s="1"/>
+      <c r="K216" s="1"/>
+      <c r="L216" s="1"/>
+      <c r="M216" s="1"/>
+      <c r="N216" s="1"/>
+      <c r="O216" s="1"/>
+      <c r="P216" s="1"/>
+      <c r="Q216" s="1"/>
+      <c r="R216" s="1"/>
+      <c r="S216" s="1"/>
+      <c r="T216" s="1"/>
+      <c r="U216" s="1"/>
+      <c r="V216" s="1"/>
+      <c r="W216" s="1"/>
+      <c r="X216" s="1"/>
+      <c r="Y216" s="1"/>
+      <c r="Z216" s="1"/>
+      <c r="AA216" s="1"/>
+      <c r="AB216" s="1"/>
+      <c r="AC216" s="1"/>
+      <c r="AD216" s="1"/>
+      <c r="AE216" s="1"/>
+    </row>
+    <row r="217" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="C217" s="72" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>